<commit_message>
Reworking annotation data for UI
</commit_message>
<xml_diff>
--- a/annotation_tool/selected_sessions_normalized_with_ner_tagged.xlsx
+++ b/annotation_tool/selected_sessions_normalized_with_ner_tagged.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN4"/>
+  <dimension ref="A1:AQ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -611,22 +611,37 @@
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
+          <t>whisper_reconstructed_ref_original</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>phi4_reconstructed_ref_original</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>parakeet_reconstructed_ref_original</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>norm_human_transcript_ner</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
           <t>whisper_reconstructed_ref</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>phi4_reconstructed_ref</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>parakeet_reconstructed_ref</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>norm_human_transcript_ner</t>
         </is>
       </c>
     </row>
@@ -912,7 +927,22 @@
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> male or a female  a male  how old are you  i am sixtyfive years old  hope you do not mind if i address you as mr emeka  i do not mind  okay thank you very much so what brought you to the clinic today  i am having [UMLS/C1299586: Has difficulty doing (qualifier value)]  okay you have been having [UMLS/C1299586: Has difficulty doing (qualifier value)] for how long has this been  it has started for two weeks  you have been having [UMLS/C1299586: Has difficulty doing (qualifier value)] for two weeks  yes  did it started gradually or  it was gradual in onset  okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day  i think it goes bad of recent it was not constant before but now it is constant  okay thank you very much is this [UMLS/C0030193: Pain] while [UMLS/C0042034: Urination] associated with a [UMLS/C0085624: Burning sensation]  is not associated with [UMLS/C0030193: Pain] or a [UMLS/C0085624: Burning sensation]  okay it is not associated with any [UMLS/C0030193: Pain] or a [UMLS/C0085624: Burning sensation]  yes it is not  do you feel [UMLS/C0085606: Urgency of micturition]  yes i feel [UMLS/C0085606: Urgency of micturition]  and then are you able to pass out this urine when you feel this [UMLS/C0085606: Urgency of micturition]  i am unable to pass out urine  okay do you feel frequent [UMLS/C0042034: Urination] the urge to always go to the toilet  yes i am always visiting the toilet especially in the night  okay [UMLS/C0028734: Nocturia] you always visit the toilet in the night  yes at morning at night at night  like how many times do you [UMLS/C0042034: Urination] in the night  it is very frequent i cannot tell  more than you used to before  yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times  do you straint in urinate  yes i [UMLS/C0080194: Muscle strain] alot and my [UMLS/C0042036: Urine]  okay it dripples  yeah after [UMLS/C0042034: Urination]  may i know if there is [UMLS/C0018965: Hematuria]  there is no [UMLS/C0018965: Hematuria] there is no [UMLS/C0015967: Fever] i do not have [UMLS/C0015967: Fever]  is there pause  there is no pause oo  do you have lower [UMLS/C0000737: Abdominal Pain]  i do not have [UMLS/C0000737: Abdominal Pain]  okay thank you very much is there a history of [UMLS/C1368081: Physical trauma] or recent catherization or [UMLS/C0161922: Repair of urethra]  no there is not  there is not history of [UMLS/C1368081: Physical trauma] or catherization  i do not have any history of that  okay thank you very much are you a main [UMLS/C0020538: Hypertensive disease] patient are you [UMLS/C0020538: Hypertensive disease]  yes i have been [UMLS/C0020538: Hypertensive disease] for ten years now  okay you have been [UMLS/C0020538: Hypertensive disease] for ten years how do you know that you are [UMLS/C0020538: Hypertensive disease]  i was told at the hospital that i was diagnosed there  you were diagnosed in a hospital ten years ago  yes  and you have been on [UMLS/C0013227: Pharmaceutical Preparations]  yes it has been controlled by [UMLS/C0013227: Pharmaceutical Preparations]  okay thank you very much how about [UMLS/C0011847: Diabetes] are you [UMLS/C0011847: Diabetes]  no i am not [UMLS/C0011847: Diabetes]  you are not [UMLS/C0011847: Diabetes] okay is there a family history of similar condition is there anyone in your family that has similar condition  yeah i can remember my dad have similar condition when he was old  when he was old what exactly was the problem did he also feel [UMLS/C0030193: Pain] while trying to urinate  he has some [UMLS/C0033213: Problem] i can tell exactly i was young at that time  okay thank you very much are you a [UMLS/C0037366: Smoke]  i do not [UMLS/C0037366: Smoke]  do you take [UMLS/C0001962: ethanol]  yeah i consume [UMLS/C0001962: ethanol] occasionally  do you take any [UMLS/C0242508: Recreational Drugs] [UMLS/C0687130: Substance of abuse]  no  thank you very much are you on your [UMLS/C0003364: Antihypertensive Agents]  yes i am on some [UMLS/C0013227: Pharmaceutical Preparations] they give me to control the [UMLS/C0020538: Hypertensive disease]  can you tell me the name of the drug you are on  amlodepine  okay you are on amlodepine is there any drug you are on  i am not on any other they give me just that one  okay thank you very much do you have any other [UMLS/C0020517: Hypersensitivity] do you have are you allergic to any [UMLS/C0013227: Pharmaceutical Preparations] or [UMLS/C0013227: Pharmaceutical Preparations]  i am not  okay thank you very much</t>
+          <t xml:space="preserve"> male or a female  a male  how old are you  i am sixtyfive years old  hope you do not mind if i address you as mr emeka  i do not mind  okay thank you very much so what brought you to the clinic today  i am having [PROBLEM: difficulty in urinating]  okay you have been having [PROBLEM: difficulty in urinating] for how long has this been  it has started for two weeks  you have been having [PROBLEM: difficulty in urinating] for two weeks  yes  did it started gradually or  it was gradual in onset  okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day  i think it goes bad of recent it was not constant before but now it is constant  okay thank you very much is this [PROBLEM: pain] while [BODY_FUNCTION: urinating] associated with a [PROBLEM: burning sensation]  is not associated with [PROBLEM: pain] or a [PROBLEM: burning sensation]  okay it is not associated with any [PROBLEM: pain] or a [PROBLEM: burning sensation]  yes it is not  do you feel [PROBLEM: urgency to urinate]  yes i feel [PROBLEM: urgency to urinate]  and then are you able to pass out this urine when you feel this [PROBLEM: urgency to urinate]  i am unable to pass out urine  okay do you feel frequent [BODY_FUNCTION: urination] the urge to always go to the toilet  yes i am always visiting the toilet especially in the night  okay [PROBLEM: nocturia] you always visit the toilet in the night  yes at morning at night at night  like how many times do you [BODY_FUNCTION: urinate] in the night  it is very frequent i cannot tell  more than you used to before  yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times  do you [PROBLEM: straint] in urinate  yes i [PROBLEM: strain] alot and my [LABORATORY_DATA: urine dripples]  okay it dripples  yeah after [BODY_FUNCTION: urination]  may i know if there is [PROBLEM: blood in the urine]  there is no [PROBLEM: blood in this urine] there is no [PROBLEM: fever] i do not have [PROBLEM: fever]  is there pause  there is no pause oo  do you have lower [PROBLEM: abdominal pain]  i do not have [PROBLEM: abdominal pain]  okay thank you very much is there a history of [PROBLEM: trauma] or recent [PROCEDURE: catherization] or [PROCEDURE: urethra instrumentation]  no there is not  there is not history of [PROBLEM: trauma] or [PROCEDURE: catherization]  i do not have any history of that  okay thank you very much are you a main [PROBLEM: hypertensive] patient are you [PROBLEM: hypertensive]  yes i have been [PROBLEM: hypertensive] for ten years now  okay you have been [PROBLEM: hypertensive] for ten years how do you know that you are [PROBLEM: hypertensive]  i was told at the hospital that i was diagnosed there  you were diagnosed in a hospital ten years ago  yes  and you have been on [MEDICINE: medications]  yes it has been controlled by [MEDICINE: medications]  okay thank you very much how about [PROBLEM: diabetic] are you [PROBLEM: diabetic]  no i am not [PROBLEM: diabetic]  you are not [PROBLEM: diabetic] okay is there a family history of similar condition is there anyone in your family that has similar condition  yeah i can remember my dad have similar condition when he was old  when he was old what exactly was the problem did he also feel [PROBLEM: pain] while trying to urinate  he has some [PROBLEM: urinal problem] i can tell exactly i was young at that time  okay thank you very much are you a [SUBSTANCE_ABUSE: smoker]  i do not [SUBSTANCE_ABUSE: smoke]  do you take [SUBSTANCE_ABUSE: alcohol]  yeah i consume [SUBSTANCE_ABUSE: alcohol] occasionally  do you take any [SUBSTANCE_ABUSE: recreational drugs] [SUBSTANCE_ABUSE: substance abuse]  no  thank you very much are you on your [MEDICINE: hypertensive agents]  yes i am on some [MEDICINE: drugs] they give me to control the [PROBLEM: hypertension]  can you tell me the name of the drug you are on  [MEDICINE: amlodepine]  okay you are on [MEDICINE: amlodepine] is there any drug you are on  i am not on any other they give me just that one  okay thank you very much do you have any other [PROBLEM: allergies] do you have are you allergic to any [MEDICINE: drug] or [MEDICINE: medication]  i am not  okay thank you very much</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>male or a female [INS:i] [INS:am] a male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did it started gradually or it was gradual in onset okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with [SUB:a-&gt;the] burning sensation it is it [INS:is] not associated with pain or a burning sensation okay so it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to urinate yes i feel [INS:the] urgency to you ring [SUB:urinate-&gt;it] and then are you able to pass out this urine when you feel this urgency to you [INS:in] [SUB:urinate-&gt;it] i am unable to pass out [SUB:urine-&gt;here] okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting [SUB:the-&gt;into] toilet especially [DEL:in] the night okay nocturia so you always visit the toilet in the night yes at morning at night at night like how many times [SUB:do-&gt;you] you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] alot and my urine [SUB:dripples-&gt;dribbles] okay it [SUB:dripples-&gt;dribbles] yeah after [SUB:urination-&gt;i] may [DEL:i] know if there is blood in the urine there is no blood in this urine there is no fever i do not have ist have fever is there pause there is no pus pause [SUB:oo-&gt;so] do you have lower abdominal pain i do not have abdominal pain okay thank you very much is there a history of trauma or any recent [SUB:catherization-&gt;catarization] or urethra instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catarization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told [SUB:at-&gt;that] the hospital that i was diagnosed there you were diagnosed in [SUB:a-&gt;the] hospital ten years ago yes yes and you have been on medications yes it has been controlled by medications okay thank you very much how about being diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some [SUB:urinal-&gt;urinary] problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational drugs substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [INS:i] [INS:am] [INS:on] [SUB:amlodepine-&gt;lodipine] okay you are on [SUB:amlodepine-&gt;lodipine] is there any other drug you are on i am not on any other [INS:drug] they give me just that one okay thank you very much do you have any other allergies [DEL:do] you have are you allergic to any drug or medication [INS:no] i am not okay thank you very much</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>male or a female [INS:i] [INS:am] a male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr [INS:i] emeka i do not mind okay thank you very much so what brought you to the clinic today i have [SUB:am-&gt;been] having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did [INS:this] it started gradually or it was gradual in onset okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with [SUB:a-&gt;the] burning sensation it is not associated with pain or [DEL:a] burning sensation okay it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to [SUB:urinate-&gt;you] yes [DEL:i] feel [DEL:urgency] [DEL:to] [DEL:urinate] and then are you able to pass out this urine when you feel this urgency to you [SUB:urinate-&gt;know] i am unable to pass out [DEL:urine] okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting the toilet especially in the night okay nocturia so you always visit the toilet in the night yes at morning at night at night like how many times [SUB:do-&gt;you] you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than you used to [INS:be] before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] alot and my urine [SUB:dripples-&gt;bubbles] okay it [SUB:dripples-&gt;bubbles] yeah after urination may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have [INS:a] fever is there pause there is no pus so pause [SUB:oo-&gt;so] do you have lower abdominal pain i do not have any abdominal pain okay thank you very much is there a history of trauma or any recent [SUB:catherization-&gt;catheterization] or [SUB:urethra-&gt;ureteral] instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you [DEL:hypertensive] yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told [DEL:at] [DEL:the] hospital that i was diagnosed [INS:in] [INS:the] there you were diagnosed in [SUB:a-&gt;the] hospital ten years ago yes and you have been on medications yes it has been controlled by medications okay thank you very much how about being diabetic are you diabetic no i am not diabetic you are not [DEL:diabetic] okay is there [DEL:a] family history of similar condition [DEL:is] there anyone in your family that has similar condition yeah i can remember my dad have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some [SUB:urinal-&gt;urinary] problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally [DEL:do] you take any [DEL:recreational] [DEL:drugs] [DEL:substance] [DEL:abuse] [DEL:no] thank you very much are you on your hypertensive agents yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [SUB:amlodepine-&gt;i] okay you are [SUB:on-&gt;the] [SUB:amlodepine-&gt;pin] is there any other drug you are on i am not on any other [INS:drug] they give me just that one okay thank you very much do you have any other [SUB:allergies-&gt;justifications] [DEL:do] you have are you allergic to any drug or medication [INS:no] i am not okay thank you very much</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>male or a female [DEL:a] male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did it started gradually or it was gradual [SUB:in-&gt;nonsense] onset okay it was gradual in [INS:on] onset has it been constant has it always been there or it just comes and goes or you feel this within [SUB:a-&gt;the] particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with a burning sensation it is not associated with pain or a burning sensation okay so it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to urinate yes i feel [INS:the] urgency to urinate and then are you able to pass out this urine when you feel this urgency to urinate i am unable to pass out urine okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting the toilet especially in the night okay nocturia so you always visit the toilet in the night yes at morning at night at night like how many times do you urinate in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] alot and my urine [SUB:dripples-&gt;dribbles] okay it [SUB:dripples-&gt;dribbles] yeah after urination may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have fever is there pause there is no pulse pause [SUB:oo-&gt;so] do you have lower abdominal pain i do not have abdominal pain okay thank you very much is there a history of trauma or any recent [SUB:catherization-&gt;caterization] or urethra instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told at the hospital that i was diagnosed there you were diagnosed in a hospital ten years ago yes and you have been on medications yes it has been controlled by medications okay thank you very much how about being diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad had have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some urinal problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational [SUB:drugs-&gt;drug] substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [INS:i] [INS:am] not [SUB:amlodepine-&gt;pain] okay you are on and you know [INS:the] [SUB:amlodepine-&gt;pain] is there any other drug you are on i am not on any other [INS:drug] they give me just that one okay thank you very much do you have any other allergies do you have are you allergic to any drug or medication [INS:no] i am not okay thank you very much madam</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1154,22 @@
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to the hospital today what was the [UMLS/C5441521: Complaint (finding)] so doctor i have been [UMLS/C0010200: Coughing] for about a week now and i have been also also have you also have what so and i also have  i have also been running [UMLS/C0039810: thermography] for about five days so you have running [UMLS/C0039810: thermography] for five days yes yes for about a week now a week yes okay all right so the [UMLS/C0010200: Coughing] did it start suddenly or gradually the [UMLS/C0010200: Coughing] started suddenly just started like that i just just woke up more morning and started [UMLS/C0010200: Coughing] about a week ago yes was there was there any [UMLS/C1457887: Symptoms] like [UMLS/C1384493: Catarrh] or  any  any [UMLS/C0011168: Deglutition Disorders] before the [UMLS/C0010200: Coughing] started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the [UMLS/C0010200: Coughing] how does it sound does it sound like [UMLS/C0234866: Barking cough] does it sound like it is comes in bouts and then you have to take a deep breath when when you say barking do you are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no mine is not that i did not i did not experience anything like that okay so is the [UMLS/C0010200: Coughing] productive of [UMLS/C5539771: Increased sputum production] yes yes it is productive when i yes when i [UMLS/C0010200: Coughing] i bring out some some substance from my [UMLS/C0226896: Oral cavity] yes so what is the colour of the substance err it is about  it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there [UMLS/C0005822: Blood Preservation] in it at any point no there was no [UMLS/C0005822: Blood Preservation] in it there was no [UMLS/C0005822: Blood Preservation] in it there was no [UMLS/C0005822: Blood Preservation] in it at any point yes and after you [UMLS/C0010200: Coughing] do you feel like [UMLS/C0042963: Vomiting] or do you [UMLS/C0042963: Vomiting] no i do not i do not i do not feel like [UMLS/C0042963: Vomiting] i do not [UMLS/C0042963: Vomiting] at all okay and you did not have [UMLS/C1384493: Catarrh] or [UMLS/C0011168: Deglutition Disorders] prior to onset of the [UMLS/C0010200: Coughing] no no there was nothing i was not i had nothing my my even when i was [UMLS/C0010200: Coughing] my [UMLS/C0817096: Chest] was not [UMLS/C0030193: Pain] me nothing it was just the [UMLS/C0010200: Coughing] then i i discovered after a few days after that i just started running [UMLS/C0039810: thermography] too my [UMLS/C0444584: Whole body] was very very hot it was very hot that i was [UMLS/C0036973: Shivering] so you are telling me there is no there is no [UMLS/C0010200: Coughing] there is no [UMLS/C0817096: Chest] [UMLS/C0030193: Pain] no there is there is no [UMLS/C0817096: Chest] [UMLS/C0030193: Pain] my [UMLS/C0817096: Chest] was not [UMLS/C0030193: Pain] me at all your [UMLS/C0817096: Chest] was not [UMLS/C0030193: Pain] me is there anybody [UMLS/C0010200: Coughing] around you no there nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is [UMLS/C0010200: Coughing] too and at work too there is nobody [UMLS/C0010200: Coughing] around me so okay so you stay alone you are not here in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the [UMLS/C0010200: Coughing] became [UMLS/C1457868: Worse] and i was i started to have some [UMLS/C0013404: Dyspnea] so like that got me really scared like i was i was i was just feeling [UMLS/C0013404: Dyspnea] for a moment comes and goes then and since that since then the [UMLS/C0013404: Dyspnea] has become more [UMLS/C1457868: Worse] so that is what exactly prompted me to completely to see you you are finding it difficult to breathe yes yes when you sleep at night you [UMLS/C0038990: Sweating] excessively no at all i do not i do not slept i do not [UMLS/C0038990: Sweating] when i sleep at night okay so what is what relieves the [UMLS/C0013404: Dyspnea] any change in position that relieves the [UMLS/C0013404: Dyspnea] or it is constant no it is not associated with  any any position nothing i just it just comes and goes like i just feel [UMLS/C0013404: Dyspnea] for a while then it relieves me then it comes again especially when i am especially when i am [UMLS/C0010200: Coughing] okay has this worsened progressively yes yes it has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the [UMLS/C0010200: Coughing] and the fact that i have i have not been feeling well generally in my body so that is so now this [UMLS/C0015967: Fever] that you were having was it did it start suddenly or gradually it started it started gradually then became i became very hot and it has been like that it has been like that so the [UMLS/C0015967: Fever] is [UMLS/C0205082: Severe (severity modifier)] you are very hot yes yes it is high did you at any point yes check by yourself at home your [UMLS/C0039810: thermography] yes i did i did i have a [UMLS/C0039818: Thermometer, device] it was about was about thirtyeightnine thirtyeightnine okay and what does what do you do that relieves the [UMLS/C0015967: Fever] i took some i took some [UMLS/C0000970: acetaminophen] it relieved a bit then but it did did not last long i just i i became hot again and it has been like that ever since so i just want to ask you some questions has anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why i am this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you [UMLS/C0004096: Asthma] during your [UMLS/C0106629: blood group A-enzyme] and genotype no i am not doctor i am fine no i have nothing and that is why this is surprising are you [UMLS/C0020538: Hypertensive disease] what did you say i cannot hear you properly sir are you [UMLS/C0020538: Hypertensive disease] or [UMLS/C0011847: Diabetes] none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just i just tried to get some [UMLS/C2723142: Cough Syrup brand of Dextromethorphan] but they did not they did not seem to work properly they did not seem to work and since the [UMLS/C0013404: Dyspnea] started i knew i knew i know i needed to like come to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that i can remember have you done any [UMLS/C0543467: Operative Surgical Procedures] before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the [UMLS/C1457887: Symptoms] you are having so do you have [UMLS/C0018681: Headache] [UMLS/C0018681: Headache] just comes once in a while maybe because the [UMLS/C0010200: Coughing] i have not been able to sleep really so kind of yeah kind of yes okay so any [UMLS/C0041657: Unconscious State] no no no no okay okay do you have catarrh no at all okay do you have any [UMLS/C0000737: Abdominal Pain] no no i do not have any [UMLS/C0011991: Diarrhea] or [UMLS/C0042963: Vomiting] no i have not [UMLS/C0042963: Vomiting] at all you have any [UMLS/C0005931: Bone and Bones] [UMLS/C0030193: Pain] yes no the no the most it is just it is just the shortest of [UMLS/C0035203: Respiration] i have been having the [UMLS/C0013404: Dyspnea] i have been having that is just that is just so in summary you are telling me in summary you are telling me you had you you have had [UMLS/C0010200: Coughing] and [UMLS/C0013404: Dyspnea] yes right and your [UMLS/C0010200: Coughing] is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your [UMLS/C0817096: Chest] to know if to know whatever is going on in your [UMLS/C0817096: Chest] whether there is a [UMLS/C0817096: Chest] [UMLS/C0009450: Communicable Diseases] that is causing you to have a [UMLS/C0015967: Fever] and the and the [UMLS/C0010200: Coughing] do you understand and then we are going to have you do some investigations like a [UMLS/C0817096: Chest] [UMLS/C0043299: Diagnostic radiologic examination] a [UMLS/C0009555: Complete Blood Count] a [UMLS/C0009555: Complete Blood Count] which will tell us whether there is an [UMLS/C0009450: Communicable Diseases] going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an [UMLS/C1155266: Inflammatory Response] going on do you understand and then we are also going to take your sputum your the [UMLS/C5539771: Increased sputum production] and we are going to send it for [UMLS/C0455287: Culture sensitivity] to know what [UMLS/C0003244: Antibodies, Bacterial] is is being [UMLS/C0430400: Laboratory culture]  please i just want to ask you do you [UMLS/C0037366: Smoke] no no i do not doctor i am a good christian i do not [UMLS/C0037366: Smoke] i do not [UMLS/C0556374: Drunk driving] you do not you do not drink [UMLS/C0001962: ethanol] either i do not i do not do any of those i do not do [UMLS/C0013227: Pharmaceutical Preparations] i do not do any of that i am going to ask you some other questions do you have their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i will need to take basically i just want to ask ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex i am married no not at all not at all i am married so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because the because of what is causing the [UMLS/C0010200: Coughing] and the [UMLS/C0015967: Fever] we have some this thing at the back of our mind which could be the because do you understand we think you have a [UMLS/C0032285: Pneumonia] a [UMLS/C0817096: Chest] [UMLS/C0009450: Communicable Diseases] so we are going to [UMLS/C5447432: Collagen Tile Brachytherapy] you on a [UMLS/C5197773: Broadly Neutralizing Antibodies] right and then we are going to start you on the [UMLS/C2723142: Cough Syrup brand of Dextromethorphan] right to treat the [UMLS/C0010200: Coughing] while we wait for the results of our investigations do you understand okay and then since there is no history of [UMLS/C0004096: Asthma] by the time you will start [UMLS/C0087111: Therapeutic procedure] with the [UMLS/C0003232: Antibiotics] and and the [UMLS/C2723142: Cough Syrup brand of Dextromethorphan] there will be the [UMLS/C0013404: Dyspnea] is going to reduce but we your we would have checked your your [UMLS/C0483415: Oxygen Saturation] and we will see that it is fine so there will be no need to place you on on [UMLS/C0030054: oxygen] so you are going to have you do a [UMLS/C0009555: Complete Blood Count] and [UMLS/C0455287: Culture sensitivity] you are going to have you do any [UMLS/C0014792: Erythrocytes] and you are going to do a [UMLS/C0817096: Chest] [UMLS/C0043299: Diagnostic radiologic examination] so let us see if it is a [UMLS/C1881747: Structural Problem] or a [UMLS/C0033213: Problem] do you understand okay doctor so doctor do i do you want to ask the question if you have any questions yes i was going to ask that are you going to keep me in the hospital or do i that can i can i be treated from home because i do not know we we we are going to admit you for some time to evaluate you and because of the [UMLS/C0013404: Dyspnea] you are having right and then we will start you on on [UMLS/C0348016: Intravenous] [UMLS/C0348016: Intravenous]  that is okay that is cool [UMLS/C0430400: Laboratory culture] and [UMLS/C0376622: ABCB1 gene] could take about seventytwo hours to to five days before it will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just yeah i will just do the [UMLS/C1825793: LAT2 gene] and wait for just for you to start the [UMLS/C0087111: Therapeutic procedure] thank you</t>
+          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to the hospital today what was the [PROBLEM: complaints] so doctor i have been [PROBLEM: coughing] for about a week now and i have been also also have you also have what so and i also have  i have also been running [BODY_MEASUREMENT: temperature] for about five days so you have running [BODY_MEASUREMENT: temperature] for five days yes yes for about a week now a week yes okay all right so the [PROBLEM: cough] did it start suddenly or gradually the [PROBLEM: cough] started suddenly just started like that i just just woke up more morning and started [PROBLEM: coughing] about a week ago yes was there was there any [PROBLEM: symptoms] like [PROBLEM: catarrh] or  any  any [PROBLEM: difficulty in swallowing] before the [PROBLEM: cough] started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the [PROBLEM: cough] how does it sound does it sound like [PROBLEM: barking] does it sound like it is comes in bouts and then you have to take a deep breath when when you say barking do you are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no mine is not that i did not i did not experience anything like that okay so is the [PROBLEM: cough] productive of [PROBLEM: phlegm] yes yes it is productive when i yes when i [PROBLEM: cough] i bring out some some substance from my [ANATOMICAL_STRUCTURE: mouth] yes so what is the colour of the substance err it is about  it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there [PROBLEM: blood] in it at any point no there was no [PROBLEM: blood] in it there was no [PROBLEM: blood] in it there was no [PROBLEM: blood] in it at any point yes and after you [PROBLEM: cough] do you feel like [PROBLEM: vomiting] or do you [PROBLEM: vomit] no i do not i do not i do not feel like [PROBLEM: vomiting] i do not [PROBLEM: vomit] at all okay and you did not have [PROBLEM: catarrh] or [PROBLEM: difficulty in swallowing] prior to onset of the [PROBLEM: cough] no no there was nothing i was not i had nothing my my even when i was [PROBLEM: coughing] my [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: paining] me nothing it was just the [PROBLEM: cough] then i i discovered after a few days after that i just started running [BODY_MEASUREMENT: temperature] too my [ANATOMICAL_STRUCTURE: body] was very very hot it was very hot that i was [PROBLEM: shivering] so you are telling me there is no there is no [PROBLEM: cough] there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] no there is there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] my [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: paining] me at all your [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: paining] me is there anybody [PROBLEM: coughing] around you no there nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is [PROBLEM: coughing] too and at work too there is nobody [PROBLEM: coughing] around me so okay so you stay alone you are not here in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the [PROBLEM: cough] became [SEVERITY: worsened] and i was i started to have some [PROBLEM: difficulty in breathing] so like that got me really scared like i was i was i was just feeling [PROBLEM: breathless] for a moment comes and goes then and since that since then the [PROBLEM: breathlessness] has become more [SEVERITY: worsened] so that is what exactly prompted me to completely to see you you are finding it difficult to breathe yes yes when you sleep at night you [PROBLEM: sweat] excessively no at all i do not i do not slept i do not [PROBLEM: sweat] when i sleep at night okay so what is what relieves the [PROBLEM: breathlessness] any change in position that relieves the [PROBLEM: breathlessness] or it is constant no it is not associated with  any any position nothing i just it just comes and goes like i just feel [PROBLEM: breathless] for a while then it relieves me then it comes again especially when i am especially when i am [PROBLEM: coughing] okay has this worsened progressively yes yes it has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the [PROBLEM: cough] and the fact that i have i have not been feeling well generally in my body so that is so now this [PROBLEM: fever] that you were having was it did it start suddenly or gradually it started it started gradually then became i became very hot and it has been like that it has been like that so the [PROBLEM: fever] is [SEVERITY: high grade] you are very hot yes yes it is high did you at any point yes check by yourself at home your [BODY_MEASUREMENT: temperature] yes i did i did i have a [MEDICAL_DEVICE: thermometer] it was about was about [MEDICINE: thirtyeightnine] [MEDICINE: thirtyeightnine] okay and what does what do you do that relieves the [PROBLEM: fever] i took some i took some [MEDICINE: paracetamol] it relieved a bit then but it did did not last long i just i i became hot again and it has been like that ever since so i just want to ask you some questions has anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why i am this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you [PROBLEM: asthmatic] during your [LABORATORY_DATA: blood group] and genotype no i am not doctor i am fine no i have nothing and that is why this is surprising are you [PROBLEM: hypertensive] what did you say i cannot hear you properly sir are you [PROBLEM: hypertensive] or [PROBLEM: diabetic] none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just i just tried to get some [MEDICINE: cough syrup] but they did not they did not seem to work properly they did not seem to work and since the [PROBLEM: difficulty breathing] started i knew i knew i know i needed to like come to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that i can remember have you done any [PROCEDURE: surgical procedure] before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the [PROBLEM: symptoms] you are having so do you have [PROBLEM: headache] [PROBLEM: headache] just comes once in a while maybe because the [PROBLEM: cough] i have not been able to sleep really so kind of yeah kind of yes okay so any [PROBLEM: loss of consciousness] no no no no okay okay do you have [MEDICINE: catarrh] no at all okay do you have any [PROBLEM: abdominal pain] no no i do not have any [PROBLEM: diarrhea] or [PROBLEM: vomiting] no i have not [PROBLEM: vomited] at all you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] yes no the no the most it is just it is just the shortest of [BODY_FUNCTION: breath] i have been having the [PROBLEM: difficulty in breathing] i have been having that is just that is just so in summary you are telling me in summary you are telling me you had you you have had [PROBLEM: cough fever] and [PROBLEM: difficulty in breathing] yes right and your [PROBLEM: cough] is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your [ANATOMICAL_STRUCTURE: chest] to know if to know whatever is going on in your [ANATOMICAL_STRUCTURE: chest] whether there is a [ANATOMICAL_STRUCTURE: chest] [PROBLEM: infection] that is causing you to have a [PROBLEM: fever] and the and the [PROBLEM: cough] do you understand and then we are going to have you do some investigations like a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] a [LABORATORY_DATA: complete blood count] a [LABORATORY_DATA: full blood count] which will tell us whether there is an [PROBLEM: infection] going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an [PROBLEM: inflammatory process] going on do you understand and then we are also going to take your sputum your the [PROBLEM: phlegm] and we are going to send it for [LABORATORY_DATA: culture sensitivity] to know what [LABORATORY_DATA: bacteria] is is being [LABORATORY_DATA: cultured]  please i just want to ask you do you [SUBSTANCE_ABUSE: smoke] no no i do not doctor i am a good christian i do not [SUBSTANCE_ABUSE: smoke] i do not [SUBSTANCE_ABUSE: drink] you do not you do not drink [SUBSTANCE_ABUSE: alcohol] either i do not i do not do any of those i do not do [SUBSTANCE_ABUSE: drugs] i do not do any of that i am going to ask you some other questions do you have their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i will need to take basically i just want to ask ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex i am married no not at all not at all i am married so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because the because of what is causing the [PROBLEM: cough] and the [PROBLEM: fever] we have some this thing at the back of our mind which could be the because do you understand we think you have a [PROBLEM: pneumonia pneumonia] a [ANATOMICAL_STRUCTURE: chest] [PROBLEM: infection] so we are going to [MED_STATUS: start] you on a [MEDICINE: broad spectrum antibiotics] right and then we are going to start you on the [MEDICINE: cough syrup] right to treat the [PROBLEM: cough] while we wait for the results of our investigations do you understand okay and then since there is no history of [PROBLEM: asthma] by the time you will start [PROCEDURE: treatment] with the [MEDICINE: antibiotics] and and the [MEDICINE: cough syrup] there will be the [PROBLEM: breathlessness] is going to reduce but we your we would have checked your your [BODY_MEASUREMENT: oxygen saturation] and we will see that it is fine so there will be no need to place you on on [MEDICINE: oxygen] so you are going to have you do a [LABORATORY_DATA: full blood count in sputum] and [LABORATORY_DATA: microscopy culture sensitivity] you are going to have you do any [LABORATORY_DATA: erythrocyte segmentation rate] and you are going to do a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] so let us see if it is a [PROBLEM: structural problem] or a [PROBLEM: functional problem] do you understand okay doctor so doctor do i do you want to ask the question if you have any questions yes i was going to ask that are you going to keep me in the hospital or do i that can i can i be treated from home because i do not know we we we are going to admit you for some time to evaluate you and because of the [PROBLEM: breathlessness] you are having right and then we will start you on on [MED_ROUTE: intravenous] [MED_ROUTE: intravenous]  that is okay that is cool [LABORATORY_DATA: culture] and [LABORATORY_DATA: sensitivity] could take about seventytwo hours to to five days before it will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just yeah i will just do the [LABORATORY_DATA: labs] and wait for just for you to start the [PROCEDURE: treatment] thank you</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not too fine i am not too fine not too fine that is why i came to the hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also [INS:at] what is [INS:the] [INS:complaints] so doctor also have been [INS:coughing] for about [INS:a] week now and [INS:i] have been also you also have what so and i also have i have also been running temperature for about five days so [INS:it] is been really you have been running temperature for five days yes yes and [INS:the] [INS:cough] has been for [INS:the] [INS:cough] has been for how long for about a week now a week yes yes and [INS:the] [INS:cough] has been for how long for about [INS:a] week now [INS:a] week yes okay all right so the cough did it start suddenly or gradually the cough started suddenly just started like that so i just just woke up more morning and started coughing about a week ago yes was there was there any symptoms like catarrh or any any difficulty in swallowing before the cough started [DEL:no] none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like barking does it sound like it is comes in bouts and then you have to take a deep breath when when you say barking do you are you [DEL:do] you mean like a dog or what do you mean by barking yes yes [INS:it] sounds like a dog barking no no no no no [DEL:no] mine is not like that i did not [DEL:i] did not experience anything like that okay so is the cough productive [SUB:of-&gt;or] phlegm yes yes it is productive when i yes when [DEL:i] cough i bring out some some substance from my mouth yes so what is the colour of the substance stuff err it is about yeah it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like vomiting i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough [SUB:no-&gt;cough] no there was not nothing i was not i had nothing my my even when i was coughing my chest was not paining me nothing it was just the cough then i [DEL:i] discovered after a few days after that i just [SUB:started-&gt;tired] running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not paining me at all your [DEL:chest] was not [DEL:paining] [DEL:me] is there anybody coughing around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and [SUB:at-&gt;i] work too there is nobody coughing around me so okay so you stay [INS:in] [INS:the] alone you are not here in [SUB:an-&gt;a] overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i [SUB:started-&gt;said] to have some difficulty in breathing so like that got me really scared like i was [DEL:i] was [DEL:i] was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to come completely to see you you are finding it difficult to breathe yes yes when you sleep at night [INS:do] you sweat excessively no at all i do not [DEL:i] [DEL:do] not slept [DEL:i] [DEL:do] not sweat when [DEL:i] sleep [DEL:at] night okay so what is what relieves the breathlessness any change [DEL:in] position that relieves the breathlessness or is it is constant [DEL:no] it is not associated with any any position nothing [DEL:i] just it just comes and goes like i just feel [SUB:breathless-&gt;breathlessness] for a while then it relieves me then it comes again especially when i am especially when [DEL:i] [DEL:am] coughing okay has this worsened progressively yes yes it has gotten very bad doctor that is why i came to the hospital does it affect does [DEL:it] affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that i have [DEL:i] have not been feeling well generally in my body so that is so now this fever that you were having was [DEL:it] did it start suddenly or gradually it started [DEL:it] [DEL:started] gradually then became i became very hot and it has been like that [DEL:it] has been like that so the fever is high grade you are very hot yes yes it is high did you at attend any point yes check by yourself at home your [SUB:temperature-&gt;job] yes i did i did i have [SUB:a-&gt;about] [SUB:thermometer-&gt;thirtyeightnine] it was about was about [DEL:thirtyeightnine] [DEL:thirtyeightnine] okay and what does what do you do that relieves the fever i took some [SUB:i-&gt;prost] took some [DEL:paracetamol] it relieved a bit then but it did did not last long [SUB:i-&gt;it] just [DEL:i] [DEL:i] became hot again and it has been like that ever since so i just want to ask you some questions has this anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why [DEL:i] [DEL:am] this is [DEL:the] first time [DEL:i] [DEL:am] experiencing this kind of thing okay this is the first time are you do you have any any medical condition like are you asthmatic [INS:do] you during your blood group and genotype [INS:oh] no i am not [INS:a] doctor i am fine no i have nothing and that is why this is surprising are you [SUB:hypertensive-&gt;a] what did you say i cannot hear you properly sir are you hypertensive or diabetic none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just [SUB:i-&gt;tried] just tried to get some cough syrup but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew [DEL:i] know [DEL:i] needed to like come [DEL:to] speak to someone to a doctor so that is why i came today for you to like for [DEL:me] [DEL:to] like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that i can remember have you done any surgical procedure before no [DEL:no] okay so i am just going to ask you some other questions just to know what exactly could be related to your [DEL:to] the symptoms you are having so do you have [INS:a] headache headache [INS:it] just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;kata] no at all okay do you have any abdominal pain no no [DEL:i] do not have any [SUB:diarrhea-&gt;abdominal] [SUB:or-&gt;pain] [DEL:vomiting] no i have [INS:no] not [SUB:vomited-&gt;pain] at all [INS:no] [INS:do] you have any bone pain yes hmm thank you no [INS:i] have not [INS:vomited] [INS:at] [SUB:the-&gt;all] no [INS:do] you have any [SUB:the-&gt;bone] most [SUB:it-&gt;yes] is just it is just the shortest of breath [SUB:i-&gt;that] have been having the difficulty in breathing [SUB:i-&gt;that] have been having that is just that is just so in summary you are telling me [DEL:in] summary you are telling [DEL:me] you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have [DEL:to] examine you right i am going to have to examine you and i am going to have to listen to your chest to know [DEL:if] [DEL:to] know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and [SUB:the-&gt;a] and [DEL:the] cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your [SUB:the-&gt;deflame] [DEL:phlegm] and we are going to send it for culture sensitivity to know what bacteria is is being cultured please i just want to ask you do you smoke no no i do not doctor i am a good christian i do not smoke i do not drink you do not you [DEL:do] not drink alcohol either i do not [SUB:i-&gt;drink] [DEL:do] not [DEL:do] any of those i do not do drugs i do not [SUB:do-&gt;drink] any of that i am going to ask you some other questions do you have they their kind of personal questions can i go ahead yeah i just want to know doctor i just want to [DEL:i] just want [DEL:to] be fine i just want to know how soon you can start treating me and what i will need [DEL:to] take basically [DEL:i] just want to ask [INS:if] ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex i am married no not at all not at all i am already [INS:i] [INS:am] married so we are going to start you from the history and the examination [SUB:we-&gt;you] have done and then [SUB:we-&gt;i] are going to ask you to do some investigations however we have some different differentials like diagnosis [SUB:the-&gt;because] because the because of what is causing the cough and the fever we have some this [SUB:thing-&gt;in] [DEL:at] the back of our mind which could be the because [DEL:do] you understand [SUB:we-&gt;you] think you have a pneumonia pneumonia [DEL:a] chest infection so we are going to start you on [SUB:a-&gt;the] [SUB:broad-&gt;blood] spectrum antibiotics right and then we are going to start you [DEL:on] [DEL:the] cough [SUB:syrup-&gt;serum] right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start treatment with the antibiotics and and the cough syrup there will [DEL:be] the breathlessness is going to reduce but we your [DEL:we] would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on [DEL:on] oxygen so you are going to have you do a full blood count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscop] [SUB:culture-&gt;contrast] sensitivity you are going to have you do any [SUB:erythrocyte-&gt;ultrasound] segmentation rate and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor so doctor [DEL:do] [DEL:i] [DEL:do] you want to ask [INS:me] [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any question questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital or do i that can i can i be treated from home because i do not know we we [DEL:we] are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then [SUB:we-&gt;okay] will [SUB:start-&gt;okay] you [SUB:on-&gt;okay] [SUB:on-&gt;okay] [SUB:intravenous-&gt;okay] [SUB:intravenous-&gt;okay] that is okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay that is cool [SUB:culture-&gt;investigation] and sensitivity could take about seventytwo hours to [SUB:to-&gt;find] five days before [SUB:it-&gt;to] will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just [INS:do] [INS:the] [INS:labs] and wait for you [INS:to] [INS:start] [INS:the] [INS:treatment] thank you very much [INS:i] think that is fine [INS:i] will just yeah i will just do the labs and wait for just for you to start the treatment thank you [INS:no] [INS:i] [INS:do] not promise</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to [SUB:the-&gt;you] hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also also [INS:at] have you also have what so and i also have i have also been running temperature for about five days so [INS:it] is been really yes yes and you have running [SUB:temperature-&gt;been] for five days yes yes for how long for about a week now a week yes okay [SUB:all-&gt;alright] right so the cough did it start suddenly or gradually the cough started suddenly just started like that i just just woke [DEL:up] more morning and [DEL:started] [DEL:coughing] about [DEL:a] week ago yes was there was there any symptoms like [SUB:catarrh-&gt;qatar] or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like [INS:the] barking does it sound like [INS:a] and it is comes in bouts and then you have to take a deep breath when when you say barking [DEL:do] you are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] mine is not that [SUB:i-&gt;no] did not [SUB:i-&gt;no] did not experience anything like that okay so is [SUB:the-&gt;no] [SUB:cough-&gt;no] productive [SUB:of-&gt;no] [SUB:phlegm-&gt;no] yes yes [SUB:it-&gt;no] is productive when [SUB:i-&gt;no] yes when [SUB:i-&gt;no] [SUB:cough-&gt;no] [SUB:i-&gt;no] bring [SUB:out-&gt;no] some some substance from my mouth yes so what is the colour of the substance err it is about yeah it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was [DEL:no] [DEL:blood] [DEL:in] [DEL:it] at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [INS:i] [SUB:vomiting-&gt;am] i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough no no there was not [INS:in] nothing i was not i had nothing my my even when i was coughing my chest was not [SUB:paining-&gt;burning] me nothing it was just the cough then i i discovered after a few days after that i just [DEL:started] running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not [INS:pain] [SUB:paining-&gt;in] me at all your chest was not [INS:pain] [SUB:paining-&gt;in] me is there anybody coughing around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and [SUB:at-&gt;i] work too there is nobody coughing around me so okay so you stay alone you are not here in [SUB:an-&gt;a] overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i started to have some difficulty in breathing so like that got me really scared like i was i was [DEL:i] was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to come completely to see you so you are finding it difficult to breathe yes [INS:the] [INS:cough] yes when you sleep at night [INS:do] you sweat excessively no at all i do not i do not slept i do not sweat when [SUB:i-&gt;a] sleep [SUB:at-&gt;department] night okay so what is what relieves the breathlessness any change [DEL:in] position that relieves the breathlessness or [DEL:it] is constant no it is not associated with any any position nothing [SUB:i-&gt;and] just it just comes and goes like i just feel breathless for a while then it relieves me then it comes again especially when [DEL:i] [DEL:am] especially when i am coughing okay has this worsened progressively yes yes [SUB:it-&gt;that] has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that i have [DEL:i] have not been feeling well generally [DEL:in] my [DEL:body] so that is so now this fever that you were having was it did it start suddenly or gradually [DEL:it] started it started gradually then became i became very hot and [DEL:it] has been like that it has been like that so the fever is high grade you are very hot yes yes it is [SUB:high-&gt;i] did you [SUB:at-&gt;have] any points that point yes check by yourself at home your temperature yes i did i did i have a [SUB:thermometer-&gt;stomach] [SUB:it-&gt;i] was about there was about [INS:thirty] [INS:eight] point [INS:nine] [INS:thirty] [SUB:thirtyeightnine-&gt;point] [SUB:thirtyeightnine-&gt;nine] okay and what does what do you do that relieves the fever well i took some i took some past [SUB:paracetamol-&gt;more] it relieved [SUB:a-&gt;the] bit then but it did did not last long i just i [DEL:i] became hot again and it has been like that ever since so i just want to ask you some questions has anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why [DEL:i] [DEL:am] this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic [INS:do] you during your [SUB:blood-&gt;need] [SUB:group-&gt;a] and genotype no i am not [INS:to] doctor i am fine no i have nothing and that is why this is surprising are you [INS:a] hypertensive what did you say [DEL:i] cannot hear you properly sir are you hypertensive or diabetic none none none none no [DEL:no] i have none of them i have none of them so what have you what have you done to care for yourself so far i just [SUB:i-&gt;try] just [DEL:i] just tried to get some cough syrup [INS:up] but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew i know i needed to like come to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that [SUB:i-&gt;current] can remember have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your [SUB:to-&gt;so] the symptoms you are having so do you have headache headache [INS:it] just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain no no [SUB:i-&gt;no] [SUB:do-&gt;no] not have any [SUB:diarrhea-&gt;no] [SUB:or-&gt;no] [SUB:vomiting-&gt;no] no [SUB:i-&gt;no] have not [SUB:vomited-&gt;no] [SUB:at-&gt;no] [SUB:all-&gt;no] you have any [SUB:bone-&gt;no] [SUB:pain-&gt;no] yes no [SUB:the-&gt;no] no [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [SUB:the-&gt;no] most [SUB:it-&gt;no] is just [SUB:it-&gt;of] is just the shortest of breath [DEL:i] have been having the difficulty in breathing [DEL:i] have been having that is just that is just so [DEL:in] summary you are telling me in summary you are telling me you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes [SUB:all-&gt;alright] right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know [DEL:if] to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and the and the cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count [INS:or] a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your the phlegm and we are going to send it for culture sensitivity to know what bacteria is is being cultured please i just want to ask you do you smoke no no i do not so doctor i am a good christian i do not smoke i do not drink you do not you do not drink alcohol either i do not i do not do any of those i do not do [SUB:drugs-&gt;jobs] i do not do any of that i am going to ask you some other questions do you have there their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i [INS:do] will need to take basically i just want [DEL:to] ask ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex [DEL:i] [DEL:am] married no not at all not at all [DEL:i] [DEL:am] married so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because [DEL:the] because of what is causing the cough and the fever we have some this [SUB:thing-&gt;in] [DEL:at] the back of our mind which could be the because do you understand we think you have a pneumonia pneumonia [DEL:a] chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start you on [DEL:the] cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start [SUB:treatment-&gt;treatments] with the antibiotics and and the cough syrup there will be the breathlessness business is going to reduce but we your we would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on on oxygen so you are going [SUB:to-&gt;having] have you do [DEL:a] full [SUB:blood-&gt;block] [SUB:count-&gt;out] in sputum and end [SUB:microscopy-&gt;microscopic] culture sensitivity you are going to have you doing [SUB:do-&gt;the] any [SUB:erythrocyte-&gt;site] [SUB:segmentation-&gt;sedimentation] [SUB:rate-&gt;rates] and you are going to do a chest xray so let us see if it is [DEL:a] structural problem or a functional problem do you understand okay doctor so doctor do [DEL:i] [DEL:do] you want to ask [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital or do i have that can [SUB:i-&gt;home] can i be treated from home because i do not know we [DEL:we] [DEL:we] are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then [DEL:we] will [DEL:start] you [DEL:on] [DEL:on] [DEL:intravenous] [DEL:intravenous] that is okay that is cool [SUB:culture-&gt;so] and [DEL:sensitivity] could take about seventytwo hours [DEL:to] [DEL:to] five days before [DEL:it] will [DEL:be] ready [DEL:do] you understand yeah [DEL:no] [DEL:problem] doctor thank you [DEL:no] [DEL:problem] doctor thank you very much i think that is fine i will just yeah i will just do the [SUB:labs-&gt;laps] and wait for just for you to start the treatment thank you</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine [INS:on] not too fine that is why i came to the hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also also have you also have what so and i also have [DEL:i] have also been running temperature for about five days so you have running [DEL:temperature] for five days yes yes and [INS:the] [INS:cough] has been for [INS:the] [INS:cough] has been for how long for about a week now a week yes okay all right so the cough did [SUB:it-&gt;this] start soddening suddenly or gradually the cough started suddenly just started like that i just just woke up more morning and started coughing about a week ago yes was there was there any symptoms like [SUB:catarrh-&gt;qatar] or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like [SUB:barking-&gt;backing] does [SUB:it-&gt;this] sound like it is comes in bouts and then you have to take a deep [DEL:breath] when when you say [SUB:barking-&gt;backing] [DEL:do] you are you do you mean like a dog or what do you mean by [SUB:barking-&gt;backing] yes yes sounds like a dog [SUB:barking-&gt;back] no no no no no [DEL:no] mine is not that [DEL:i] did not [DEL:i] did not experience anything like that okay so is the cough productive of [SUB:phlegm-&gt;flame] yes yes it is productive when [DEL:i] yes when i cough i bring out some some substance from my mouth yes so what is the colour of the substance err it is about yeah it is clear it is whitish it is not [DEL:it] is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [DEL:vomiting] i do not vomit at all okay and you did not have [SUB:catarrh-&gt;catar] or difficulty in swallowing prior to [INS:the] onset of the cough no no [INS:no] there was nothing i was not i had nothing my my even when i was coughing my chest was not [SUB:paining-&gt;painting] me nothing it was just the cough then i [DEL:i] discovered after a few days after that i just [SUB:started-&gt;hired] running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is [DEL:no] cough there is no chest pain no there is there is no chest pain my chest was not paining me at all your [SUB:chest-&gt;just] was not [SUB:paining-&gt;pain] [DEL:me] is there anybody coughing around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have [DEL:anybody] around [DEL:me] that is coughing too and [SUB:at-&gt;i] work too there is nobody coughing around me so okay so you stay alone you are not here in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was [DEL:i] [DEL:started] to have some difficulty in breathing so like that got me really scared like i was [DEL:i] was [DEL:i] was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to come completely to see you you are finding it difficult to breathe yes yes when you sleep at night [INS:do] you sweat excessively no at all i do not [SUB:i-&gt;sleep] [DEL:do] not slept i do not sweat when [SUB:i-&gt;okay] sleep [DEL:at] night okay so what is what relieves the breathlessness any change in position that relieves the breathlessness or [SUB:it-&gt;this] is constant no it is not associated with any any position nothing i just it just comes and goes like i just feel breathless for a while then it relieves me then it comes again especially when i am especially when i am coughing okay has this worsened progressively yes yes [SUB:it-&gt;that] has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that i have [DEL:i] have not been feeling well generally in my body so that is so now this fever that you were having was it did [SUB:it-&gt;you] start suddenly [SUB:or-&gt;it] gradually it started [DEL:it] [DEL:started] gradually then became i became very hot and [DEL:it] has been like that it has been like that so the fever is [SUB:high-&gt;highgrade] [DEL:grade] you are very hot yes yes it is high did you attend [INS:a] [SUB:at-&gt;question] any point yes check by yourself at home your temperature yes i did i did i have [DEL:a] thermometer [SUB:it-&gt;i] was about was about thirtyeightnine [SUB:thirtyeightnine-&gt;thirtynine] okay and what does what do you do that relieves the fever i took some [SUB:i-&gt;past] took some [DEL:paracetamol] it relieved [SUB:a-&gt;the] bit then but it did [INS:it] did not last long [INS:it] [SUB:i-&gt;is] just [SUB:i-&gt;it] [DEL:i] became hot again and it has been like that ever since so i just want to ask you some questions has this anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why i am this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic [INS:do] you during your blood group and genotype [INS:oh] no i am not doctor i am fine no i have nothing and that is why this is surprising are you [SUB:hypertensive-&gt;hypocensing] what did you say i cannot hear you properly sir are you hypertensive or diabetic none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just [DEL:i] just [DEL:i] just tried to get some [INS:coughs] [SUB:cough-&gt;here] [SUB:syrup-&gt;up] but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew [DEL:i] knew [DEL:i] know i needed to like come [DEL:to] speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that [SUB:i-&gt;current] can remember have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the symptoms you are having so do you have headache headache yes just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain no no i do not have any [SUB:diarrhea-&gt;problem] [DEL:or] [DEL:vomiting] no i have not vomited at all you have any bone pain yes no [DEL:the] no the most it is just [DEL:it] is just the shortest of breath i have been having the difficulty in breathing [SUB:i-&gt;has] have been having that is just that is just so in summary you are telling me [SUB:in-&gt;some] summary you are telling me you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know if to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and the and [DEL:the] cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count [INS:of] a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your the [SUB:phlegm-&gt;flame] and we are going to send it for [SUB:culture-&gt;cultural] sensitivity to know what bacteria is is being [SUB:cultured-&gt;caught] please i just want to ask you do you smoke no no i do not so doctor i am a good christian i [SUB:do-&gt;just] not [DEL:smoke] i do not [SUB:drink-&gt;think] you do not you [DEL:do] not drink alcohol either i do not [SUB:i-&gt;drink] [DEL:do] not [DEL:do] any of those i do not do drugs i do not [SUB:do-&gt;drink] any of that i am going to ask you some other questions do you have there their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i will need [DEL:to] take basically [DEL:i] just want to ask [INS:if] ifi just want to ask if you have multiple sexual partners and then your sexual practices no no [INS:do] you have oral sex i am married no not at all not at all [DEL:i] [DEL:am] married so we are going to start you from the history and the examination [SUB:we-&gt;you] have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because [DEL:the] because of what is causing the cough and the fever we have some this [DEL:thing] at the back of our mind which could be the because [DEL:do] you understand we think you have a pneumonia [DEL:pneumonia] a chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start you on the cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start treatment with the antibiotics and and the cough syrup there will be the breathlessness is going to reduce but we your [DEL:we] would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on [DEL:on] oxygen so you are going to have you do a full [SUB:blood-&gt;block] count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscopic] [SUB:culture-&gt;control] sensitivity you are going to have you do any [SUB:erythrocyte-&gt;intrusive] [SUB:segmentation-&gt;sedimentation] rate and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor so doctor [DEL:do] [DEL:i] [DEL:do] you want to ask [INS:me] [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital [DEL:or] [DEL:do] [DEL:i] that can i can [DEL:i] be treated from home because i do not know we [DEL:we] [DEL:we] are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then [DEL:we] will [DEL:start] you [DEL:on] [DEL:on] [DEL:intravenous] [DEL:intravenous] that is okay that is cool [DEL:culture] and [DEL:sensitivity] could take about seventytwo hours to [DEL:to] five days before [SUB:it-&gt;you] will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just yeah i will just do the labs and wait for just for you to start the treatment thank you</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1381,22 @@
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may i help you yeah good afternoon my name is miss sharon  yes okay so do you have any [UMLS/C5441521: Complaint (finding)] yes doctor i have been stooling for about four days now and i have been [UMLS/C0000737: Abdominal Pain] two alongside so that is those are my two [UMLS/C5441521: Complaint (finding)] okay okay so which one started first the stooling or the [UMLS/C0000737: Abdominal Pain] yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is it watery is he semi solid or it is in normal form well formed stools it is very watery very watery very watery yes okay all right so like how many episodes of  you said you have been stolen for over four days right yes and how many episodes do you do you have per day of stooling my about six about six to seven episodes actually about around that of passage of watery stool yes yes yes doctor okay okay so  is the stool containing mucus is it [UMLS/C0225345: Mucous connective tissue] no no there is no [UMLS/C3550578: Abnormal mucus] no [UMLS/C3550578: Abnormal mucus] in it was there any [UMLS/C0005822: Blood Preservation] in it no [UMLS/C0005822: Blood Preservation] at all there is no [UMLS/C0005822: Blood Preservation] in it okay did you change did you eat a from a new restaurant or did you did you eat something different ermactually a few days ago i like just before it started i actually had a take out in a restaurant with my family which all of us ate and  one of my child actually [UMLS/C0042963: Vomiting] but [UMLS/C0042963: Vomiting] stopped and he feels good now so it is just me right now with the [UMLS/C5441521: Complaint (finding)] i have of the of the [UMLS/C2129214: Loose stool] are you also [UMLS/C0042963: Vomiting] yes ii [UMLS/C0042963: Vomiting] about two two episodes about two times yes what what what what was inside the [UMLS/C0042963: Vomiting] what was the components of the [UMLS/C5867201: Iflavirus vomitus] was it what you ate or was it greenish or was there [UMLS/C0005822: Blood Preservation] in it no there was no [UMLS/C0005822: Blood Preservation] it was just the content of what i ate was the [UMLS/C0042963: Vomiting] was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know it just i just [UMLS/C0042963: Vomiting] that is all i i cannot really remember how you came out to be honest okay was there any is there any [UMLS/C0000731: Abdomen distended] distension like a [UMLS/C0038999: Swelling] [UMLS/C0038999: Swelling] yeah was there [UMLS/C0038999: Swelling] in your [UMLS/C0038351: Stomach] no just the [UMLS/C0000737: Abdominal Pain] the [UMLS/C0030193: Pain] is just at my the lower part of my [UMLS/C0038351: Stomach] okuhm all right all right thank you so you said your son also ate ate the same the same food that you bought and he is now [UMLS/C0042963: Vomiting] how is he feeling now he feels he is okay he after the episode of [UMLS/C0042963: Vomiting] he he got he got well and he is okay how is your [UMLS/C0003618: Desire for food] like my [UMLS/C0003618: Desire for food] is is here and there know it is not really good like so now let us okay okay so let us talk about let us talk about your the [UMLS/C0030193: Pain] you were having so can you describe the [UMLS/C0030193: Pain] for me what is the what is the nature of the [UMLS/C0030193: Pain] is it a [UMLS/C1444775: Sharp sensation quality] [UMLS/C0030193: Pain] or a [UMLS/C0030193: Pain] that holds you and leaves you whatwhat kind of [UMLS/C0030193: Pain] is it yeah i will describe it like like has a [UMLS/C0458254: Cramping Pain] like the [UMLS/C0030193: Pain] i feel during [UMLS/C0025344: Menstruation] so that is the kind of [UMLS/C0030193: Pain] like that is the way i can describe it and where where is this [UMLS/C0030193: Pain] located in your [UMLS/C0000726: Abdomen] the lower part the lower part does this [UMLS/C0030193: Pain] does it move to another part of your [UMLS/C0444584: Whole body] when you start feeling it no just just the lower part of my like moving to the [UMLS/C0004600: Back] just the lower part it does not move to your [UMLS/C0004600: Back] no no not at all it stays in the same space yes yes okay okay so what what do you think makes this [UMLS/C0030193: Pain] [UMLS/C1457868: Worse] well maybe if i if i do not eat i do not know if i do not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse per se but i will say maybe if i do not eat yes okay what what what relieves the [UMLS/C0030193: Pain]  nothing i do not know i do not know anything that reduce the [UMLS/C0030193: Pain] it just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any [UMLS/C0030193: Pain] at all and ten is the worst [UMLS/C0030193: Pain] you have felt in your life so what would you give this [UMLS/C0030193: Pain] i will the [UMLS/C0030193: Pain] like five or ten five  ten yes no [UMLS/C0033213: Problem] so  let us yeah take some history do you have are you [UMLS/C0020538: Hypertensive disease] no i am not are you [UMLS/C0011847: Diabetes] no i am not do you are you a known [UMLS/C0014869: Peptic Esophagitis] also patient no no are you [UMLS/C0022949: lactose] intolerant no the only the only ailment i am being treated for i am being treated for is [UMLS/C0004096: Asthma] i am a known [UMLS/C0004096: Asthma] and and i am on i use [UMLS/C0242903: Anesthetics, Inhalation] and how many how many exacerbations do you have in a year about in the last one just one okay okay that is good have you had any previous history of [UMLS/C0005841: Blood Transfusion] any history of [UMLS/C0543467: Operative Surgical Procedures] no no none at all okay   do you drink [UMLS/C0001962: ethanol] or do you [UMLS/C0037366: Smoke] no i do not i do not do any of those i do not at all and since you have been feeling these [UMLS/C1457887: Symptoms] that you are having has has it progressively worsened yeah i i feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel [UMLS/C0232132: Weak arterial pulse] yeah i feel kind of [UMLS/C0232132: Weak arterial pulse] yeah yeah my my i feel sometimes my [UMLS/C0226896: Oral cavity] is kind of dry to kind of okay okay okay no [UMLS/C0033213: Problem] so do you asides the [UMLS/C0004096: Asthma] do you have any other ailments you think the doctor should know about no not at all at all i have no other no other medical condition do you have any [UMLS/C0013182: Drug Allergy] no i do not react no at all i do not react to any [UMLS/C0013227: Pharmaceutical Preparations] at all okay please are you married yes i am married with two kids  yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [UMLS/C0042963: Vomiting] was there any any of your family members that also had the same [UMLS/C1457887: Symptoms] no no no no no other just me just me and my son yes okay no [UMLS/C0033213: Problem] okay do you i am just going to ask some questions just to rule out every other thing do you do you have [UMLS/C0018681: Headache] no doctor do you have [UMLS/C0817096: Chest] [UMLS/C0030193: Pain] no doctor at all no do you have an [UMLS/C0000737: Abdominal Pain] oh do you you have an [UMLS/C0000737: Abdominal Pain] do you have any change in your bowel habits  i do not know how to answer that other than the just the  the okay i think i think i think that is fine your [UMLS/C0042036: Urine] your your [UMLS/C0042036: Urine] has it has it changed in quantity no not at all how about the [UMLS/C0016708: Micturition frequency and polyuria] has it changed no no my [UMLS/C0042034: Urination] is fine do you have any do you have any [UMLS/C0005931: Bone and Bones] [UMLS/C0030193: Pain] no all right no [UMLS/C0033213: Problem] so ermthank you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a [UMLS/C0033213: Problem] and they can also come to have differential diagnosis of what could be the because of your [UMLS/C1457887: Symptoms] and we would like to examine you right check your level of [UMLS/C0204837: Hypodermoclysis] check your general physical appearance to see whether you and access your your general health right we also like to do an [UMLS/C0562238: abdominal examination] right to to also give us more information on the [UMLS/C0000737: Abdominal Pain] you are having if you could lead us to what is causing the [UMLS/C1457887: Symptoms] you are having the [UMLS/C0000737: Abdominal Pain] and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some [UMLS/C0009450: Communicable Diseases] which could have which could have caused the [UMLS/C0011991: Diarrhea] you want to say something so what exactly is wrong what exactly is wrong what exactly is the because okay it is just the food i ate right so yeah it looks like you have had a [UMLS/C0016479: Food Poisoning] had a [UMLS/C0016479: Food Poisoning] but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your [UMLS/C0009555: Complete Blood Count] to know if there is a there is some [UMLS/C0009450: Communicable Diseases] which could be [UMLS/C0017160: Gastroenteritis] we want to do your [UMLS/C0005833: Blood Sedimentation] rates to know if there is any sign any any type of kind of [UMLS/C1290884: Inflammatory disorder] that could cause [UMLS/C0011991: Diarrhea] like [UMLS/C0021390: Inflammatory Bowel Diseases] right and then we would also want to do a [UMLS/C0015733: Feces] and sensitivity and to look out for [UMLS/C0597428: Sedimentation procedure] and some [UMLS/C0003244: Antibodies, Bacterial] that could cause you to be having [UMLS/C0011991: Diarrhea] we also check your retroviral status to know if you have [UMLS/C0035366: Retroviridae] which could also be a because of of [UMLS/C0011991: Diarrhea] although that comes in the chronic chronic setting however would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some [UMLS/C0011947: Dialysis Solutions] to you know give you some strength and restore your [UMLS/C0002371: aluminum hydroxide] because you have been losing some [UMLS/C0016286: Fluid Therapy] from from the stooling and the [UMLS/C0042963: Vomiting] we will also check your [UMLS/C0013832: Electrolytes] [UMLS/C0013832: Electrolytes] to know what is your [UMLS/C0013832: Electrolytes] picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an [UMLS/C0034606: Radionuclide Imaging] throughout any structural or functional [UMLS/C0033213: Problem] that could be in the [UMLS/C0000726: Abdomen] which would be could be causing the [UMLS/C0011991: Diarrhea] and the the the [UMLS/C0000737: Abdominal Pain] do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine  yeah so that will be fine thank you so you will be attended to all right thank you very much doctor</t>
+          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may i help you yeah good afternoon my name is miss sharon  yes okay so do you have any [PROBLEM: complaints] yes doctor i have been stooling for about four days now and i have been [PROBLEM: abdominal pain] two alongside so that is those are my two [PROBLEM: complaints] okay okay so which one started first the stooling or the [PROBLEM: abdominal pain] yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is it watery is he semi solid or it is in normal form well formed stools it is very watery very watery very watery yes okay all right so like how many episodes of  you said you have been stolen for over four days right yes and how many episodes do you do you have per day of stooling my about six about six to seven episodes actually about around that of passage of watery stool yes yes yes doctor okay okay so  is the stool containing mucus is it [ANATOMICAL_STRUCTURE: mucoid] no no there is no [PROBLEM: mucus] no [PROBLEM: mucus] in it was there any [PROBLEM: blood] in it no [PROBLEM: blood] at all there is no [PROBLEM: blood] in it okay did you change did you eat a from a new restaurant or did you did you eat something different ermactually a few days ago i like just before it started i actually had a take out in a restaurant with my family which all of us ate and  one of my child actually [PROBLEM: vomited] but [PROBLEM: vomiting] stopped and he feels good now so it is just me right now with the [PROBLEM: complaints] i have of the of the [PROBLEM: loose stool] are you also [PROBLEM: vomiting] yes ii [PROBLEM: vomited] about two two episodes about two times yes what what what what was inside the [PROBLEM: vomit] what was the components of the [PROBLEM: vomitus] was it what you ate or was it [PROBLEM: greenish] or was there [PROBLEM: blood] in it no there was no [PROBLEM: blood] it was just the content of what i ate was the [PROBLEM: vomiting] was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know it just i just [PROBLEM: vomited] that is all i i cannot really remember how you came out to be honest okay was there any is there any [PROBLEM: abdominal distension] distension like a [PROBLEM: swelling] [PROBLEM: swelling] yeah was there [PROBLEM: swelling] in your [ANATOMICAL_STRUCTURE: stomach] no just the [PROBLEM: abdominal pain] the [PROBLEM: pain] is just at my the lower part of my [ANATOMICAL_STRUCTURE: stomach] okuhm all right all right thank you so you said your son also ate ate the same the same food that you bought and he is now [PROBLEM: vomiting] how is he feeling now he feels he is okay he after the episode of [PROBLEM: vomiting] he he got he got well and he is okay how is your [BODY_FUNCTION: appetite] like my [BODY_FUNCTION: appetite] is is here and there know it is not really good like so now let us okay okay so let us talk about let us talk about your the [PROBLEM: pain] you were having so can you describe the [PROBLEM: pain] for me what is the what is the nature of the [PROBLEM: pain] is it a [SEVERITY: sharp] [PROBLEM: pain] or a [PROBLEM: pain] that holds you and leaves you whatwhat kind of [PROBLEM: pain] is it yeah i will describe it like like has a [PROBLEM: cramp pain] like the [PROBLEM: pain] i feel during [BODY_FUNCTION: menstruation] so that is the kind of [PROBLEM: pain] like that is the way i can describe it and where where is this [PROBLEM: pain] located in your [ANATOMICAL_STRUCTURE: abdomen] the lower part the lower part does this [PROBLEM: pain] does it move to another part of your [ANATOMICAL_STRUCTURE: body] when you start feeling it no just just the lower part of my like moving to the [ANATOMICAL_STRUCTURE: back] just the lower part it does not move to your [ANATOMICAL_STRUCTURE: back] no no not at all it stays in the same space yes yes okay okay so what what do you think makes this [PROBLEM: pain] [SEVERITY: worse] well maybe if i if i do not eat i do not know if i do not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse per se but i will say maybe if i do not eat yes okay what what what relieves the [PROBLEM: pain]  nothing i do not know i do not know anything that reduce the [PROBLEM: pain] it just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any [PROBLEM: pain] at all and ten is the worst [PROBLEM: pain] you have felt in your life so what would you give this [PROBLEM: pain] i will the [PROBLEM: pain] like five or ten five  ten yes no [PROBLEM: problem] so  let us yeah take some history do you have are you [PROBLEM: hypertensive] no i am not are you [PROBLEM: diabetic] no i am not do you are you a known [PROBLEM: peptic] also patient no no are you [MEDICINE: lactose] intolerant no the only the only ailment i am being treated for i am being treated for is [PROBLEM: asthma] i am a known [PROBLEM: asthmatic] and and i am on i use [MEDICINE: inhalers] and how many how many exacerbations do you have in a year about in the last one just one okay okay that is good have you had any previous history of [PROCEDURE: blood transfusion] any history of [PROCEDURE: surgeries] no no none at all okay   do you drink [SUBSTANCE_ABUSE: alcohol] or do you [SUBSTANCE_ABUSE: smoke] no i do not i do not do any of those i do not at all and since you have been feeling these [PROBLEM: symptoms] that you are having has has it progressively worsened yeah i i feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel [PROBLEM: weak] yeah i feel kind of [PROBLEM: weak] yeah yeah my my i feel sometimes my [ANATOMICAL_STRUCTURE: mouth] is kind of dry to kind of okay okay okay no [PROBLEM: problem] so do you asides the [PROBLEM: asthma] do you have any other ailments you think the doctor should know about no not at all at all i have no other no other medical condition do you have any [PROBLEM: drug allergies] no i do not react no at all i do not react to any [MEDICINE: drugs] at all okay please are you married yes i am married with two kids  yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [PROBLEM: vomiting] was there any any of your family members that also had the same [PROBLEM: symptoms] no no no no no other just me just me and my son yes okay no [PROBLEM: problem] okay do you i am just going to ask some questions just to rule out every other thing do you do you have [PROBLEM: headaches] no doctor do you have [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] no doctor at all no do you have an [PROBLEM: abdominal pain] oh do you you have an [PROBLEM: abdominal pain] do you have any change in your bowel habits  i do not know how to answer that other than the just the  the okay i think i think i think that is fine your [LABORATORY_DATA: urine] your your [LABORATORY_DATA: urine] has it has it changed in quantity no not at all how about the [PROBLEM: frequency of urination] has it changed no no my [BODY_FUNCTION: urination] is fine do you have any do you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] no all right no [PROBLEM: problem] so [MEDICINE: ermthank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a [PROBLEM: problem] and they can also come to have differential diagnosis of what could be the because of your [PROBLEM: symptoms] and we would like to examine you right check your level of [PROCEDURE: hydration] check your general physical appearance to see whether you and access your your general health right we also like to do an [PROCEDURE: abdominal examination] right to to also give us more information on the [PROBLEM: abdominal pain] you are having if you could lead us to what is causing the [PROBLEM: symptoms] you are having the [PROBLEM: abdominal pain] and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some [PROBLEM: infection] which could have which could have caused the [PROBLEM: diarrhea] you want to say something so what exactly is wrong what exactly is wrong what exactly is the because okay it is just the food i ate right so yeah it looks like you have had a [PROBLEM: food poisoning] had a [PROBLEM: food poisoning] but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your [LABORATORY_DATA: blood count] to know if there is a there is some [PROBLEM: infection] which could be [PROBLEM: gastroenteritis] we want to do your [LABORATORY_DATA: erythrocyte sedimentation] rates to know if there is any sign any any type of kind of [PROBLEM: inflammatory disorder] that could cause [PROBLEM: diarrhea] like [PROBLEM: inflammatory bowel disease] right and then we would also want to do a [LABORATORY_DATA: stool culture microscopy] and sensitivity and to look out for [LABORATORY_DATA: parasites] and some [LABORATORY_DATA: bacteria] that could cause you to be having [PROBLEM: diarrhea] we also check your retroviral status to know if you have [PROBLEM: retroviral disease] which could also be a because of of [PROBLEM: diarrhea] although that comes in the chronic chronic setting however would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some [MEDICINE: fluids] to you know give you some strength and restore your [LABORATORY_DATA: hydration level] because you have been losing some [PROBLEM: fluid] from from the stooling and the [PROBLEM: vomiting] we will also check your [LABORATORY_DATA: electrolytes] [LABORATORY_DATA: electrolytes] to know what is your [LABORATORY_DATA: electrolyte] picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an [PROCEDURE: abdominal scan] throughout any structural or functional [PROBLEM: problems] that could be in the [ANATOMICAL_STRUCTURE: abdominal] which would be could be causing the [PROBLEM: diarrhea] and the the the [PROBLEM: abdominal pain] do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine  yeah so that will be fine thank you so you will be attended to all right thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may [DEL:i] help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about about four days now and i have been abdominal pain two alongside so that [DEL:is] those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the [SUB:stool-&gt;tool] is [SUB:it-&gt;he] watery is he semi solid or it is [DEL:in] normal form well from formed stools it is very watery very watery very watery yes okay all right so like how many episodes of you said you have been still stolen for over four days right yes and how many episodes do you [DEL:do] you have [SUB:per-&gt;for] day of stooling my about six about six to seven episodes actually about around that of passage of what watery [SUB:stool-&gt;to] yes yes yes yes doctor okay okay so is the stool containing [SUB:mucus-&gt;mucous] is it mucoid no no no there is no [SUB:mucus-&gt;mucous] no [SUB:mucus-&gt;mucous] in it was there any blood in it no blood at all there [SUB:is-&gt;was] no blood in it okay did you change did you eat [DEL:a] from a new restaurant or did you did you eat something different ermactually a few days ago [DEL:i] like just before it started i actually had a take [DEL:out] in a restaurant with my family which was all [SUB:of-&gt;heads] [DEL:us] ate and one of my child actually [SUB:vomited-&gt;vomitedited] but the vomiting stopped and [SUB:he-&gt;it] feels good now so it is just me right now with the complaints i have of the of the loose [SUB:stool-&gt;yes] are you also [DEL:vomiting] yes ii vomited about two two episodes about two times yes what what what what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomit] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know [SUB:it-&gt;i] just i just [SUB:vomited-&gt;wanted] that [SUB:is-&gt;tell] [SUB:all-&gt;so] [SUB:i-&gt;like] i cannot really remember how you came out to be honest okay was there any is there any abdominal distension distension like [DEL:a] swelling swelling yeah was there swelling in your stomach no just the muscle [INS:is] there any abdominal [INS:distension] [INS:distension] like [INS:swelling] [INS:swelling] yeah was there [INS:swelling] [INS:in] your [INS:stomach] no just [INS:abdominal] pain the pain is just at my the lower part of my stomach okuhm [SUB:all-&gt;alright] right [DEL:all] right thank you so you said your son also ate ate the same the same food that you bought and he is now vomiting how is he feeling now he feels he is okay [DEL:he] after the episode of vomiting he [DEL:he] got [DEL:he] got well and he is okay how is your appetite like my appetite is [DEL:is] here and there know it is not really good like [SUB:so-&gt;before] now let [DEL:us] okay okay so let us talk about let [DEL:us] talk about your the pain you were having so can you describe the pain for me what is the what [DEL:is] the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it [INS:i] will describe [INS:it] [INS:as] [INS:a] [INS:cramp] [INS:pain] like the yeah i feel [INS:do] you want [INS:me] [INS:to] show [INS:so] that [INS:is] [INS:a] kind [INS:of] [INS:pain] [INS:is] [INS:it] [INS:i] will describe it like like has a cramp pain like [INS:it] the [SUB:pain-&gt;been] [SUB:i-&gt;a] feel during menstruation so that is the kind of pain like that is the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just just the lower part [DEL:of] my like moving [DEL:to] the back just the lower part [DEL:it] does not move [DEL:to] your back no no not [DEL:at] [DEL:all] it stays in the same space yes yes okay okay so what what do you think makes this pain worse well maybe if i if i do not eat i do not know if i do not eat here maybe [INS:do] not know if [INS:i] [INS:do] not eat yeah maybe something around that yeah but i do not feel like if it just comes and goes i do not feel like there [INS:is] anything that makes you [SUB:it-&gt;to] [SUB:worse-&gt;want] [SUB:per-&gt;to] [SUB:se-&gt;say] but i will say maybe if i do not eat yes okay what what what relieves the pain [INS:i] [INS:am] not nothing i do not know i [SUB:do-&gt;did] not know when you anything that [INS:it] would reduce the [SUB:pain-&gt;that] it just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will give the pain like five [INS:out] [SUB:or-&gt;of] ten five five over ten yes no problem so let us yeah take some history [DEL:do] you have are you hypertensive no i am not are you diabetic no i am not [DEL:do] you are you a known [SUB:peptic-&gt;because] also patient no no are you lactose intolerant no the only the only ailment [SUB:i-&gt;be] [DEL:am] being treated for [SUB:i-&gt;you] [SUB:am-&gt;a] being treated for [SUB:is-&gt;no] [SUB:asthma-&gt;are] [SUB:i-&gt;you] [SUB:am-&gt;lactose] [SUB:a-&gt;intolerant] known [SUB:asthmatic-&gt;the] and and i have [SUB:am-&gt;been] [SUB:on-&gt;treated] [SUB:i-&gt;for] use [SUB:inhalers-&gt;asthmatic] and [INS:i] how many how many exacerbations do you have in a year about [DEL:in] the last one just one okay [INS:one] okay that is good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not [DEL:i] do not [DEL:do] any of those i do not [DEL:at] [DEL:all] and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i [DEL:i] feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my i feel sometimes my mouth is kind of dry [SUB:to-&gt;too] kind of okay okay okay no problem so do you asides the asthma do you have any other ailments that you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no [DEL:at] [DEL:all] [DEL:i] [DEL:do] not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [DEL:vomiting] was there any any of your family members that also had the same symptoms no no no no no other just me just [DEL:me] and my son yes okay no [DEL:problem] okay [DEL:do] you i am just going to ask some questions just to rule [DEL:out] every other thing do you [DEL:do] you have headaches no doctor do you have chest pain no doctor [INS:i] [SUB:at-&gt;do] [SUB:all-&gt;not] no do you have an abdominal pain [DEL:oh] do you you have an abdominal pain do you have any change in your bowel habits i do not know how to answer that other [DEL:than] the just the the okay i think [DEL:i] think [DEL:i] think that is fine your urine your your [DEL:urine] has it has [DEL:it] changed in quantity no not at all how about the frequency of urination has it changed no no my urination is fine do you have any [DEL:do] you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and they can also come to have [INS:a] differential diagnosis of what could be the because of your symptoms and [SUB:we-&gt;i] would like to examine you right check your level of hydration check your general physical appearance [DEL:to] see whether you and access your your general health right we also like to do an abdominal examination right to [DEL:to] also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some infection which could have which could have caused the diarrhea you want to say something so what exactly is wrong what exactly is wrong what exactly [DEL:is] the because okay it is just the food i ate right [DEL:so] yeah it looks like you have had a food poisoning however [INS:we] are going [INS:to] have [INS:to] evaluate you and find [INS:out] had [SUB:a-&gt;exactly] [SUB:food-&gt;is] [SUB:poisoning-&gt;the] but however we are going to [INS:do] some very serious tests [INS:i] [INS:am] have to check your [INS:blood] [INS:count] [INS:to] make sure there [INS:is] some [INS:infection] [INS:i] [INS:do] not know [INS:to] evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to know if there is [DEL:a] there [DEL:is] some infection which could be gastroenteritis [SUB:we-&gt;you] want to do your erythrocyte [SUB:sedimentation-&gt;segmentation] rates to know if there is any sign any any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and then [DEL:we] would also want to do a stool culture microscopy and sensitivity and to look out for parasites and some bacteria that could cause you to be having diarrhea we also check your retroviral status to know if you have [INS:a] retroviral disease which could also be a because of [DEL:of] diarrhea although that comes in the chronic chronic setting however [INS:we] would also need to just rule that out do you understand okay doctor okay however we are going to start you on [DEL:on] some some fluids to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your electrolytes electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan [INS:to] rule throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would [DEL:be] could be causing the diarrhea and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get [SUB:on-&gt;out] with [SUB:it-&gt;here] you are fine yeah so that will be fine thank you so you will be attended to [SUB:all-&gt;alright] right thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may [DEL:i] help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and [SUB:i-&gt;having] have been abdominal pain two alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is [SUB:it-&gt;he] watery is he semi solid or [DEL:it] is [SUB:in-&gt;it] normal form well formed stools it is very watery very watery very watery yes okay [DEL:all] right so like how many episodes of you said you have been stolen for over four days right yes and how many episodes do you do you have per day of stooling my about six about six to seven episodes actually about around that number yes of passage of the water watery [SUB:stool-&gt;tube] yes yes yes doctor okay okay so is this [INS:is] the [SUB:stool-&gt;still] containing mucus is it mucoid no no there is no mucus no [DEL:mucus] in it was there any blood in it no blood at all there is no blood in it okay did you change did you eat [DEL:a] from a new restaurant or did you did you eat something different ermactually a few days ago [DEL:i] like just before [SUB:it-&gt;you] started i actually had [SUB:a-&gt;the] take out in a restaurant with my family which all [SUB:of-&gt;was] [SUB:us-&gt;it] ate and [SUB:one-&gt;all] of my child actually vomited but the vomiting stopped and [SUB:he-&gt;it] feels good now so it is just [DEL:me] right now with the [SUB:complaints-&gt;complaint] i have of the of the loose [SUB:stool-&gt;so] are you also vomiting yes [INS:i] [INS:i] ii vomited about two two episodes about two times yes what what what what was inside the vomit what was the con components [DEL:of] the [DEL:vomitus] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know [SUB:it-&gt;i] just i just want [INS:to] tell [SUB:vomited-&gt;you] that is [SUB:all-&gt;the] [SUB:i-&gt;line] i cannot really remember how you came out to be honest okay was there any is there any abdominal [SUB:distension-&gt;distention] [SUB:distension-&gt;distention] like a swelling swelling yeah was there swelling in your stomach no just the abdominal pain the pain is just at my the lower part of my stomach okuhm [SUB:all-&gt;alright] right [DEL:all] right thank you so you said your son also ate ate the same the same food that you bought and [DEL:he] is now vomiting how is he feeling now [SUB:he-&gt;it] feels [SUB:he-&gt;it] is okay [DEL:he] after the episode [DEL:of] [DEL:vomiting] he [DEL:he] got he got well and [SUB:he-&gt;it] is okay how is your appetite like my appetite is [SUB:is-&gt;yeah] here and there know it is not really good like so now this let [SUB:us-&gt;before] okay okay so let us talk about let us talk about your the pain you were having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it yeah i will describe it like like has a [SUB:cramp-&gt;camp] pain like the pain i feel during menstruation so that is the kind of pain like that [DEL:is] the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to any another part of your body when you start feeling it no just just the lower part of my like moving [DEL:to] the [DEL:back] just the lower part [DEL:it] does not move [DEL:to] your [DEL:back] no no not [DEL:at] [DEL:all] [DEL:it] stays [DEL:in] the same space yes yes okay okay so what what do you think makes this [SUB:pain-&gt;play] worse well maybe if i if [DEL:i] do not eat i do not know if [DEL:i] [DEL:do] not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse [SUB:per-&gt;i] [SUB:se-&gt;say] but i will say maybe if i do not eat yes okay what what what relieves the pain not nothing i do not know i do not know anything that reduce the [DEL:pain] [DEL:it] just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i would will the pain like five [INS:out] [SUB:or-&gt;of] ten five [INS:out] [INS:of] ten yes no problem [DEL:so] let us yeah take some history do you have are you hypertensive no i am not are you diabetic no i am not do you are you a known [SUB:peptic-&gt;ulcer] also patient no no are you lactose intolerant no the only the only ailment i [SUB:am-&gt;will] being treated for [INS:is] [INS:asthma] i [SUB:am-&gt;have] being treated for is asthma i [SUB:am-&gt;have] [SUB:a-&gt;nonasthmatic] known [DEL:asthmatic] and and i am on i use inhalers and how many recently how many exacerbations do you have in a year how about [DEL:in] the last one just one okay okay that [SUB:is-&gt;was] good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those [DEL:i] [DEL:do] not [DEL:at] [DEL:all] and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i [DEL:i] feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your [SUB:body-&gt;bodys] [DEL:is] dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my [DEL:i] feel sometimes my mouth is kind of dry to kind of okay okay okay no problem so do you asides the asthma do you have any other ailments that you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no [DEL:at] [DEL:all] [DEL:i] [DEL:do] not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [INS:vomit] [SUB:vomiting-&gt;symptoms] was there any any of your family members that also had the same symptoms no no no no no other just me just [DEL:me] and my son yes okay no problem okay do you i am just going to ask some questions just to rule out every other thing do you [DEL:do] you have headaches no doctor do you have chest pain [INS:i] no doctor [SUB:at-&gt;i] [SUB:all-&gt;thought] no do you have an abdominal pain [DEL:oh] do you you have an abdominal pain [DEL:do] you have any change in your bowel habits i do not know how to answer that other [DEL:than] the just the the okay i think [DEL:i] think [DEL:i] think that is fine your urine your your urine has it has [DEL:it] changed in quantity no not at all how about the frequency of urination has it changed no no my [DEL:urination] [DEL:is] fine do you have any [DEL:do] you have any bone pain no [DEL:all] right no [DEL:problem] so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and they can also come to have differential diagnosis of what could be the because of your symptoms and [SUB:we-&gt;they] would like to examine you right check your level of hydration check your general physical appearance to see whether you you and access your your general health right we also like to do an abdominal examination right to [DEL:to] also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes yes although although it seems like what you ate the restaurants you got food from there must have been where you got some [INS:so] infection which could have which could have caused the [SUB:diarrhea-&gt;diarrhoea] you want to say something yeah so what exactly is wrong what exactly is wrong what exactly is the because [INS:it] okay it is just the food [DEL:i] ate right [DEL:so] yeah [DEL:it] looks like you have had [DEL:a] [DEL:food] poisoning had [SUB:a-&gt;the] food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to know if there is [DEL:a] there [DEL:is] some infection which could be [SUB:gastroenteritis-&gt;gastritis] we want to do your erythrocyte sedimentation rates to know if there is any sign any any type [DEL:of] kind of inflammatory disorder that could cause [SUB:diarrhea-&gt;diarrhoea] like inflammatory bowel disease right and then [DEL:we] would also want to do [SUB:a-&gt;is] [SUB:stool-&gt;to] culture microscopy and sensitivity and to look out for parasites and some bacteria that could cause you to be having [SUB:diarrhea-&gt;diarrhoea] [SUB:we-&gt;and] also check your retroviral status to know if you have [SUB:retroviral-&gt;viral] disease which could also be a because of of diarrhoea [SUB:diarrhea-&gt;or] although that comes in the chronic [INS:a] chronic setting however [INS:we] would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some fluids to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your electrolytes electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan [INS:to] rule throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would [DEL:be] could be causing the [SUB:diarrhea-&gt;diarrhoea] and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine yeah so that will be fine thank you so you will [SUB:be-&gt;been] attended to [SUB:all-&gt;alright] right thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may [DEL:i] help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and [SUB:i-&gt;having] have been abdominal pain two alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the [SUB:of-&gt;tool] the [DEL:stool] is [SUB:it-&gt;he] watery is he semi solid or it is [SUB:in-&gt;a] normal form [SUB:well-&gt;wellformed] formed stools it is very watery very watery very watery yes okay all right so like how many episodes of you said you have been stolen for over four days right yes and how many episodes do you [DEL:do] you have per day of stooling my about six about six to seven episodes actually about around that number yes of passage of watery stool yes yes yes doctor okay okay so is the [SUB:stool-&gt;tool] containing mucus is it mucoid no no no there is no mucus no mucus [DEL:in] [DEL:it] was there any blood in it no blood at all there is no blood in it okay did you change did you eat [DEL:a] from a new restaurant or did you did you eat something different ermactually a few days ago i like just before [SUB:it-&gt;i] started i actually had a take [DEL:out] in a restaurant with my family which all of us ate and one of my child actually vomited but the vomiting stopped and [SUB:he-&gt;it] feels good now so it is just [DEL:me] right now with the complaints i have of the [DEL:of] the loose [SUB:stool-&gt;yes] are you also [SUB:vomiting-&gt;said] yes ii [DEL:vomited] about two two episodes about two times yes what what what what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomiters] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know [DEL:it] just i just [SUB:vomited-&gt;wanted] that [SUB:is-&gt;ask] [DEL:all] i [DEL:i] cannot really remember how you came out to be honest okay was there any is there any abdominal distension distension like a swelling swelling yeah was there swelling in your stomach no just the abdominal pain the pain is just at my the lower part of my stomach okuhm all right all right thank you so you said your son also ate ate the same the same [DEL:food] that you bought and he is now vomiting how is he feeling now he feels he is okay [DEL:he] after the episode of vomiting he [DEL:he] got [DEL:he] got well and [SUB:he-&gt;it] is okay okay how is your appetite like my appetite is [DEL:is] here and there know it is not really good like so now let us okay okay so let us talk about let us talk about your the pain you were having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it yeah i will describe it like like has a cramp pain like the pain i feel during my [SUB:menstruation-&gt;session] so that is the kind of pain like that is the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just just the lower part [DEL:of] my like moving [DEL:to] the back just the lower part [DEL:it] does not move [DEL:to] your [DEL:back] no no not [DEL:at] [DEL:all] [DEL:it] stays [DEL:in] the same space yes yes okay okay so what what do you think makes this pain worse [DEL:well] maybe if i if [DEL:i] do not eat i do not know if [SUB:i-&gt;is] [SUB:do-&gt;easier] not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it [SUB:worse-&gt;well] per se but i will say maybe if i do not eat yes okay what what what relieves the pain nothing i do not know i do not know anything that reduce the [DEL:pain] [DEL:it] just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will give the pain like five or ten five over ten yes no problem so let us yeah take some history [DEL:do] you have are you hypertensive no i am not are you diabetic no i am not do you are you a known [SUB:peptic-&gt;ulcer] also patient no no are you lactose [INS:in] intolerant no the only the only ailment i am being treated for i [SUB:am-&gt;have] being treated for is asthma [SUB:i-&gt;my] [SUB:am-&gt;nonasmatic] [DEL:a] known [DEL:asthmatic] and and i am [SUB:on-&gt;only] i use [SUB:inhalers-&gt;als] and how many how many exacerbations do you have in a year about [DEL:in] the last one just one okay okay that is good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those i do not have [INS:it] at all and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i [DEL:i] feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my i feel sometimes my mouth is kind of dry to kind [SUB:of-&gt;up] okay okay okay no problem so do you have asides the asthma do you have any other ailments that you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no at all i do not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the vomiting was there any any of your family members that also had the same symptoms no no no no no that other just me and just me and my son yes okay no [DEL:problem] okay do you i am just going to ask some questions just to rule [DEL:out] every other thing do you [DEL:do] you have headaches no not [INS:at] doctor do you have chest pain no doctor at all no do you have an abdominal pain [DEL:oh] do you you have an abdominal pain do you have any change in your [SUB:bowel-&gt;dowel] habits yeah i do not know how to answer that other than the just the the okay i think [DEL:i] think [DEL:i] think that is fine your urine your your [DEL:urine] has it has [DEL:it] changed in quantity no not at all how about the frequency of urination has it changed no no my [SUB:urination-&gt;initial] [DEL:is] fine [DEL:do] you have any [DEL:do] you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and then they can also come to have differential diagnosis of what could be the because of your symptoms and then we would like to examine you right check your level of [SUB:hydration-&gt;vibration] check your general physical appearance to see whether you and access your your general health right we also like to do an abdominal examination right [SUB:to-&gt;so] [DEL:to] also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some infection which could have which could have caused the [DEL:diarrhea] you want to say something so what exactly is wrong what exactly is wrong what exactly is the because okay it is just the food i ate right [DEL:so] yeah it looks like you have had a food poisoning had [SUB:a-&gt;the] food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series [DEL:of] tests i am going to check your blood count to know if there is [DEL:a] there [DEL:is] some infection which could be [INS:a] gastroenteritis we want to do your erythrocyte sedimentation rates to know if there is any sign any any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and then we would also want to do a stool culture microscopy and sensitivity and to look out for parasites and some [SUB:bacteria-&gt;bacterias] that could cause you to be having diarrhea we also check your retroviral status to know if you have [INS:a] retroviral disease which could also be a because of [DEL:of] diarrhea although that comes in the chronic chronic setting however [INS:i] would also need to just rule that out do you understand okay doctor okay however we are going to start you on [DEL:on] some some [DEL:fluids] to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your [SUB:electrolytes-&gt;electrolyte] electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan [INS:to] rule throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would [DEL:be] could be causing the diarrhea and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine yeah [DEL:so] that will [DEL:be] fine thank you so you will be attended to all right thank you very much doctor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add audio playback, click-to-seek, and manual span annotation to webapp
- NER: rework all_dataset_ner.ipynb and add ner_union_experiment.ipynb (union NER); refresh NER-tagged result spreadsheets
- Audio: prepare_annotations.py exports audio_file; regenerate whisper/phi4 JSON; add AUDIO_BASE_DIR config and safe /api/audio route; add session audio player in annotate.html
- Seek: proportional click-to-seek on error spans and any text position
- Manual spans: add start_idx/end_idx/source to Annotation model + POST handler; text-selection creates MANUAL spans with overlap rejection and rendering; fix humanNerText scope bug blocking saves
</commit_message>
<xml_diff>
--- a/annotation_tool/selected_sessions_normalized_with_ner_tagged.xlsx
+++ b/annotation_tool/selected_sessions_normalized_with_ner_tagged.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ4"/>
+  <dimension ref="A1:AW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,15 +631,45 @@
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
+          <t>norm_whisper_asr_ner</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>norm_phi4_asr_ner</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>norm_parakeet_asr_ner</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>whisper_reconstructed_medical_errors</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>phi4_reconstructed_medical_errors</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>parakeet_reconstructed_medical_errors</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
           <t>whisper_reconstructed_ref</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>phi4_reconstructed_ref</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>parakeet_reconstructed_ref</t>
         </is>
@@ -932,17 +962,47 @@
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>male or a female [INS:i] [INS:am] a male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did it started gradually or it was gradual in onset okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with [SUB:a-&gt;the] burning sensation it is it [INS:is] not associated with pain or a burning sensation okay so it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to urinate yes i feel [INS:the] urgency to you ring [SUB:urinate-&gt;it] and then are you able to pass out this urine when you feel this urgency to you [INS:in] [SUB:urinate-&gt;it] i am unable to pass out [SUB:urine-&gt;here] okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting [SUB:the-&gt;into] toilet especially [DEL:in] the night okay nocturia so you always visit the toilet in the night yes at morning at night at night like how many times [SUB:do-&gt;you] you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] alot and my urine [SUB:dripples-&gt;dribbles] okay it [SUB:dripples-&gt;dribbles] yeah after [SUB:urination-&gt;i] may [DEL:i] know if there is blood in the urine there is no blood in this urine there is no fever i do not have ist have fever is there pause there is no pus pause [SUB:oo-&gt;so] do you have lower abdominal pain i do not have abdominal pain okay thank you very much is there a history of trauma or any recent [SUB:catherization-&gt;catarization] or urethra instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catarization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told [SUB:at-&gt;that] the hospital that i was diagnosed there you were diagnosed in [SUB:a-&gt;the] hospital ten years ago yes yes and you have been on medications yes it has been controlled by medications okay thank you very much how about being diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some [SUB:urinal-&gt;urinary] problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational drugs substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [INS:i] [INS:am] [INS:on] [SUB:amlodepine-&gt;lodipine] okay you are on [SUB:amlodepine-&gt;lodipine] is there any other drug you are on i am not on any other [INS:drug] they give me just that one okay thank you very much do you have any other allergies [DEL:do] you have are you allergic to any drug or medication [INS:no] i am not okay thank you very much</t>
+          <t>male or a female i am a male how old are you i am sixtyfive years old i hope you do not mind i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having [PROBLEM: difficulty in urinating] you have been having [PROBLEM: difficulty in urinating] for how long has this been that is nothing for two weeks you have been having [PROBLEM: difficulty urinating] for two weeks yes did this started gradually or it was gradual in onset it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it got bad recently it was not constant before but now it is constant okay thank you very much is this [PROBLEM: pain] while [BODY_FUNCTION: urinating] associated with the [PROBLEM: burning sensation] it is it is not associated with [PROBLEM: pain] or a [PROBLEM: burning sensation] okay so it is not associated with any [PROBLEM: pain] or a [PROBLEM: burning sensation] yes it is not do you feel the [PROBLEM: urgency to urinate] yes i feel the [PROBLEM: urgency] to you ring it and then are you able to pass out this urine when you feel this urgency to you in it i am unable to pass out here okay do you feel frequent [BODY_FUNCTION: urination] the urge to always go to the toilet yes i am always just into it especially the night okay [PROBLEM: nocturia] so you always use the toilet in the night yes at morning at night at night like how many times you you need in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [PROBLEM: strain] to urinate yes i [PROBLEM: strain] a lot and my [LABORATORY_DATA: urine] dribbles okay it dribbles yes after i might know if there is [PROBLEM: blood in the urine] there is no [PROBLEM: blood in this urine] there is no [PROBLEM: fever] i do not have ist have [PROBLEM: fever] is there [PROBLEM: pus] there is no [PROBLEM: pus] okay so do you have lower [PROBLEM: abdominal pain] i do not have [PROBLEM: abdominal pain] oh thank you very much is there a history of [PROBLEM: trauma] or any recent [PROCEDURE: catarization] or [PROCEDURE: urethra instrumentation] no there is none there is no history of [PROBLEM: trauma] or [PROBLEM: catarization] i do not have any history oh thank you very much are you a known [PROBLEM: hypertensive] patient are you [PROBLEM: hypertensive] yes i have been [PROBLEM: hypertensive] for ten years now okay you have been [PROBLEM: hypertensive] for ten years how do you know you are [PROBLEM: hypertensive] i was told that the hospital  i was diagnosed there you were diagnosed in the hospital ten years ago yes yes and you have been on [MEDICINE: medications] yes that is been controlled by [MEDICINE: medications] okay thank you very much how about being [PROBLEM: diabetic] are you [PROBLEM: diabetic] no i am not [PROBLEM: diabetic] you are not [PROBLEM: diabetic] okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad had similar condition when he was old when he was old what exactly was the [PROBLEM: problem] did he also feel [PROBLEM: pain] while trying to urinate he had some [PROBLEM: urinary problem] i cannot tell exactly i was young at that time okay thank you very much are you a [SUBSTANCE_ABUSE: smoker] i do not [SUBSTANCE_ABUSE: smoke] do you take [SUBSTANCE_ABUSE: alcohol] yeah i consume [SUBSTANCE_ABUSE: alcohol] occasionally do you take any [SUBSTANCE_ABUSE: recreational drugs] [SUBSTANCE_ABUSE: substance abuse] no thank you very much are you on your [MEDICINE: hypertensive agent] yes i am on some [MEDICINE: drugs] they gave me to control the [PROBLEM: hypertension] can you tell me the name of the drug you are on i am on [MEDICINE: lodipine] okay you are on [MEDICINE: lodipine] is there any other drug you are on i am not on any other drug they gave me just that one oh thank you very much do you have any allergies are you allergic to any [MEDICINE: drug] or [MEDICINE: medication] no i am not okay thank you very much</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>male or a female [INS:i] [INS:am] a male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr [INS:i] emeka i do not mind okay thank you very much so what brought you to the clinic today i have [SUB:am-&gt;been] having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did [INS:this] it started gradually or it was gradual in onset okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with [SUB:a-&gt;the] burning sensation it is not associated with pain or [DEL:a] burning sensation okay it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to [SUB:urinate-&gt;you] yes [DEL:i] feel [DEL:urgency] [DEL:to] [DEL:urinate] and then are you able to pass out this urine when you feel this urgency to you [SUB:urinate-&gt;know] i am unable to pass out [DEL:urine] okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting the toilet especially in the night okay nocturia so you always visit the toilet in the night yes at morning at night at night like how many times [SUB:do-&gt;you] you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than you used to [INS:be] before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] alot and my urine [SUB:dripples-&gt;bubbles] okay it [SUB:dripples-&gt;bubbles] yeah after urination may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have [INS:a] fever is there pause there is no pus so pause [SUB:oo-&gt;so] do you have lower abdominal pain i do not have any abdominal pain okay thank you very much is there a history of trauma or any recent [SUB:catherization-&gt;catheterization] or [SUB:urethra-&gt;ureteral] instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you [DEL:hypertensive] yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told [DEL:at] [DEL:the] hospital that i was diagnosed [INS:in] [INS:the] there you were diagnosed in [SUB:a-&gt;the] hospital ten years ago yes and you have been on medications yes it has been controlled by medications okay thank you very much how about being diabetic are you diabetic no i am not diabetic you are not [DEL:diabetic] okay is there [DEL:a] family history of similar condition [DEL:is] there anyone in your family that has similar condition yeah i can remember my dad have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some [SUB:urinal-&gt;urinary] problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally [DEL:do] you take any [DEL:recreational] [DEL:drugs] [DEL:substance] [DEL:abuse] [DEL:no] thank you very much are you on your hypertensive agents yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [SUB:amlodepine-&gt;i] okay you are [SUB:on-&gt;the] [SUB:amlodepine-&gt;pin] is there any other drug you are on i am not on any other [INS:drug] they give me just that one okay thank you very much do you have any other [SUB:allergies-&gt;justifications] [DEL:do] you have are you allergic to any drug or medication [INS:no] i am not okay thank you very much</t>
+          <t>male or a female i am a male how old are you i am sixtyfive years old i hope you do not mind i address you as mr i maker i do not mind okay thank you very much so what brought you to the clinic today i have been having [PROBLEM: difficulty in urinating] you have been having [PROBLEM: difficulty in urinating] for how long has this been that is lasted for two weeks you have been having [PROBLEM: difficulty urinating] for two weeks yes did this start as gradually or it was gradual in onset it was gradual in onset has it been constant has he always been there or he just comes and goes or he feels this within a particular period of the day i think he got bad of recent it was not constant before but now it is constant okay thank you very much is this [PROBLEM: pain] while [BODY_FUNCTION: urinating] associated with the [PROBLEM: burning sensation] it is not associated with [PROBLEM: pain] [PROBLEM: burning sensation] it is not associated with any [PROBLEM: pain] or a [PROBLEM: burning sensation] yes it is not do you feel the urgency to you know and then are you able to pass out this urine when you feel this urgency to you know i am unable to pass out okay do you feel frequent [BODY_FUNCTION: urination] the urge to always go to the toilet yes i am always using the toilet especially in the night okay [PROBLEM: nocturia] so you always use the toilet in the night yes at morning at night at night like how many times you you need in the night it is very frequent i cannot tell more than it used to be for yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [PROBLEM: strain to urinate] yes i [PROBLEM: strain] a lot and my [BODY_MEASUREMENT: urine bubbles] okay it bubbles yes after [BODY_FUNCTION: urination]  i know if there is [PROBLEM: blood in the urine] there is no blood in this urine there is no [PROBLEM: fever] i do not have a [PROBLEM: fever] is there pus there is no [PROBLEM: pus] so okay so do you have lower [PROBLEM: abdominal pain] i do not have any [PROBLEM: abdominal pain] oh thank you very much is there a history of [PROBLEM: trauma] or any recent [PROCEDURE: catheterization] or [PROCEDURE: ureteral instrumentation] no there is none there is no history of [PROBLEM: trauma] or [PROCEDURE: catheterization] i do not have any history of that oh thank you very much are you a known [PROBLEM: hypertensive] yes i have been [PROBLEM: hypertensive] for ten years now okay you have been [PROBLEM: hypertensive] for ten years how do you know you are [PROBLEM: hypertensive] i was told that i was diagnosed in the hospital i was diagnosed in the hospital ten years ago yes and you have been on [MEDICINE: medications] yes that has been controlled by [MEDICINE: medications] okay thank you very much how about being [PROBLEM: diabetic] are you [PROBLEM: diabetic] no i am not [PROBLEM: diabetic] is there anyone in your family that has similar condition yeah i can remember my dad had similar condition when he was old when he was old what exactly was the problem did he also feel [PROBLEM: pain] while trying to urinate he had some [PROBLEM: urinary problem] i cannot tell exactly i was young at that time okay thank you very much are you a [SUBSTANCE_ABUSE: smoker] i do not [SUBSTANCE_ABUSE: smoke] do you take [SUBSTANCE_ABUSE: alcohol] yeah i consume [SUBSTANCE_ABUSE: alcohol] occasionally are you on your [MEDICINE: hypertensive agents] yes i am on some [MEDICINE: drugs] they gave me to control the [PROBLEM: hypertension] can you tell me the name of the drug you are on i am on load the pin is there any other drug you are on i am not on any other drug they gave me just that one thank you very much do you have any other justifications are you allergic to any [MEDICINE: drug] or [MEDICINE: medication] no i am not okay thank you very much</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>male or a female [DEL:a] male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did it started gradually or it was gradual [SUB:in-&gt;nonsense] onset okay it was gradual in [INS:on] onset has it been constant has it always been there or it just comes and goes or you feel this within [SUB:a-&gt;the] particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with a burning sensation it is not associated with pain or a burning sensation okay so it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to urinate yes i feel [INS:the] urgency to urinate and then are you able to pass out this urine when you feel this urgency to urinate i am unable to pass out urine okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting the toilet especially in the night okay nocturia so you always visit the toilet in the night yes at morning at night at night like how many times do you urinate in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] alot and my urine [SUB:dripples-&gt;dribbles] okay it [SUB:dripples-&gt;dribbles] yeah after urination may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have fever is there pause there is no pulse pause [SUB:oo-&gt;so] do you have lower abdominal pain i do not have abdominal pain okay thank you very much is there a history of trauma or any recent [SUB:catherization-&gt;caterization] or urethra instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told at the hospital that i was diagnosed there you were diagnosed in a hospital ten years ago yes and you have been on medications yes it has been controlled by medications okay thank you very much how about being diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad had have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some urinal problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational [SUB:drugs-&gt;drug] substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [INS:i] [INS:am] not [SUB:amlodepine-&gt;pain] okay you are on and you know [INS:the] [SUB:amlodepine-&gt;pain] is there any other drug you are on i am not on any other [INS:drug] they give me just that one okay thank you very much do you have any other allergies do you have are you allergic to any drug or medication [INS:no] i am not okay thank you very much madam</t>
+          <t>male or a female male how old are you i am sixtyfive years old i hope you do not mind i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having [PROBLEM: difficulty in urinating] you have been having [PROBLEM: difficulty in urinating] for how long has this been it has lasted for two weeks you have been having [PROBLEM: difficulty urinating] for two weeks yes did this start gradually or it was gradual nonsense okay it was gradual in on set has it been constant has it always been there or it just comes and goes or you feel this within the particular period of the day i think it got bad of recent it was not constant before but now it is constant okay thank you very much is this [PROBLEM: pain] while [BODY_FUNCTION: urinating] associated with a [PROBLEM: burning sensation] it is not associated with [PROBLEM: pain] or a [PROBLEM: burning sensation] okay so it is not associated with any [PROBLEM: pain] or a [PROBLEM: burning sensation] yes it is not do you feel the [PROBLEM: urgency to urinate] yes i feel the [PROBLEM: urgency to urinate] and then are you able to pass out this urine when you feel this urgency to urinate i am unable to [PROBLEM: pass out urine] okay do you feel frequent [BODY_FUNCTION: urination] the urge to always go to the toilet yes i am always using the toilet especially in the night okay [PROBLEM: nocturia] so you always use the toilet in the night yes at morning at night at night like how many times do you [BODY_FUNCTION: urinate] in the night it is very frequent i cannot tell more than it used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [PROBLEM: strain] to urinate yes i [PROBLEM: strain] a lot and my [LABORATORY_DATA: urine] dribbles okay it dribbles yes after urination may i know if there is [PROBLEM: blood in the urine] there is no [PROBLEM: blood in this urine] there is no [PROBLEM: fever] i do not have [PROBLEM: fever] is there [BODY_MEASUREMENT: pulse] there is no [BODY_MEASUREMENT: pulse] okay so do you have lower [PROBLEM: abdominal pain] i do not have [PROBLEM: abdominal pain] oh thank you very much is there a history of [PROBLEM: trauma] or any recent caterization or [PROCEDURE: urethra instrumentation] no there is none there is no history of [PROBLEM: trauma] or [PROCEDURE: catheterization] i do not have any history of that oh thank you very much are you a known [PROBLEM: hypertensive] patient are you [PROBLEM: hypertensive] yes i have been [PROBLEM: hypertensive] for ten years now okay you have been [PROBLEM: hypertensive] for ten years how do you know you are [PROBLEM: hypertensive] i was told at the hospital i was diagnosed there you were diagnosed in a hospital ten years ago yes and you have been on [MEDICINE: medications] yes that is been controlled by [MEDICINE: medications] okay thank you very much how about being [PROBLEM: diabetic] are you [PROBLEM: diabetic] no i am not [PROBLEM: diabetic] you are not [PROBLEM: diabetic] okay is there a family history of similar conditions is there anyone in your family that has similar [PROBLEM: conditions] yeah i can remember my dad had a similar condition when he was old when he was old what exactly was the [PROBLEM: problem] did he also feel [PROBLEM: pain] while trying to urinate he had some [PROBLEM: urinal problem] i cannot tell exactly i was young at that time okay thank you very much are you a [SUBSTANCE_ABUSE: smoker] i do not [SUBSTANCE_ABUSE: smoke] do you take [SUBSTANCE_ABUSE: alcohol] yeah i consume [SUBSTANCE_ABUSE: alcohol] occasionally do you take any [SUBSTANCE_ABUSE: recreational drug substance abuse] no thank you very much are you on your [MEDICINE: hypertensive agent] yes i am on some [MEDICINE: drugs] they gave me to control the [PROBLEM: hypertension] can you tell me the name of the drug you are on i am not [PROBLEM: pain] okay you are on and you know the [PROBLEM: pain] is there any other drug you are on i am not on any other drug they gave me just that one oh thank you very much do you have any [PROBLEM: allergies] do you have are you allergic to any [MEDICINE: drug] or [MEDICINE: medication] no i am not okay thank you very much madam</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>male or a female [INS:i] [INS:am] a male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating [DEL:okay] you have been having difficulty in urinating for how long has this been [SUB:it-&gt;that] [SUB:has-&gt;is] [SUB:started-&gt;nothing] for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did [SUB:it-&gt;this] started gradually or it was gradual in onset [DEL:okay] it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it [SUB:goes-&gt;got] bad [DEL:of] [SUB:recent-&gt;recently] it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with [SUB:a-&gt;the] burning sensation [INS:it] [INS:is] [INS:it] is not associated with pain or a burning sensation okay [INS:so] it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to urinate yes i feel [INS:the] urgency to [INS:you] [INS:ring] [SUB:urinate-&gt;it] and then are you able to pass out this urine when you feel this urgency to [INS:you] [INS:in] [SUB:urinate-&gt;it] i am unable to pass out [SUB:urine-&gt;here] okay do you feel frequent urination the urge to always go to the toilet yes i am always [SUB:visiting-&gt;just] [SUB:the-&gt;into] [SUB:toilet-&gt;it] especially [DEL:in] the night okay nocturia [INS:so] you always [SUB:visit-&gt;use] the toilet in the night yes at morning at night at night like how many times [SUB:do-&gt;you] you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] [SUB:alot-&gt;lot] and my urine [SUB:dripples-&gt;dribbles] okay it [SUB:dripples-&gt;dribbles] [SUB:yeah-&gt;yes] after [DEL:urination] [SUB:may-&gt;i] [SUB:i-&gt;might] know if there is blood in the urine there is no blood in this urine there is no fever i do not [INS:have] [INS:ist] have fever is there [SUB:pause-&gt;pus] there is no [INS:pus] [SUB:pause-&gt;okay] [SUB:oo-&gt;so] do you have lower abdominal pain i do not have abdominal pain [SUB:okay-&gt;oh] thank you very much is there a history of trauma or [INS:any] recent [SUB:catherization-&gt;catarization] or urethra instrumentation no there is [SUB:not-&gt;none] there is [SUB:not-&gt;no] history of trauma or [SUB:catherization-&gt;catarization] i do not have any history [DEL:of] [DEL:that] [SUB:okay-&gt;oh] thank you very much are you a [SUB:main-&gt;known] hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know [DEL:that] you are hypertensive i was told [SUB:at-&gt;that] the hospital [DEL:that] i was diagnosed there you were diagnosed in [SUB:a-&gt;the] hospital ten years ago [INS:yes] yes and you have been on medications yes [SUB:it-&gt;that] [SUB:has-&gt;is] been controlled by medications okay thank you very much how about [INS:being] diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad [SUB:have-&gt;had] similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he [SUB:has-&gt;had] some [SUB:urinal-&gt;urinary] problem i [SUB:can-&gt;cannot] tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational drugs substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they [SUB:give-&gt;gave] me to control the hypertension can you tell me the name of the drug you are [INS:on] [INS:i] [INS:am] on [SUB:amlodepine-&gt;lodipine] okay you are on [SUB:amlodepine-&gt;lodipine] is there any [INS:other] drug you are on i am not on any other [INS:drug] they [SUB:give-&gt;gave] me just that one [SUB:okay-&gt;oh] thank you very much do you have any [DEL:other] allergies [DEL:do] [DEL:you] [DEL:have] are you allergic to any drug or medication [INS:no] i am not okay thank you very much</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>male or a female [INS:i] [INS:am] a male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr [INS:i] [SUB:emeka-&gt;maker] i do not mind okay thank you very much so what brought you to the clinic today i [INS:have] [SUB:am-&gt;been] having difficulty in urinating [DEL:okay] you have been having difficulty in urinating for how long has this been [SUB:it-&gt;that] [SUB:has-&gt;is] [SUB:started-&gt;lasted] for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did [INS:this] [SUB:it-&gt;start] [SUB:started-&gt;as] gradually or it was gradual in onset [DEL:okay] it was gradual in onset has it been constant has [SUB:it-&gt;he] always been there or [SUB:it-&gt;he] just comes and goes or [SUB:you-&gt;he] [SUB:feel-&gt;feels] this within a particular period of the day i think [SUB:it-&gt;he] [SUB:goes-&gt;got] bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with [SUB:a-&gt;the] burning sensation [INS:it] is not associated with pain [DEL:or] [DEL:a] burning sensation [DEL:okay] it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to [DEL:urinate] [DEL:yes] [DEL:i] [DEL:feel] [DEL:urgency] [SUB:to-&gt;you] [SUB:urinate-&gt;know] and then are you able to pass out this urine when you feel this urgency to [INS:you] [SUB:urinate-&gt;know] i am unable to pass out [DEL:urine] okay do you feel frequent urination the urge to always go to the toilet yes i am always [SUB:visiting-&gt;using] the toilet especially in the night okay nocturia [INS:so] you always [SUB:visit-&gt;use] the toilet in the night yes at morning at night at night like how many times [SUB:do-&gt;you] you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than [SUB:you-&gt;it] used to [INS:be] [SUB:before-&gt;for] yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] [SUB:alot-&gt;lot] and my urine [SUB:dripples-&gt;bubbles] okay it [SUB:dripples-&gt;bubbles] [SUB:yeah-&gt;yes] after urination [DEL:may] i know if there is blood in the urine there is no blood in this urine there is no fever i do not have [INS:a] fever is there [SUB:pause-&gt;pus] there is no [INS:pus] [INS:so] [SUB:pause-&gt;okay] [SUB:oo-&gt;so] do you have lower abdominal pain i do not have [INS:any] abdominal pain [SUB:okay-&gt;oh] thank you very much is there a history of trauma or [INS:any] recent [SUB:catherization-&gt;catheterization] or [SUB:urethra-&gt;ureteral] instrumentation no there is [SUB:not-&gt;none] there is [SUB:not-&gt;no] history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that [SUB:okay-&gt;oh] thank you very much are you a [DEL:main] [DEL:hypertensive] [DEL:patient] [DEL:are] [SUB:you-&gt;known] hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know [DEL:that] you are hypertensive i was told [DEL:at] [DEL:the] [DEL:hospital] that i was diagnosed [INS:in] [INS:the] [SUB:there-&gt;hospital] [SUB:you-&gt;i] [SUB:were-&gt;was] diagnosed in [SUB:a-&gt;the] hospital ten years ago yes and you have been on medications yes [SUB:it-&gt;that] has been controlled by medications okay thank you very much how about [INS:being] diabetic are you diabetic no i am not diabetic [DEL:you] [DEL:are] [DEL:not] [DEL:diabetic] [DEL:okay] [DEL:is] [DEL:there] [DEL:a] [DEL:family] [DEL:history] [DEL:of] [DEL:similar] [DEL:condition] is there anyone in your family that has similar condition yeah i can remember my dad [SUB:have-&gt;had] similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he [SUB:has-&gt;had] some [SUB:urinal-&gt;urinary] problem i [SUB:can-&gt;cannot] tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally [DEL:do] [DEL:you] [DEL:take] [DEL:any] [DEL:recreational] [DEL:drugs] [DEL:substance] [DEL:abuse] [DEL:no] [DEL:thank] [DEL:you] [DEL:very] [DEL:much] are you on your hypertensive agents yes i am on some drugs they [SUB:give-&gt;gave] me to control the hypertension can you tell me the name of the drug you are on [SUB:amlodepine-&gt;i] [SUB:okay-&gt;am] [SUB:you-&gt;on] [SUB:are-&gt;load] [SUB:on-&gt;the] [SUB:amlodepine-&gt;pin] is there any [INS:other] drug you are on i am not on any other [INS:drug] they [SUB:give-&gt;gave] me just that one [DEL:okay] thank you very much do you have any other [DEL:allergies] [DEL:do] [DEL:you] [SUB:have-&gt;justifications] are you allergic to any drug or medication [INS:no] i am not okay thank you very much</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>male or a female [DEL:a] male how old are you i am sixtyfive years old [INS:i] hope you do not mind [DEL:if] i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating [DEL:okay] you have been having difficulty in urinating for how long has this been it has [SUB:started-&gt;lasted] for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did [SUB:it-&gt;this] [SUB:started-&gt;start] gradually or it was gradual [DEL:in] [SUB:onset-&gt;nonsense] okay it was gradual in [INS:on] [SUB:onset-&gt;set] has it been constant has it always been there or it just comes and goes or you feel this within [SUB:a-&gt;the] particular period of the day i think it [SUB:goes-&gt;got] bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with a burning sensation [INS:it] is not associated with pain or a burning sensation okay [INS:so] it is not associated with any pain or a burning sensation yes it is not do you feel [INS:the] urgency to urinate yes i feel [INS:the] urgency to urinate and then are you able to pass out this urine when you feel this urgency to urinate i am unable to pass out urine okay do you feel frequent urination the urge to always go to the toilet yes i am always [SUB:visiting-&gt;using] the toilet especially in the night okay nocturia [INS:so] you always [SUB:visit-&gt;use] the toilet in the night yes at morning at night at night like how many times do you urinate in the night it is very frequent i cannot tell more than [SUB:you-&gt;it] used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain [INS:a] [SUB:alot-&gt;lot] and my urine [SUB:dripples-&gt;dribbles] okay it [SUB:dripples-&gt;dribbles] [SUB:yeah-&gt;yes] after urination may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have fever is there [SUB:pause-&gt;pulse] there is no [INS:pulse] [SUB:pause-&gt;okay] [SUB:oo-&gt;so] do you have lower abdominal pain i do not have abdominal pain [SUB:okay-&gt;oh] thank you very much is there a history of trauma or [INS:any] recent [SUB:catherization-&gt;caterization] or urethra instrumentation no there is [SUB:not-&gt;none] there is [SUB:not-&gt;no] history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that [SUB:okay-&gt;oh] thank you very much are you a [SUB:main-&gt;known] hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know [DEL:that] you are hypertensive i was told at the hospital [DEL:that] i was diagnosed there you were diagnosed in a hospital ten years ago yes and you have been on medications yes [SUB:it-&gt;that] [SUB:has-&gt;is] been controlled by medications okay thank you very much how about [INS:being] diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar [SUB:condition-&gt;conditions] is there anyone in your family that has similar [SUB:condition-&gt;conditions] yeah i can remember my dad [INS:had] [SUB:have-&gt;a] similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he [SUB:has-&gt;had] some urinal problem i [SUB:can-&gt;cannot] tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational [SUB:drugs-&gt;drug] substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they [SUB:give-&gt;gave] me to control the hypertension can you tell me the name of the drug you are on [INS:i] [INS:am] [INS:not] [SUB:amlodepine-&gt;pain] okay you are on [INS:and] [INS:you] [INS:know] [INS:the] [SUB:amlodepine-&gt;pain] is there any [INS:other] drug you are on i am not on any other [INS:drug] they [SUB:give-&gt;gave] me just that one [SUB:okay-&gt;oh] thank you very much do you have any [DEL:other] allergies do you have are you allergic to any drug or medication [INS:no] i am not okay thank you very much [INS:madam]</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>male or a female a male how old are you i am sixtyfive years old hope you do not mind if i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did it started gradually or it was gradual in onset okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with a burning sensation is not associated with pain or a burning sensation okay it is not associated with any pain or a burning sensation yes it is not do you feel urgency to urinate yes i feel urgency to [SUB:urinate-&gt;it] and then are you able to pass out this urine when you feel this urgency to [SUB:urinate-&gt;it] i am unable to pass out urine okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting the toilet especially in the night okay nocturia you always visit the toilet in the night yes at morning at night at night like how many times do you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] in urinate yes i strain alot and my urine [SUB:dripples-&gt;dribbles] okay it dripples yeah after [DEL:urination] may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have fever is there [SUB:pause-&gt;pus] there is no [INS:pus] pause oo do you have lower abdominal pain i do not have abdominal pain okay thank you very much is there a history of trauma or recent [SUB:catherization-&gt;catarization] or urethra instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catarization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told at the hospital that i was diagnosed there you were diagnosed in a hospital ten years ago yes and you have been on medications yes it has been controlled by medications okay thank you very much how about diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some [SUB:urinal-&gt;urinary] problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational drugs substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [SUB:amlodepine-&gt;lodipine] okay you are on [SUB:amlodepine-&gt;lodipine] is there any drug you are on i am not on any other they give me just that one okay thank you very much do you have any other allergies do you have are you allergic to any drug or medication i am not okay thank you very much</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>male or a female a male how old are you i am sixtyfive years old hope you do not mind if i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did it started gradually or it was gradual in onset okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with a burning sensation is not associated with pain or a burning sensation okay it is not associated with any pain or a burning sensation yes it is not do you feel urgency to [DEL:urinate] yes i feel [DEL:urgency] [SUB:to-&gt;you] [SUB:urinate-&gt;know] and then are you able to pass out this urine when you feel this urgency to [SUB:urinate-&gt;know] i am unable to pass out urine okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting the toilet especially in the night okay nocturia you always visit the toilet in the night yes at morning at night at night like how many times do you [SUB:urinate-&gt;need] in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] [SUB:in-&gt;to] urinate yes i strain alot and my urine [SUB:dripples-&gt;bubbles] okay it dripples yeah after urination may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have fever is there pause there is no [INS:pus] pause oo do you have lower abdominal pain i do not have abdominal pain okay thank you very much is there a history of trauma or recent [SUB:catherization-&gt;catheterization] or [SUB:urethra-&gt;ureteral] instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that okay thank you very much are you a main [DEL:hypertensive] patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told at the hospital that i was diagnosed there you were diagnosed in a hospital ten years ago yes and you have been on medications yes it has been controlled by medications okay thank you very much how about diabetic are you diabetic no i am not diabetic you are not [DEL:diabetic] okay is there a family history of similar condition is there anyone in your family that has similar condition yeah i can remember my dad have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some [SUB:urinal-&gt;urinary] problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any [DEL:recreational] [DEL:drugs] [DEL:substance] [DEL:abuse] no thank you very much are you on your hypertensive agents yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [SUB:amlodepine-&gt;i] okay you are on [SUB:amlodepine-&gt;pin] is there any drug you are on i am not on any other they give me just that one okay thank you very much do you have any other [DEL:allergies] do you have are you allergic to any drug or medication i am not okay thank you very much</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>male or a female a male how old are you i am sixtyfive years old hope you do not mind if i address you as mr emeka i do not mind okay thank you very much so what brought you to the clinic today i am having difficulty in urinating okay you have been having difficulty in urinating for how long has this been it has started for two weeks you have been having difficulty [DEL:in] urinating for two weeks yes did it started gradually or it was gradual in onset okay it was gradual in onset has it been constant has it always been there or it just comes and goes or you feel this within a particular period of the day i think it goes bad of recent it was not constant before but now it is constant okay thank you very much is this pain while urinating associated with a burning sensation is not associated with pain or a burning sensation okay it is not associated with any pain or a burning sensation yes it is not do you feel urgency to urinate yes i feel urgency to urinate and then are you able to pass out this urine when you feel this urgency to urinate i am unable to pass out urine okay do you feel frequent urination the urge to always go to the toilet yes i am always visiting the toilet especially in the night okay nocturia you always visit the toilet in the night yes at morning at night at night like how many times do you urinate in the night it is very frequent i cannot tell more than you used to before yes it is more than the usual two times to zero times i usually use the toilet but now it is about five times do you [SUB:straint-&gt;strain] in urinate yes i strain alot and my urine [SUB:dripples-&gt;dribbles] okay it dripples yeah after urination may i know if there is blood in the urine there is no blood in this urine there is no fever i do not have fever is there [SUB:pause-&gt;pulse] there is no [INS:pulse] pause oo do you have lower abdominal pain i do not have abdominal pain okay thank you very much is there a history of trauma or recent [SUB:catherization-&gt;caterization] or urethra instrumentation no there is not there is not history of trauma or [SUB:catherization-&gt;catheterization] i do not have any history of that okay thank you very much are you a main hypertensive patient are you hypertensive yes i have been hypertensive for ten years now okay you have been hypertensive for ten years how do you know that you are hypertensive i was told at the hospital that i was diagnosed there you were diagnosed in a hospital ten years ago yes and you have been on medications yes it has been controlled by medications okay thank you very much how about diabetic are you diabetic no i am not diabetic you are not diabetic okay is there a family history of similar condition is there anyone in your family that has similar [SUB:condition-&gt;conditions] yeah i can remember my dad have similar condition when he was old when he was old what exactly was the problem did he also feel pain while trying to urinate he has some urinal problem i can tell exactly i was young at that time okay thank you very much are you a smoker i do not smoke do you take alcohol yeah i consume alcohol occasionally do you take any recreational [SUB:drugs-&gt;drug] substance abuse no thank you very much are you on your hypertensive [SUB:agents-&gt;agent] yes i am on some drugs they give me to control the hypertension can you tell me the name of the drug you are on [SUB:amlodepine-&gt;pain] okay you are on [SUB:amlodepine-&gt;pain] is there any drug you are on i am not on any other they give me just that one okay thank you very much do you have any other allergies do you have are you allergic to any drug or medication i am not okay thank you very much</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1155,12 @@
 3          3       3          i          i         =            &lt;NA&gt;
 4          4       4         am         am         =            &lt;NA&gt;
 ...      ...     ...        ...        ...       ...             ...
-2240    &lt;NA&gt;    2016          _         no       ins             532
-2241    &lt;NA&gt;    2017          _          i       ins             533
-2242    &lt;NA&gt;    2018          _         do       ins             534
-2243    &lt;NA&gt;    2019          _        not       ins             535
-2244    &lt;NA&gt;    2020          _    promise       ins             536
-[2245 rows x 6 columns]</t>
+2235    &lt;NA&gt;    2016          _         no       ins             532
+2236    &lt;NA&gt;    2017          _          i       ins             533
+2237    &lt;NA&gt;    2018          _         do       ins             534
+2238    &lt;NA&gt;    2019          _        not       ins             535
+2239    &lt;NA&gt;    2020          _    promise       ins             536
+[2240 rows x 6 columns]</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
@@ -1112,12 +1172,12 @@
 3          3       3          i          i         =            &lt;NA&gt;
 4          4       4         am         am         =            &lt;NA&gt;
 ...      ...     ...        ...        ...       ...             ...
-2742    2069    2579      start      start         =            &lt;NA&gt;
-2743    2070    2580        the        the         =            &lt;NA&gt;
-2744    2071    2581  treatment  treatment         =            &lt;NA&gt;
-2745    2072    2582      thank      thank         =            &lt;NA&gt;
-2746    2073    2583        you        you         =            &lt;NA&gt;
-[2747 rows x 6 columns]</t>
+2740    2069    2579      start      start         =            &lt;NA&gt;
+2741    2070    2580        the        the         =            &lt;NA&gt;
+2742    2071    2581  treatment  treatment         =            &lt;NA&gt;
+2743    2072    2582      thank      thank         =            &lt;NA&gt;
+2744    2073    2583        you        you         =            &lt;NA&gt;
+[2745 rows x 6 columns]</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
@@ -1129,12 +1189,12 @@
 3          3       3          i          i         =            &lt;NA&gt;
 4          4       4         am         am         =            &lt;NA&gt;
 ...      ...     ...        ...        ...       ...             ...
-2107    2069    1899      start      start         =            &lt;NA&gt;
-2108    2070    1900        the        the         =            &lt;NA&gt;
-2109    2071    1901  treatment  treatment         =            &lt;NA&gt;
-2110    2072    1902      thank      thank         =            &lt;NA&gt;
-2111    2073    1903        you        you         =            &lt;NA&gt;
-[2112 rows x 6 columns]</t>
+2105    2069    1899      start      start         =            &lt;NA&gt;
+2106    2070    1900        the        the         =            &lt;NA&gt;
+2107    2071    1901  treatment  treatment         =            &lt;NA&gt;
+2108    2072    1902      thank      thank         =            &lt;NA&gt;
+2109    2073    1903        you        you         =            &lt;NA&gt;
+[2110 rows x 6 columns]</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -1159,17 +1219,47 @@
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not too fine i am not too fine not too fine that is why i came to the hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also [INS:at] what is [INS:the] [INS:complaints] so doctor also have been [INS:coughing] for about [INS:a] week now and [INS:i] have been also you also have what so and i also have i have also been running temperature for about five days so [INS:it] is been really you have been running temperature for five days yes yes and [INS:the] [INS:cough] has been for [INS:the] [INS:cough] has been for how long for about a week now a week yes yes and [INS:the] [INS:cough] has been for how long for about [INS:a] week now [INS:a] week yes okay all right so the cough did it start suddenly or gradually the cough started suddenly just started like that so i just just woke up more morning and started coughing about a week ago yes was there was there any symptoms like catarrh or any any difficulty in swallowing before the cough started [DEL:no] none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like barking does it sound like it is comes in bouts and then you have to take a deep breath when when you say barking do you are you [DEL:do] you mean like a dog or what do you mean by barking yes yes [INS:it] sounds like a dog barking no no no no no [DEL:no] mine is not like that i did not [DEL:i] did not experience anything like that okay so is the cough productive [SUB:of-&gt;or] phlegm yes yes it is productive when i yes when [DEL:i] cough i bring out some some substance from my mouth yes so what is the colour of the substance stuff err it is about yeah it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like vomiting i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough [SUB:no-&gt;cough] no there was not nothing i was not i had nothing my my even when i was coughing my chest was not paining me nothing it was just the cough then i [DEL:i] discovered after a few days after that i just [SUB:started-&gt;tired] running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not paining me at all your [DEL:chest] was not [DEL:paining] [DEL:me] is there anybody coughing around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and [SUB:at-&gt;i] work too there is nobody coughing around me so okay so you stay [INS:in] [INS:the] alone you are not here in [SUB:an-&gt;a] overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i [SUB:started-&gt;said] to have some difficulty in breathing so like that got me really scared like i was [DEL:i] was [DEL:i] was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to come completely to see you you are finding it difficult to breathe yes yes when you sleep at night [INS:do] you sweat excessively no at all i do not [DEL:i] [DEL:do] not slept [DEL:i] [DEL:do] not sweat when [DEL:i] sleep [DEL:at] night okay so what is what relieves the breathlessness any change [DEL:in] position that relieves the breathlessness or is it is constant [DEL:no] it is not associated with any any position nothing [DEL:i] just it just comes and goes like i just feel [SUB:breathless-&gt;breathlessness] for a while then it relieves me then it comes again especially when i am especially when [DEL:i] [DEL:am] coughing okay has this worsened progressively yes yes it has gotten very bad doctor that is why i came to the hospital does it affect does [DEL:it] affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that i have [DEL:i] have not been feeling well generally in my body so that is so now this fever that you were having was [DEL:it] did it start suddenly or gradually it started [DEL:it] [DEL:started] gradually then became i became very hot and it has been like that [DEL:it] has been like that so the fever is high grade you are very hot yes yes it is high did you at attend any point yes check by yourself at home your [SUB:temperature-&gt;job] yes i did i did i have [SUB:a-&gt;about] [SUB:thermometer-&gt;thirtyeightnine] it was about was about [DEL:thirtyeightnine] [DEL:thirtyeightnine] okay and what does what do you do that relieves the fever i took some [SUB:i-&gt;prost] took some [DEL:paracetamol] it relieved a bit then but it did did not last long [SUB:i-&gt;it] just [DEL:i] [DEL:i] became hot again and it has been like that ever since so i just want to ask you some questions has this anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why [DEL:i] [DEL:am] this is [DEL:the] first time [DEL:i] [DEL:am] experiencing this kind of thing okay this is the first time are you do you have any any medical condition like are you asthmatic [INS:do] you during your blood group and genotype [INS:oh] no i am not [INS:a] doctor i am fine no i have nothing and that is why this is surprising are you [SUB:hypertensive-&gt;a] what did you say i cannot hear you properly sir are you hypertensive or diabetic none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just [SUB:i-&gt;tried] just tried to get some cough syrup but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew [DEL:i] know [DEL:i] needed to like come [DEL:to] speak to someone to a doctor so that is why i came today for you to like for [DEL:me] [DEL:to] like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that i can remember have you done any surgical procedure before no [DEL:no] okay so i am just going to ask you some other questions just to know what exactly could be related to your [DEL:to] the symptoms you are having so do you have [INS:a] headache headache [INS:it] just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;kata] no at all okay do you have any abdominal pain no no [DEL:i] do not have any [SUB:diarrhea-&gt;abdominal] [SUB:or-&gt;pain] [DEL:vomiting] no i have [INS:no] not [SUB:vomited-&gt;pain] at all [INS:no] [INS:do] you have any bone pain yes hmm thank you no [INS:i] have not [INS:vomited] [INS:at] [SUB:the-&gt;all] no [INS:do] you have any [SUB:the-&gt;bone] most [SUB:it-&gt;yes] is just it is just the shortest of breath [SUB:i-&gt;that] have been having the difficulty in breathing [SUB:i-&gt;that] have been having that is just that is just so in summary you are telling me [DEL:in] summary you are telling [DEL:me] you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have [DEL:to] examine you right i am going to have to examine you and i am going to have to listen to your chest to know [DEL:if] [DEL:to] know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and [SUB:the-&gt;a] and [DEL:the] cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your [SUB:the-&gt;deflame] [DEL:phlegm] and we are going to send it for culture sensitivity to know what bacteria is is being cultured please i just want to ask you do you smoke no no i do not doctor i am a good christian i do not smoke i do not drink you do not you [DEL:do] not drink alcohol either i do not [SUB:i-&gt;drink] [DEL:do] not [DEL:do] any of those i do not do drugs i do not [SUB:do-&gt;drink] any of that i am going to ask you some other questions do you have they their kind of personal questions can i go ahead yeah i just want to know doctor i just want to [DEL:i] just want [DEL:to] be fine i just want to know how soon you can start treating me and what i will need [DEL:to] take basically [DEL:i] just want to ask [INS:if] ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex i am married no not at all not at all i am already [INS:i] [INS:am] married so we are going to start you from the history and the examination [SUB:we-&gt;you] have done and then [SUB:we-&gt;i] are going to ask you to do some investigations however we have some different differentials like diagnosis [SUB:the-&gt;because] because the because of what is causing the cough and the fever we have some this [SUB:thing-&gt;in] [DEL:at] the back of our mind which could be the because [DEL:do] you understand [SUB:we-&gt;you] think you have a pneumonia pneumonia [DEL:a] chest infection so we are going to start you on [SUB:a-&gt;the] [SUB:broad-&gt;blood] spectrum antibiotics right and then we are going to start you [DEL:on] [DEL:the] cough [SUB:syrup-&gt;serum] right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start treatment with the antibiotics and and the cough syrup there will [DEL:be] the breathlessness is going to reduce but we your [DEL:we] would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on [DEL:on] oxygen so you are going to have you do a full blood count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscop] [SUB:culture-&gt;contrast] sensitivity you are going to have you do any [SUB:erythrocyte-&gt;ultrasound] segmentation rate and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor so doctor [DEL:do] [DEL:i] [DEL:do] you want to ask [INS:me] [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any question questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital or do i that can i can i be treated from home because i do not know we we [DEL:we] are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then [SUB:we-&gt;okay] will [SUB:start-&gt;okay] you [SUB:on-&gt;okay] [SUB:on-&gt;okay] [SUB:intravenous-&gt;okay] [SUB:intravenous-&gt;okay] that is okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay that is cool [SUB:culture-&gt;investigation] and sensitivity could take about seventytwo hours to [SUB:to-&gt;find] five days before [SUB:it-&gt;to] will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just [INS:do] [INS:the] [INS:labs] and wait for you [INS:to] [INS:start] [INS:the] [INS:treatment] thank you very much [INS:i] think that is fine [INS:i] will just yeah i will just do the labs and wait for just for you to start the treatment thank you [INS:no] [INS:i] [INS:do] not promise</t>
+          <t>good afternoon sir i am doctor [MEDICINE: shadekoff] good afternoon doctor how are you doing today sir doctor i am not too fine i am not too fine that is why i came to the hospital today what are the [PROBLEM: complaints] so doctor i have been [PROBLEM: coughing] for about a week now and i have been also at what is the [PROBLEM: complaints] so doctor i have been [PROBLEM: coughing] for about a week now and i have been also you also have what so and i also have i have also been running [BODY_MEASUREMENT: temperature] for about five days so it is been really you have been running [BODY_MEASUREMENT: temperature] for five days yes yes and the [PROBLEM: cough] has been for the [PROBLEM: cough] has been for how long for about a week now a week yes yes and the [PROBLEM: cough] has been for how long for about a week now a week yes okay all right so the [PROBLEM: cough] did it start suddenly or gradually the [PROBLEM: cough] started suddenly it started like that so i just woke up one morning and started [PROBLEM: coughing] by a week ago yes was there any [PROBLEM: symptoms] like [PROBLEM: catarrh] or any [PROBLEM: difficulty in swallowing] before the [PROBLEM: cough] started none like that i had nothing like that you had nothing like that yes so now the [PROBLEM: cough] how does it sound does it sound like [PROBLEM: barking] does it sound like it comes in [PROBLEM: barking] and then you have to take a deep [BODY_FUNCTION: breath] when you say barking do you mean like a dog or what do you mean by barking yes yes it sounds like a dog [PROBLEM: barking] no no no no no mine is not like that i did not experience anything like that okay so is the [PROBLEM: cough] productive or [PROBLEM: phlegm] yes yes it is productive when i [PROBLEM: cough] i bring out some substance from my [ANATOMICAL_STRUCTURE: mouth] yes so what is the colour of the substance stuff yeah it is about yeah it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there [PROBLEM: blood] in it at any point no there was no [PROBLEM: blood] in it there was no [PROBLEM: blood] in it there was no [PROBLEM: blood] in it at any point yes and after you [PROBLEM: cough] do you feel like [PROBLEM: vomiting] or do you [PROBLEM: vomit] no i do not i do not i do not feel like [PROBLEM: vomiting] i do not [PROBLEM: vomit] at all okay and you did not have [PROBLEM: catarrh] or [PROBLEM: difficulty swallowing] prior to onset of the [PROBLEM: cough] [PROBLEM: cough] no i was not in i was not i had nothing even when i was [PROBLEM: coughing] my [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: paining] me it was just the [PROBLEM: cough] and i discovered after a few days after that i was tired running [BODY_MEASUREMENT: temperature] too my body was very very hot it was very hot i was [PROBLEM: shivering] so you are telling me there is no there is no [PROBLEM: cough] there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] no there there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] my [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: paining] me at all is there anybody [PROBLEM: coughing] around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is [PROBLEM: coughing] too and i walk too there is nobody [PROBLEM: coughing] around me so okay so you stay in the room you are not in a crowded place yes but yes but doctor i noticed what actually tell me to come is the fact that about two days ago i noticed that the [PROBLEM: cough] became [SEVERITY: worsened] and i was i said to have some [PROBLEM: difficulty in breathing] so that got me really scared i was feeling [PROBLEM: breathless] for a moment and since then the [PROBLEM: breathlessness] has become more [SEVERITY: worsened] so that is what exactly prompted me to come quickly to see you you are finding it difficult to breathe yes when you sleep at night do you [PROBLEM: sweat] excessively no at all i do not [PROBLEM: sweat] so what relieves the [PROBLEM: breathlessness] any changing position that relieves the [PROBLEM: breathlessness] or is it constant it is not associated with any position or nothing it just comes and goes i just feel [PROBLEM: breathlessness] for a while then it releases me then it comes again especially when i am [PROBLEM: coughing] has this [SEVERITY: worsened] progressively yes yes it is gotten very bad doctor that is why i came to the hospital does it affect your daily activities yes it does doctor i have not been able to [BODY_FUNCTION: walk] for the past two days because of the [PROBLEM: cough] and the fact that i have not been feeling well generally in my body now this [PROBLEM: fever] that you were having did it start suddenly or gradually it started gradually then i became very hot and it has been like that so the [PROBLEM: fever] is [SEVERITY: high grade] you are very hot yes yes it is high did you at attend the question time check by yourself at your temporary job yes i did i did i was about [MEDICINE: thirtyeightnine] it is about [MEDICINE: thirtysevennine] [MEDICINE: thirtysevennine] okay and what do you do that released the [PROBLEM: fever] i took some prost more it relieved a bit then but it did not last long it just became hot again and it has been like that ever since so i just want to ask you some questions has this thing happened before in the past okay has it happened in the past no no no no this is the first time i am expressing this kind of thing okay this is the first time do you have any any medical condition like are you [PROBLEM: asthmatic] do you need a [LABORATORY_DATA: blood group] on genotype oh no i am not a doctor i am fine no i have not seen no i am are you a potential user i cannot hear you properly are you [PROBLEM: hypertensive] or [PROBLEM: diabetic] none none no no no i have none of them i have none of them so what have you what have you done to care for yourself so far  i just i just tried to try to get some [MEDICINE: cough syrup] but they did not probably did not seem to work properly they did not seem to work and since the [PROBLEM: difficulty in breathing] started i knew i needed to speak to someone to a doctor so that is why i came today for you to know what is wrong with me and treat myself basically have you been admitted before no not that i can remember have you done any [PROCEDURE: surgical procedure] before no okay so i am just going to ask you some other questions just to know what exactly could be related to the [PROBLEM: symptoms] you are having so do you have a [PROBLEM: headache] [PROBLEM: headache] it just comes once in a while maybe because the [PROBLEM: cough] i have not been able to sleep so kind of yeah kind of yes okay so any [PROBLEM: loss of consciousness] no no no no okay do you have kata no at all okay do you have any [PROBLEM: abdominal pain] no no do you have any [PROBLEM: abdominal pain] no i have no [PROBLEM: abdominal pain] at all no do you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] yes hmm thank you no i have not [PROBLEM: vomited] at all no do you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] yes hmm no it is just the [BODY_FUNCTION: shoulders of breath] that have been having the [PROBLEM: difficulty in breathing] that have been having so in summary you are telling me you have had [PROBLEM: cough] [PROBLEM: fever] and [PROBLEM: difficulty in breathing] yes right and your [PROBLEM: cough] is productive yes all right so i am going to have to examine you right i am going to have to examine you and i am going to have to listen to your [ANATOMICAL_STRUCTURE: chest] to know whatever is going on in your [ANATOMICAL_STRUCTURE: chest] whether it is a [ANATOMICAL_STRUCTURE: chest] [PROBLEM: infection] that is causing you to have a [PROBLEM: fever] and a [PROBLEM: cough] do you understand and then we are going to have you do some investigations like a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] a [LABORATORY_DATA: complete blood count] a [LABORATORY_DATA: full blood count] which will tell us whether there is an [PROBLEM: infection] going on depending on the parameters that are elevated or reduced do you understand we are going to do  ifide segmentation rates to know whether there is an [PROBLEM: inflammatory process] going on do you understand and then we are also going to take your sputum your [PROBLEM: deflame] and we are going to send it for [LABORATORY_DATA: culture sensitivity] to know what [LABORATORY_DATA: bacteria] is being [LABORATORY_DATA: cultured] please i just want to ask you do you [SUBSTANCE_ABUSE: smoke] no no i do not i am a good christian i do not [SUBSTANCE_ABUSE: smoke] i do not [SUBSTANCE_ABUSE: drink] you do not drink [SUBSTANCE_ABUSE: alcohol] either i do not [SUBSTANCE_ABUSE: drink] any of those i do not do [SUBSTANCE_ABUSE: drugs] i do not [SUBSTANCE_ABUSE: drink] any of that i am going to ask you some other questions do you have they are kind of personal questions can i go ahead yeah i just want to know i just want to be fine i just want to know how soon you can start treating me i just want to ask if i just want to ask if you have multiple sexual partners and then your sexual practice no no you have oral sex i am married no not at all not at all i am already i am free so we are going to start you from the history and the [PROCEDURE: examination] you have done and then i am going to ask you to do some [PROCEDURE: investigations] however we have some  different house like diagnosis because what the cost of what is causing the [PROBLEM: cough] and the [PROBLEM: fever] we have some  just in the back of our mind which could be the because you understand you think you have a [PROBLEM: pneumonia pneumonia chest infection] so we are going to [MED_STATUS: start] you on the [MEDICINE: blood spectrum antibiotics] right and then we are going to [MED_STATUS: start] your [MEDICINE: cough serum] right to treat the [PROBLEM: cough] while we wait for the results of our investigations do you understand okay and then since there is no history of [PROBLEM: asthma] by the time you start start [PROCEDURE: treatment] with the [MEDICINE: antibiotics] and the [MEDICINE: cough syrup] the [PROBLEM: breathlessness] is going to reduce but we would have checked your [BODY_MEASUREMENT: oxygen saturation] and we see that it is fine so there will be no need to place you on [MEDICINE: oxygen] so we are going to have you do a [LABORATORY_DATA: full blood count] a [LABORATORY_DATA: sputum] and [LABORATORY_DATA: microscop contrast sensitivity] you are going to have you do an [PROCEDURE: ultrasound segmentation rate] and you are going to do a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] so let us see if it is a [PROBLEM: structural problem] or a [PROBLEM: functional problem] do you understand okay doctor okay you want to ask me a question do you have any question question yes i was going to ask that i am able to keep me in your speech or do i can i can i be treated from home because i do not know we we are going to  admit you  for some time to evaluate you because because of the [PROBLEM: breathlessness] you are having right okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay okay for the investigation cultural sensitivity could take about seventytwo hours to find this for you to be ready do you understand no problem doctor thank you no problem doctor thank you very much i think that is fine i will just do the [LABORATORY_DATA: labs] and wait for you to start the [PROCEDURE: treatment] thank you very much i think that is fine i will just yeah i will just do the [LABORATORY_DATA: labs] and wait for just for you to start the [PROCEDURE: treatment] thank you no i do not promise</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to [SUB:the-&gt;you] hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also also [INS:at] have you also have what so and i also have i have also been running temperature for about five days so [INS:it] is been really yes yes and you have running [SUB:temperature-&gt;been] for five days yes yes for how long for about a week now a week yes okay [SUB:all-&gt;alright] right so the cough did it start suddenly or gradually the cough started suddenly just started like that i just just woke [DEL:up] more morning and [DEL:started] [DEL:coughing] about [DEL:a] week ago yes was there was there any symptoms like [SUB:catarrh-&gt;qatar] or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like [INS:the] barking does it sound like [INS:a] and it is comes in bouts and then you have to take a deep breath when when you say barking [DEL:do] you are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] mine is not that [SUB:i-&gt;no] did not [SUB:i-&gt;no] did not experience anything like that okay so is [SUB:the-&gt;no] [SUB:cough-&gt;no] productive [SUB:of-&gt;no] [SUB:phlegm-&gt;no] yes yes [SUB:it-&gt;no] is productive when [SUB:i-&gt;no] yes when [SUB:i-&gt;no] [SUB:cough-&gt;no] [SUB:i-&gt;no] bring [SUB:out-&gt;no] some some substance from my mouth yes so what is the colour of the substance err it is about yeah it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was [DEL:no] [DEL:blood] [DEL:in] [DEL:it] at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [INS:i] [SUB:vomiting-&gt;am] i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough no no there was not [INS:in] nothing i was not i had nothing my my even when i was coughing my chest was not [SUB:paining-&gt;burning] me nothing it was just the cough then i i discovered after a few days after that i just [DEL:started] running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not [INS:pain] [SUB:paining-&gt;in] me at all your chest was not [INS:pain] [SUB:paining-&gt;in] me is there anybody coughing around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and [SUB:at-&gt;i] work too there is nobody coughing around me so okay so you stay alone you are not here in [SUB:an-&gt;a] overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i started to have some difficulty in breathing so like that got me really scared like i was i was [DEL:i] was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to come completely to see you so you are finding it difficult to breathe yes [INS:the] [INS:cough] yes when you sleep at night [INS:do] you sweat excessively no at all i do not i do not slept i do not sweat when [SUB:i-&gt;a] sleep [SUB:at-&gt;department] night okay so what is what relieves the breathlessness any change [DEL:in] position that relieves the breathlessness or [DEL:it] is constant no it is not associated with any any position nothing [SUB:i-&gt;and] just it just comes and goes like i just feel breathless for a while then it relieves me then it comes again especially when [DEL:i] [DEL:am] especially when i am coughing okay has this worsened progressively yes yes [SUB:it-&gt;that] has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that i have [DEL:i] have not been feeling well generally [DEL:in] my [DEL:body] so that is so now this fever that you were having was it did it start suddenly or gradually [DEL:it] started it started gradually then became i became very hot and [DEL:it] has been like that it has been like that so the fever is high grade you are very hot yes yes it is [SUB:high-&gt;i] did you [SUB:at-&gt;have] any points that point yes check by yourself at home your temperature yes i did i did i have a [SUB:thermometer-&gt;stomach] [SUB:it-&gt;i] was about there was about [INS:thirty] [INS:eight] point [INS:nine] [INS:thirty] [SUB:thirtyeightnine-&gt;point] [SUB:thirtyeightnine-&gt;nine] okay and what does what do you do that relieves the fever well i took some i took some past [SUB:paracetamol-&gt;more] it relieved [SUB:a-&gt;the] bit then but it did did not last long i just i [DEL:i] became hot again and it has been like that ever since so i just want to ask you some questions has anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why [DEL:i] [DEL:am] this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic [INS:do] you during your [SUB:blood-&gt;need] [SUB:group-&gt;a] and genotype no i am not [INS:to] doctor i am fine no i have nothing and that is why this is surprising are you [INS:a] hypertensive what did you say [DEL:i] cannot hear you properly sir are you hypertensive or diabetic none none none none no [DEL:no] i have none of them i have none of them so what have you what have you done to care for yourself so far i just [SUB:i-&gt;try] just [DEL:i] just tried to get some cough syrup [INS:up] but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew i know i needed to like come to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that [SUB:i-&gt;current] can remember have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your [SUB:to-&gt;so] the symptoms you are having so do you have headache headache [INS:it] just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain no no [SUB:i-&gt;no] [SUB:do-&gt;no] not have any [SUB:diarrhea-&gt;no] [SUB:or-&gt;no] [SUB:vomiting-&gt;no] no [SUB:i-&gt;no] have not [SUB:vomited-&gt;no] [SUB:at-&gt;no] [SUB:all-&gt;no] you have any [SUB:bone-&gt;no] [SUB:pain-&gt;no] yes no [SUB:the-&gt;no] no [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [SUB:the-&gt;no] most [SUB:it-&gt;no] is just [SUB:it-&gt;of] is just the shortest of breath [DEL:i] have been having the difficulty in breathing [DEL:i] have been having that is just that is just so [DEL:in] summary you are telling me in summary you are telling me you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes [SUB:all-&gt;alright] right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know [DEL:if] to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and the and the cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count [INS:or] a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your the phlegm and we are going to send it for culture sensitivity to know what bacteria is is being cultured please i just want to ask you do you smoke no no i do not so doctor i am a good christian i do not smoke i do not drink you do not you do not drink alcohol either i do not i do not do any of those i do not do [SUB:drugs-&gt;jobs] i do not do any of that i am going to ask you some other questions do you have there their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i [INS:do] will need to take basically i just want [DEL:to] ask ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex [DEL:i] [DEL:am] married no not at all not at all [DEL:i] [DEL:am] married so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because [DEL:the] because of what is causing the cough and the fever we have some this [SUB:thing-&gt;in] [DEL:at] the back of our mind which could be the because do you understand we think you have a pneumonia pneumonia [DEL:a] chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start you on [DEL:the] cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start [SUB:treatment-&gt;treatments] with the antibiotics and and the cough syrup there will be the breathlessness business is going to reduce but we your we would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on on oxygen so you are going [SUB:to-&gt;having] have you do [DEL:a] full [SUB:blood-&gt;block] [SUB:count-&gt;out] in sputum and end [SUB:microscopy-&gt;microscopic] culture sensitivity you are going to have you doing [SUB:do-&gt;the] any [SUB:erythrocyte-&gt;site] [SUB:segmentation-&gt;sedimentation] [SUB:rate-&gt;rates] and you are going to do a chest xray so let us see if it is [DEL:a] structural problem or a functional problem do you understand okay doctor so doctor do [DEL:i] [DEL:do] you want to ask [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital or do i have that can [SUB:i-&gt;home] can i be treated from home because i do not know we [DEL:we] [DEL:we] are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then [DEL:we] will [DEL:start] you [DEL:on] [DEL:on] [DEL:intravenous] [DEL:intravenous] that is okay that is cool [SUB:culture-&gt;so] and [DEL:sensitivity] could take about seventytwo hours [DEL:to] [DEL:to] five days before [DEL:it] will [DEL:be] ready [DEL:do] you understand yeah [DEL:no] [DEL:problem] doctor thank you [DEL:no] [DEL:problem] doctor thank you very much i think that is fine i will just yeah i will just do the [SUB:labs-&gt;laps] and wait for just for you to start the treatment thank you</t>
+          <t>good afternoon sir i am doctor shadak good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to you today what was the [PROBLEM: complaints] so doctor i have been [PROBLEM: coughing] for about a week now and i have been also also at yes you also have what so and i also have  i have also been running [BODY_MEASUREMENT: temperature] for about five days so it is been really yes yes and the [PROBLEM: cough] has been for the [PROBLEM: cough] has been for how long for about a week now a week yes okay alright so  the [PROBLEM: cough] did it start suddenly or gradually the [PROBLEM: cough] started suddenly just started like that i just was there was there any [PROBLEM: symptoms] like [PROBLEM: qatar] or any  any [PROBLEM: difficulty in swallowing] before the [PROBLEM: cough] started no none like that i had nothing like that nothing like that you had nothing like that yes so now the [PROBLEM: cough] how does it sound does it sound like the barking does it sound like a and it comes in and then you have to take a deep breath when you say barking are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no substance from my [ANATOMICAL_STRUCTURE: mouth] yes so what is the colour of the substance yeah it is about yeah it is clear it is whitish it is normal it is just normal it is looking like saliva but it is very thick it is very thick was there [PROBLEM: blood] in it at any point no there was no [PROBLEM: blood] in it there was no [PROBLEM: blood] in it at any point and after you [PROBLEM: cough] do you feel like [PROBLEM: vomiting] or do you [PROBLEM: vomit] no i do not i do not i do not feel like i am i do not [PROBLEM: vomit] at all okay and you did not have [MEDICINE: catarrh] or [PROBLEM: difficulty swallowing] prior to onset of the [PROBLEM: cough] no no that was not in my i was not i had nothing my my even when i was [PROBLEM: coughing] my [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: burning] me nothing it was just the [PROBLEM: cough] and i i discovered after a few days after that i was running [BODY_MEASUREMENT: temperature] too my [ANATOMICAL_STRUCTURE: body] was very very hot it was very hot i was [PROBLEM: shivering] so you are telling me there is no there is no [PROBLEM: cough] there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] no there is there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] my [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: pain] in me at all the [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: pain] in me is there anybody [PROBLEM: coughing] around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not remember anybody around me that is [PROBLEM: coughing] too and i walk to there is nobody [PROBLEM: coughing] around me so okay so you stay alone you are not in a crowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the [PROBLEM: cough] became [SEVERITY: worsened] and i was i started to have some [PROBLEM: difficulty in breathing] so like that got me really scared i was i was feeling [PROBLEM: breathless] for a moment comes and goes and and since that since then the [PROBLEM: breathlessness] have become more [SEVERITY: worsened] so that is what exactly prompted me to come quickly to see you so you are finding it difficult to breathe yes the [PROBLEM: cough] yes when you sleep at night do you [PROBLEM: sweat] excessively no at all i do not i do not sleep i do not [PROBLEM: sweat] in a sleep department yes okay so what is what removes the [PROBLEM: breathlessness] any changing position that relieves the [PROBLEM: breathlessness] or is constant no it is not associated with any any position nothing and it just comes and goes like i just feel [PROBLEM: breathless] with a while then it releases me then it comes again especially when especially when i am [PROBLEM: coughing] okay has this worsened progressively yes yes that is gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to [BODY_FUNCTION: walk] for the past two days because of the [PROBLEM: cough] and the fact that i have not been feeling well generally so no no this [PROBLEM: fever] that you were having was it did it start suddenly or gradually started it started gradually then became i became very hot and has been like that it has been like that so the [PROBLEM: fever] is [SEVERITY: high grade] very hot yes yes it is i do you have any points that you can check by yourself at home your [BODY_MEASUREMENT: temperature] yes i did i did i have a [ANATOMICAL_STRUCTURE: stomach] i was about there was about thirty eight point nine thirty point nine okay and  what do what do you do that releases the [PROBLEM: fever] well i took some i took some past more it relieved the bit then but it did not last long i just i became hot again and it has been like that ever since so i just want to ask you some questions has this happened before in the past okay has it happened in the past no no no no this is the first time i am expressing this this is the first time i am expressing this kind of thing okay this is the first time are you do you have any medical condition like are you [PROBLEM: asthmatic] do you do you need a [BODY_MEASUREMENT: blood pressure] no i am not to doctor i am fine no i have not no are you a [PROBLEM: hypertensive] or [PROBLEM: diabetic] are you a [PROBLEM: hypertensive] or [PROBLEM: diabetic] none none none none no i have none of them i have none of them so what have you what have you done to care for yourself so far i just try to get some [MEDICINE: cough syrup] up but they did not they did not seem to work properly they did not seem to work and since  the [PROBLEM: difficulty in breathing] started i knew i knew i know i needed to like because to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that current but none have you done any [PROCEDURE: surgical procedure] before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your so the [PROBLEM: symptoms] you are having so do you have [PROBLEM: headache] [PROBLEM: headache] it just comes once in a while maybe because the [PROBLEM: cough] i have not been able to sleep really so kind of yeah kind of yes okay so any [PROBLEM: loss of consciousness] no no no no okay do you have [MEDICINE: catar] no at all okay do you have any [PROBLEM: abdominal pain] no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no no the most of the just the [PROBLEM: shouters of breath] have been happening the [PROBLEM: difficulty in breathing] have been happening so that is the summary you are telling me in summary you are telling me you had you have had [PROBLEM: cough] [PROBLEM: fever] and [PROBLEM: difficulty in breathing] yes right and your [PROBLEM: cough] is productive yes alright so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your [ANATOMICAL_STRUCTURE: chest] to know to know whatever is going on in your [ANATOMICAL_STRUCTURE: chest] there is a [ANATOMICAL_STRUCTURE: chest] [PROBLEM: infection] that is causing you to have a [PROBLEM: fever] and the and the [PROBLEM: cough] do you understand and then we are going to have you do some [PROCEDURE: investigations] like a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] a [LABORATORY_DATA: complete blood count] or a [LABORATORY_DATA: full blood count] to tell us whether there is an [PROBLEM: infection] going on depending on the parameters that are elevated or reduced do you understand we are going to do a [LABORATORY_DATA: neutrophil segmentation rate] to know whether there is an [PROBLEM: inflammatory process] [ANATOMICAL_STRUCTURE: brain] on do you understand and then we are also going to take your sputum your the [PROBLEM: phlegm] and we are going to  send it for [LABORATORY_DATA: culture sensitivity] to know what [LABORATORY_DATA: bacteria] is  is being [LABORATORY_DATA: cultured]  please i just want to ask you do you [SUBSTANCE_ABUSE: smoke] no no i do not so doctor i am a good christian i do not [SUBSTANCE_ABUSE: smoke] i do not [SUBSTANCE_ABUSE: drink] you do not you do not drink [SUBSTANCE_ABUSE: alcohol] either i do not i do not do any of those i do not do jobs i do not do any of that i am going to ask you some other questions  do you have  there are kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i do not want to ask if i do not want to ask if you have multiple sexual partners and your sexual practices no no oral sex no none at all not at all so we are going to start you from the history and the [PROCEDURE: examination] we have done and then we are going to ask you to do some [PROCEDURE: investigations] however we have some differentials like diagnoses the because of what is causing the [PROBLEM: cough] and the [PROBLEM: fever] we have some just in the back of our mind which could be the because do you understand we think you have a [PROBLEM: pneumonia pneumonia chest infection] so we are going to [MED_STATUS: start] you on a broad spectrum [MEDICINE: antibiotics] right and then we are going to start you on [MEDICINE: cough syrup] right to treat the [PROBLEM: cough] while we wait for the results of our investigations do you understand okay and then since there is no history of [PROBLEM: asthma] by the time you start [PROCEDURE: treatments] with the [MEDICINE: antibiotics] and the [MEDICINE: cough syrup] there will be the [PROBLEM: breathlessness] business is going to reduce but we your we would have checked your [BODY_MEASUREMENT: oxygen saturation] and we see that it is fine so there will be no need to place you on on [MEDICINE: oxygen] so you are against having you do full [PROBLEM: block out in   sputum] and [LABORATORY_DATA: end microscopic culture sensitivity] are going to have you doing the enteric site sedimentation rates and are going to do a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] so let us see if it is [PROBLEM: structural problem] or a [PROBLEM: functional problem] do you understand okay do you want to ask a question do you have any questions yes i was going to ask that are you going to keep me in your hospital or do i have to go home can i be treated from home because i do not know we are going to admit you for some time to evaluate you and because of the [PROBLEM: breathlessness] you are having right okay that is fine so thank you very much i think that is fine i will just yeah i will just do the laps and wait for is for you to start the [PROCEDURE: treatment] thank you</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine [INS:on] not too fine that is why i came to the hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also also have you also have what so and i also have [DEL:i] have also been running temperature for about five days so you have running [DEL:temperature] for five days yes yes and [INS:the] [INS:cough] has been for [INS:the] [INS:cough] has been for how long for about a week now a week yes okay all right so the cough did [SUB:it-&gt;this] start soddening suddenly or gradually the cough started suddenly just started like that i just just woke up more morning and started coughing about a week ago yes was there was there any symptoms like [SUB:catarrh-&gt;qatar] or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like [SUB:barking-&gt;backing] does [SUB:it-&gt;this] sound like it is comes in bouts and then you have to take a deep [DEL:breath] when when you say [SUB:barking-&gt;backing] [DEL:do] you are you do you mean like a dog or what do you mean by [SUB:barking-&gt;backing] yes yes sounds like a dog [SUB:barking-&gt;back] no no no no no [DEL:no] mine is not that [DEL:i] did not [DEL:i] did not experience anything like that okay so is the cough productive of [SUB:phlegm-&gt;flame] yes yes it is productive when [DEL:i] yes when i cough i bring out some some substance from my mouth yes so what is the colour of the substance err it is about yeah it is clear it is whitish it is not [DEL:it] is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [DEL:vomiting] i do not vomit at all okay and you did not have [SUB:catarrh-&gt;catar] or difficulty in swallowing prior to [INS:the] onset of the cough no no [INS:no] there was nothing i was not i had nothing my my even when i was coughing my chest was not [SUB:paining-&gt;painting] me nothing it was just the cough then i [DEL:i] discovered after a few days after that i just [SUB:started-&gt;hired] running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is [DEL:no] cough there is no chest pain no there is there is no chest pain my chest was not paining me at all your [SUB:chest-&gt;just] was not [SUB:paining-&gt;pain] [DEL:me] is there anybody coughing around you no there is nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have [DEL:anybody] around [DEL:me] that is coughing too and [SUB:at-&gt;i] work too there is nobody coughing around me so okay so you stay alone you are not here in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was [DEL:i] [DEL:started] to have some difficulty in breathing so like that got me really scared like i was [DEL:i] was [DEL:i] was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to come completely to see you you are finding it difficult to breathe yes yes when you sleep at night [INS:do] you sweat excessively no at all i do not [SUB:i-&gt;sleep] [DEL:do] not slept i do not sweat when [SUB:i-&gt;okay] sleep [DEL:at] night okay so what is what relieves the breathlessness any change in position that relieves the breathlessness or [SUB:it-&gt;this] is constant no it is not associated with any any position nothing i just it just comes and goes like i just feel breathless for a while then it relieves me then it comes again especially when i am especially when i am coughing okay has this worsened progressively yes yes [SUB:it-&gt;that] has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that i have [DEL:i] have not been feeling well generally in my body so that is so now this fever that you were having was it did [SUB:it-&gt;you] start suddenly [SUB:or-&gt;it] gradually it started [DEL:it] [DEL:started] gradually then became i became very hot and [DEL:it] has been like that it has been like that so the fever is [SUB:high-&gt;highgrade] [DEL:grade] you are very hot yes yes it is high did you attend [INS:a] [SUB:at-&gt;question] any point yes check by yourself at home your temperature yes i did i did i have [DEL:a] thermometer [SUB:it-&gt;i] was about was about thirtyeightnine [SUB:thirtyeightnine-&gt;thirtynine] okay and what does what do you do that relieves the fever i took some [SUB:i-&gt;past] took some [DEL:paracetamol] it relieved [SUB:a-&gt;the] bit then but it did [INS:it] did not last long [INS:it] [SUB:i-&gt;is] just [SUB:i-&gt;it] [DEL:i] became hot again and it has been like that ever since so i just want to ask you some questions has this anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why i am this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic [INS:do] you during your blood group and genotype [INS:oh] no i am not doctor i am fine no i have nothing and that is why this is surprising are you [SUB:hypertensive-&gt;hypocensing] what did you say i cannot hear you properly sir are you hypertensive or diabetic none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just [DEL:i] just [DEL:i] just tried to get some [INS:coughs] [SUB:cough-&gt;here] [SUB:syrup-&gt;up] but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew [DEL:i] knew [DEL:i] know i needed to like come [DEL:to] speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that [SUB:i-&gt;current] can remember have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the symptoms you are having so do you have headache headache yes just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain no no i do not have any [SUB:diarrhea-&gt;problem] [DEL:or] [DEL:vomiting] no i have not vomited at all you have any bone pain yes no [DEL:the] no the most it is just [DEL:it] is just the shortest of breath i have been having the difficulty in breathing [SUB:i-&gt;has] have been having that is just that is just so in summary you are telling me [SUB:in-&gt;some] summary you are telling me you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know if to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and the and [DEL:the] cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count [INS:of] a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your the [SUB:phlegm-&gt;flame] and we are going to send it for [SUB:culture-&gt;cultural] sensitivity to know what bacteria is is being [SUB:cultured-&gt;caught] please i just want to ask you do you smoke no no i do not so doctor i am a good christian i [SUB:do-&gt;just] not [DEL:smoke] i do not [SUB:drink-&gt;think] you do not you [DEL:do] not drink alcohol either i do not [SUB:i-&gt;drink] [DEL:do] not [DEL:do] any of those i do not do drugs i do not [SUB:do-&gt;drink] any of that i am going to ask you some other questions do you have there their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i will need [DEL:to] take basically [DEL:i] just want to ask [INS:if] ifi just want to ask if you have multiple sexual partners and then your sexual practices no no [INS:do] you have oral sex i am married no not at all not at all [DEL:i] [DEL:am] married so we are going to start you from the history and the examination [SUB:we-&gt;you] have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because [DEL:the] because of what is causing the cough and the fever we have some this [DEL:thing] at the back of our mind which could be the because [DEL:do] you understand we think you have a pneumonia [DEL:pneumonia] a chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start you on the cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start treatment with the antibiotics and and the cough syrup there will be the breathlessness is going to reduce but we your [DEL:we] would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on [DEL:on] oxygen so you are going to have you do a full [SUB:blood-&gt;block] count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscopic] [SUB:culture-&gt;control] sensitivity you are going to have you do any [SUB:erythrocyte-&gt;intrusive] [SUB:segmentation-&gt;sedimentation] rate and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor so doctor [DEL:do] [DEL:i] [DEL:do] you want to ask [INS:me] [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital [DEL:or] [DEL:do] [DEL:i] that can i can [DEL:i] be treated from home because i do not know we [DEL:we] [DEL:we] are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then [DEL:we] will [DEL:start] you [DEL:on] [DEL:on] [DEL:intravenous] [DEL:intravenous] that is okay that is cool [DEL:culture] and [DEL:sensitivity] could take about seventytwo hours to [DEL:to] five days before [SUB:it-&gt;you] will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just yeah i will just do the labs and wait for just for you to start the treatment thank you</t>
+          <t>good afternoon sir i am doctor [PROBLEM: shadakoff] good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine on not too fine that is why i came to the hospital today what is the [PROBLEM: complaints] so doctor i have been [PROBLEM: coughing] for about a week now and i have been also at yes you also have what so and i also have also been running [BODY_MEASUREMENT: temperature] for about five days it is been really five days yes yes and the [PROBLEM: cough] has been for the [PROBLEM: cough] has been for how long for about a week now a week yes okay all right so  the [PROBLEM: cough] did this start soddening the or gradually the [PROBLEM: cough] started suddenly just started like that i just woke up more morning and started [PROBLEM: coughing] by a week ago yes was there any [PROBLEM: symptoms] like [PROBLEM: qatar] or any [PROBLEM: difficulty in swallowing] before the [PROBLEM: cough] started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the [PROBLEM: cough] how does it sound does it sound like backing does this sound like it comes in body and then you have to take a different when you say backing are you do you mean like a dog or what do you mean by backing yes yes sounds like a dog back no no no no no mine is not that okay so is the [PROBLEM: cough] productive of flame yes yes it is productive yes when i [PROBLEM: cough] i bring out some substance from my [ANATOMICAL_STRUCTURE: mouth] yes so what is the colour of the substance yeah it is about yeah it is clear it is whitish it is just normal it is looking like saliva but it is very thick it is very thick was there [PROBLEM: blood] in it at any point no there was no [PROBLEM: blood] in it there was no [PROBLEM: blood] in it there was no [PROBLEM: blood] in it at any point okay and after you [PROBLEM: cough] do you feel like [PROBLEM: vomiting] or do you [PROBLEM: vomit] no i do not i do not i do not feel like i do not [PROBLEM: vomit] at all okay and you did not have [PROBLEM: catar or difficulty in swallowing] prior to the onset of the [PROBLEM: cough] no no no i was nothing i was not i had nothing even when i was [PROBLEM: coughing] my [ANATOMICAL_STRUCTURE: chest] was not painting me nothing it was just the [PROBLEM: cough] and i discovered after a few days after that i was hired running [BODY_MEASUREMENT: temperature] too my [ANATOMICAL_STRUCTURE: body] was very very hot it was very hot i was [PROBLEM: shivering] so you are telling me there is no [PROBLEM: cough] there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] no there is no [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] my [ANATOMICAL_STRUCTURE: chest] was not [PROBLEM: paining] me at all it just was not [PROBLEM: pain] is there anybody [PROBLEM: coughing] around you no there is nobody i stay alone right now so i have nobody around me i do not tell you people so i do not remember [PROBLEM: coughing] too and i walk too there is nobody [PROBLEM: coughing] around me okay so you stay alone you are not in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the [PROBLEM: cough] became [SEVERITY: worsened] and i said to have some [PROBLEM: difficulty in breathing] so like that got me really scared i was feeling [PROBLEM: breathless] for a moment comes and goes and since that since then the [PROBLEM: breathlessness] has become more [SEVERITY: worsened] so that is what exactly prompted me to come quickly to see you you are finding it difficult to [BODY_FUNCTION: breathe] yes yes when you sleep at night do you [PROBLEM: sweat] excessively no at all i do not sleep i do not [PROBLEM: sweat] yes okay okay so what is what relieves the [PROBLEM: breathlessness] any change in position that relieves the [PROBLEM: breathlessness] or this constant no it is not associated with any position nothing i just it just comes and goes like i just feel [PROBLEM: breathless] for a while then it relieves me then it comes again especially when i am sitting when i am [PROBLEM: coughing] has this [SEVERITY: worsened] progressively yes yes that is gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the [PROBLEM: cough] and the fact that i have not been feeling well generally in my body so that is now this [PROBLEM: fever] that you were having was it did you start sodding it gradually it started gradually then i became very hot and has been like that it has been like that so the [PROBLEM: fever] is highgrade you are very hot yes yes it is high did you attend a question to try and check by yourself at your [BODY_MEASUREMENT: temperature] yes i did i did i average thermometer i was about [MEDICINE: thirtyeightnine] [MEDICINE: thirtynine] okay and what do you do that relieves the [PROBLEM: fever] i took some past more it relieved the bit then but it did it did not last long it is just it became what again and it has been like that ever since so i just want to ask you some questions has this thing happened before in the past okay has it happened in the past no no no no this is the first time i am expressing as i am this is the first time i am experiencing this kind of thing okay it is the first time are you do you have any medical condition like are you [PROBLEM: asthmatic] do you need a blood group and genotype oh no i am not doctor i am fine no i have nothing are you [PROBLEM: hypocensing] i cannot hear you properly sir are you [PROBLEM: hypertensive] or [PROBLEM: diabetic] none none no no no [PROBLEM: i] have none of them i have none of them so what have you what have you done to care for yourself so far i just tried to get some [PROBLEM: coughs] here up but they did not seem to work properly they did not seem to work and since the [PROBLEM: difficulty in breathing] started i know i needed to speak to someone to a doctor so that is why i came today for you to like for me to know what is wrong with me and treat myself basically have you been admitted before no not that current but none have you done any [PROCEDURE: surgical procedure] before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the [PROBLEM: symptoms] you are having so do you have [PROBLEM: headache] [PROBLEM: headache] yes it comes once in a while maybe because the [PROBLEM: cough] i have not been able to sleep really so kind of yeah kind of yes okay so any [PROBLEM: loss of consciousness] no no no no okay okay do you have [MEDICINE: catar] no at all okay do you have any [PROBLEM: abdominal pain] no no i do not have a [PROBLEM: problem] no i am not [PROBLEM: vomited] at all you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] yes no no the most it is just the [PROBLEM: shortness of breath] i have been having the [PROBLEM: difficulty in breathing] has been having so in summary you are telling me some are telling me you had you have had [PROBLEM: cough] [PROBLEM: fever] and [PROBLEM: difficulty in breathing] yes right and your [PROBLEM: cough] is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your [ANATOMICAL_STRUCTURE: chest] to know if to know whatever is going on in your [ANATOMICAL_STRUCTURE: chest] whether there is a [ANATOMICAL_STRUCTURE: chest] [PROBLEM: infection] that is causing you to have a [PROBLEM: fever] and the [PROBLEM: cough] do you understand and then we are going to have you do some investigations like a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] a [LABORATORY_DATA: complete blood count] of a [LABORATORY_DATA: full blood count] to tell us whether there is an [PROBLEM: infection] going on depending on the parameters that are indicated or reduced do you understand we are going to do a neutrocyte segmentation rate to know whether there is an [PROBLEM: inflammatory process] going on do you understand and then we are also going to take your sputum the flame and we are going to send it for [PROBLEM: cultural sensitivity] to know what bacteria is being caught please i just want to ask you do you [SUBSTANCE_ABUSE: smoke] no no i do not so doctor i am a good christian i just spoke i do not think you do not drink [SUBSTANCE_ABUSE: alcohol] either i do not [SUBSTANCE_ABUSE: drink] any of those i do not do [SUBSTANCE_ABUSE: drugs] i do not [SUBSTANCE_ABUSE: drink] of that i am going to ask you some other questions do you have there are kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start with me i just want to ask if i just want to ask if you have multiple sexual partners and your sexual practices no no do you have oral sex i am married no not at all not at all so we are going to start you from the history and the [PROCEDURE: examination] you have done and then we are going to ask you to do some [PROCEDURE: investigations] however we have some differentials like diagnosis the because of what is causing the [PROBLEM: cough] and the [PROBLEM: fever] we have some at the back of our mind which could be the because you understand we think you have a [PROBLEM: pneumonia] a [ANATOMICAL_STRUCTURE: chest] [PROBLEM: infection] so we are going to [MED_STATUS: start] you on a broad spectrum [MEDICINE: antibiotics] right and then we are going to start on the [MEDICINE: cough syrup] right to treat the [PROBLEM: cough] while we wait for the results of our [PROCEDURE: investigations] do you understand okay and then since there is no history of [PROBLEM: asthma] by the time you start [PROCEDURE: treatment] with the [MEDICINE: antibiotics] and the [MEDICINE: cough syrup] there will be the [PROBLEM: breathlessness] is going to reduce but we will have checked your [BODY_MEASUREMENT: oxygen saturation] and we see that it is fine so there will be no need to place you on [MEDICINE: oxygen] so we are going to have you do a [LABORATORY_DATA: full block count] a [LABORATORY_DATA: sputum] and [LABORATORY_DATA: microscopic control sensitivity] i am going to have you do an intrusive [LABORATORY_DATA: sedimentation rate] and we are going to do a [ANATOMICAL_STRUCTURE: chest] [PROCEDURE: xray] so let us see if it is a [PROBLEM: structural problem] or a [PROBLEM: functional problem] do you understand okay doctor okay you want to ask me a question do you have any questions yes i was going to ask that are you going to keep me in your hospital can i be treated from home because i do not know we are going to admit you for some time to evaluate you and because of the [PROBLEM: breathlessness] you are having right okay okay that is fine seventytwo hours to five days for you to be ready do you understand no problem doctor no problem doctor thank you very much i think that is fine i will just yeah i will just do the [LABORATORY_DATA: labs] and wait for you to start the [PROCEDURE: treatment] thank you</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor [DEL:sadeko] [DEL:good] [SUB:afternoon-&gt;shadekoff] good afternoon doctor how are you doing today sir doctor i am not [DEL:i] [SUB:am-&gt;too] [SUB:not-&gt;fine] [SUB:too-&gt;i] [SUB:fine-&gt;am] not too fine that is why i came to the hospital today what [SUB:was-&gt;are] the complaints so doctor i have been coughing for about a week now and i have been also [INS:at] [INS:what] [INS:is] [INS:the] [INS:complaints] [INS:so] [INS:doctor] [SUB:also-&gt;i] have [INS:been] [INS:coughing] [INS:for] [INS:about] [INS:a] [INS:week] [INS:now] [INS:and] [INS:i] [INS:have] [INS:been] [INS:also] you also have what so and i also have i have also been running temperature for about five days so [INS:it] [INS:is] [INS:been] [INS:really] you have [INS:been] running temperature for five days yes yes [INS:and] [INS:the] [INS:cough] [INS:has] [INS:been] [INS:for] [INS:the] [INS:cough] [INS:has] [INS:been] [INS:for] [INS:how] [INS:long] [INS:for] [INS:about] [INS:a] [INS:week] [INS:now] [INS:a] [INS:week] [INS:yes] [INS:yes] [INS:and] [INS:the] [INS:cough] [INS:has] [INS:been] [INS:for] [INS:how] [INS:long] for about a week now a week yes okay all right so the cough did it start suddenly or gradually the cough started suddenly [SUB:just-&gt;it] started like that [SUB:i-&gt;so] [SUB:just-&gt;i] just woke up [SUB:more-&gt;one] morning and started coughing [SUB:about-&gt;by] a week ago yes [DEL:was] [DEL:there] was there any symptoms like catarrh or [DEL:any] any difficulty in swallowing before the cough started [DEL:no] none like that i had [DEL:nothing] [DEL:like] [DEL:that] nothing like that you had nothing like that yes [DEL:okay] so now the cough how does it sound does it sound like barking does it sound like it [DEL:is] comes in [SUB:bouts-&gt;barking] and then you have to take a deep breath [DEL:when] when you say barking [DEL:do] [DEL:you] [DEL:are] [DEL:you] do you mean like a dog or what do you mean by barking yes yes [INS:it] sounds like a dog barking [DEL:no] no no no no no mine is not [DEL:that] [DEL:i] [SUB:did-&gt;like] [SUB:not-&gt;that] i did not experience anything like that okay so is the cough productive [SUB:of-&gt;or] phlegm yes yes it is productive [DEL:when] [DEL:i] [DEL:yes] when i cough i bring out [DEL:some] some substance from my mouth yes so what is the colour of the substance [INS:stuff] [SUB:err-&gt;yeah] it is about [INS:yeah] it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like vomiting i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough [SUB:no-&gt;cough] no [SUB:there-&gt;i] was [INS:not] [SUB:nothing-&gt;in] i was not i had nothing [DEL:my] [DEL:my] even when i was coughing my chest was not paining me [DEL:nothing] it was just the cough [DEL:then] [SUB:i-&gt;and] i discovered after a few days after that i [SUB:just-&gt;was] [SUB:started-&gt;tired] running temperature too my body was very very hot it was very hot [DEL:that] i was shivering so you are telling me there is no there is no cough there is no chest pain no there [DEL:is] there is no chest pain my chest was not paining me at all [DEL:your] [DEL:chest] [DEL:was] [DEL:not] [DEL:paining] [DEL:me] is there anybody coughing around you no there [INS:is] nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and [SUB:at-&gt;i] [SUB:work-&gt;walk] too there is nobody coughing around me so okay so you stay [INS:in] [INS:the] [SUB:alone-&gt;room] you are not [DEL:here] in [SUB:an-&gt;a] [SUB:overcrowded-&gt;crowded] place yes but yes but doctor i noticed what actually [SUB:prompted-&gt;tell] me to come is the fact that about two days ago i noticed that the cough became worsened and i was i [SUB:started-&gt;said] to have some difficulty in breathing so [DEL:like] that got me really scared [DEL:like] i was [DEL:i] [DEL:was] [DEL:i] [DEL:was] [DEL:just] feeling breathless for a moment [DEL:comes] and [DEL:goes] [DEL:then] [DEL:and] [DEL:since] [DEL:that] since then the breathlessness has become more worsened so that is what exactly prompted me to [INS:come] [SUB:completely-&gt;quickly] to see you you are finding it difficult to breathe [DEL:yes] yes when you sleep at night [INS:do] you sweat excessively no at all [DEL:i] [DEL:do] [DEL:not] [DEL:i] [DEL:do] [DEL:not] [DEL:slept] i do not sweat [DEL:when] [DEL:i] [DEL:sleep] [DEL:at] [DEL:night] [DEL:okay] so [DEL:what] [DEL:is] what relieves the breathlessness any [DEL:change] [SUB:in-&gt;changing] position that relieves the breathlessness or [DEL:it] is [SUB:constant-&gt;it] [SUB:no-&gt;constant] it is not associated with [DEL:any] any position [DEL:nothing] [SUB:i-&gt;or] [SUB:just-&gt;nothing] it just comes and goes [DEL:like] i just feel [SUB:breathless-&gt;breathlessness] for a while then it [SUB:relieves-&gt;releases] me then it comes again [DEL:especially] [DEL:when] [DEL:i] [DEL:am] especially when i am coughing [DEL:okay] has this worsened progressively yes yes it [SUB:has-&gt;is] gotten very bad doctor that is why i came to the hospital [DEL:does] [DEL:it] [DEL:affect] does it affect your daily activities yes it does doctor i have not been able to [SUB:work-&gt;walk] for the past two days because of the cough and the fact that [DEL:i] [DEL:have] i have not been feeling well generally in my body [DEL:so] [DEL:that] [DEL:is] [DEL:so] now this fever that you were having [DEL:was] [DEL:it] did it start suddenly or gradually [DEL:it] [DEL:started] it started gradually then [DEL:became] i became very hot and [DEL:it] [DEL:has] [DEL:been] [DEL:like] [DEL:that] it has been like that so the fever is high grade you are very hot yes yes it is high did you at [INS:attend] [SUB:any-&gt;the] [SUB:point-&gt;question] [SUB:yes-&gt;time] check by yourself at [SUB:home-&gt;your] [SUB:your-&gt;temporary] [SUB:temperature-&gt;job] yes i did i did i [SUB:have-&gt;was] [SUB:a-&gt;about] [SUB:thermometer-&gt;thirtyeightnine] it [DEL:was] [DEL:about] [SUB:was-&gt;is] about [SUB:thirtyeightnine-&gt;thirtysevennine] [SUB:thirtyeightnine-&gt;thirtysevennine] okay and [DEL:what] [DEL:does] what do you do that [SUB:relieves-&gt;released] the fever i took some [DEL:i] [DEL:took] [SUB:some-&gt;prost] [SUB:paracetamol-&gt;more] it relieved a bit then but it [DEL:did] did not last long [SUB:i-&gt;it] just [DEL:i] [DEL:i] became hot again and it has been like that ever since so i just want to ask you some questions has [INS:this] [SUB:anything-&gt;thing] happened before in the past okay has it happened in the past no no no no [DEL:this] [DEL:is] [DEL:the] [DEL:first] [DEL:time] [DEL:i] [DEL:am] [DEL:experiencing] [DEL:that] [DEL:is] [DEL:why] [DEL:i] [DEL:am] this is the first time i am [SUB:experiencing-&gt;expressing] this kind of thing okay this is the first time [DEL:are] [DEL:you] do you have [INS:any] any medical condition like are you asthmatic [INS:do] [INS:you] [SUB:during-&gt;need] [SUB:your-&gt;a] blood group [SUB:and-&gt;on] genotype [INS:oh] no i am not [INS:a] doctor i am fine no i have [DEL:nothing] [DEL:and] [DEL:that] [SUB:is-&gt;not] [SUB:why-&gt;seen] [SUB:this-&gt;no] [SUB:is-&gt;i] [SUB:surprising-&gt;am] are you [DEL:hypertensive] [DEL:what] [SUB:did-&gt;a] [SUB:you-&gt;potential] [SUB:say-&gt;user] i cannot hear you properly [DEL:sir] are you hypertensive or diabetic [DEL:none] none none [SUB:none-&gt;no] no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just [SUB:i-&gt;tried] [SUB:just-&gt;to] [SUB:tried-&gt;try] to get some cough syrup but they did not [SUB:they-&gt;probably] did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew [DEL:i] [DEL:knew] [DEL:i] [DEL:know] i needed [DEL:to] [DEL:like] [DEL:come] to speak to someone to a doctor so that is why i came today for you to [DEL:like] [DEL:for] [DEL:me] [DEL:to] [DEL:like] know what is wrong with me and treat myself basically [DEL:have] [DEL:you] [DEL:been] have you been admitted before no [DEL:not] [DEL:not] not that i can remember have you done any surgical procedure before [DEL:no] no okay so i am just going to ask you some other questions just to know what exactly could be related [DEL:to] [DEL:your] to the symptoms you are having so do you have [INS:a] headache headache [INS:it] just comes once in a while maybe because the cough i have not been able to sleep [DEL:really] so kind of yeah kind of yes okay so any loss of consciousness no no no no [DEL:okay] okay do you have [SUB:catarrh-&gt;kata] no at all okay do you have any abdominal pain no no [DEL:i] do [SUB:not-&gt;you] have any [DEL:diarrhea] [SUB:or-&gt;abdominal] [SUB:vomiting-&gt;pain] no i have [INS:no] [SUB:not-&gt;abdominal] [SUB:vomited-&gt;pain] at all [INS:no] [INS:do] you have any bone pain yes [INS:hmm] [INS:thank] [INS:you] no [INS:i] [INS:have] [INS:not] [INS:vomited] [INS:at] [SUB:the-&gt;all] no [INS:do] [INS:you] [INS:have] [INS:any] [SUB:the-&gt;bone] [SUB:most-&gt;pain] [SUB:it-&gt;yes] [SUB:is-&gt;hmm] [SUB:just-&gt;no] it is just the [SUB:shortest-&gt;shoulders] of breath [SUB:i-&gt;that] have been having the difficulty in breathing [SUB:i-&gt;that] have been having [DEL:that] [DEL:is] [DEL:just] [DEL:that] [DEL:is] [DEL:just] so in summary you are telling me [DEL:in] [DEL:summary] [DEL:you] [DEL:are] [DEL:telling] [DEL:me] [DEL:you] [DEL:had] [DEL:you] you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going [DEL:to] [DEL:have] to have to examine you right i am going to have to examine you and i am going to have to listen to your chest [DEL:to] [DEL:know] [DEL:if] to know whatever is going on in your chest whether [SUB:there-&gt;it] is a chest infection that is causing you to have a fever [DEL:and] [DEL:the] and [SUB:the-&gt;a] cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do [DEL:you] [DEL:know] [SUB:electrocyte-&gt;ifide] segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your [DEL:the] [SUB:phlegm-&gt;deflame] and we are going to send it for culture sensitivity to know what bacteria [DEL:is] is being cultured please i just want to ask you do you smoke no no i do not [DEL:doctor] i am a good christian i do not smoke i do not drink [DEL:you] [DEL:do] [DEL:not] you do not drink alcohol either [DEL:i] [DEL:do] [DEL:not] i do not [SUB:do-&gt;drink] any of those i do not do drugs i do not [SUB:do-&gt;drink] any of that i am going to ask you some other questions do you have [INS:they] [SUB:their-&gt;are] kind of personal questions can i go ahead yeah i just want to know [DEL:doctor] [DEL:i] [DEL:just] [DEL:want] [DEL:to] i just want to be fine i just want to know how soon you can start treating me [DEL:and] [DEL:what] [DEL:i] [DEL:will] [DEL:need] [DEL:to] [DEL:take] [DEL:basically] i just want to ask [INS:if] [SUB:ifi-&gt;i] just want to ask if you have multiple sexual partners and then your sexual [SUB:practices-&gt;practice] no no you have oral sex i am married no not at all not at all [INS:i] [INS:am] [INS:already] i am [SUB:married-&gt;free] so we are going to start you from the history and the examination [SUB:we-&gt;you] have done and then [SUB:we-&gt;i] [SUB:are-&gt;am] going to ask you to do some investigations however we have some [INS:different] [SUB:differentials-&gt;house] like diagnosis [SUB:the-&gt;because] [SUB:because-&gt;what] the [SUB:because-&gt;cost] of what is causing the cough and the fever we have some [DEL:this] [SUB:thing-&gt;just] [SUB:at-&gt;in] the back of our mind which could be the because [DEL:do] you understand [SUB:we-&gt;you] think you have a pneumonia pneumonia [DEL:a] chest infection so we are going to start you on [SUB:a-&gt;the] [SUB:broad-&gt;blood] spectrum antibiotics right and then we are going to start [DEL:you] [DEL:on] [SUB:the-&gt;your] cough [SUB:syrup-&gt;serum] right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you [SUB:will-&gt;start] start treatment with the antibiotics [DEL:and] and the cough syrup [DEL:there] [DEL:will] [DEL:be] the breathlessness is going to reduce but [DEL:we] [DEL:your] we would have checked [DEL:your] your oxygen saturation and we [DEL:will] see that it is fine so there will be no need to place you [DEL:on] on oxygen so [SUB:you-&gt;we] are going to have you do a full blood count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscop] [SUB:culture-&gt;contrast] sensitivity you are going to have you do [SUB:any-&gt;an] [SUB:erythrocyte-&gt;ultrasound] segmentation rate and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor [DEL:so] [DEL:doctor] [DEL:do] [DEL:i] [SUB:do-&gt;okay] you want to ask [INS:me] [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any [INS:question] [SUB:questions-&gt;question] yes i was going to ask that [SUB:are-&gt;i] [SUB:you-&gt;am] [SUB:going-&gt;able] to keep me in [SUB:the-&gt;your] [SUB:hospital-&gt;speech] or do i [DEL:that] can i can i be treated from home because i do not know [DEL:we] we we are going to admit you for some time to evaluate you [SUB:and-&gt;because] because of the breathlessness you are having right [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [INS:okay] [SUB:and-&gt;okay] [SUB:then-&gt;okay] [SUB:we-&gt;okay] [SUB:will-&gt;okay] [SUB:start-&gt;okay] [SUB:you-&gt;okay] [SUB:on-&gt;okay] [SUB:on-&gt;okay] [SUB:intravenous-&gt;okay] [SUB:intravenous-&gt;okay] [SUB:that-&gt;okay] [SUB:is-&gt;okay] okay [SUB:that-&gt;okay] [SUB:is-&gt;for] [SUB:cool-&gt;the] [SUB:culture-&gt;investigation] [SUB:and-&gt;cultural] sensitivity could take about seventytwo hours [DEL:to] to [SUB:five-&gt;find] [SUB:days-&gt;this] [SUB:before-&gt;for] [SUB:it-&gt;you] [SUB:will-&gt;to] be ready do you understand [DEL:yeah] no problem doctor thank you no problem doctor [INS:thank] [INS:you] [INS:very] [INS:much] [INS:i] [INS:think] [INS:that] [INS:is] [INS:fine] [INS:i] [INS:will] [INS:just] [INS:do] [INS:the] [INS:labs] [INS:and] [INS:wait] [INS:for] [INS:you] [INS:to] [INS:start] [INS:the] [INS:treatment] thank you very much i think that is fine i will just yeah i will just do the labs and wait for just for you to start the treatment thank you [INS:no] [INS:i] [INS:do] [INS:not] [INS:promise]</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor [SUB:sadeko-&gt;shadak] good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to [DEL:the] [SUB:hospital-&gt;you] today what was the complaints so doctor i have been coughing for about a week now and i have been also also [INS:at] [SUB:have-&gt;yes] you also have what so and i also have i have also been running temperature for about five days so [INS:it] [INS:is] [INS:been] [INS:really] [INS:yes] [INS:yes] [INS:and] [SUB:you-&gt;the] [SUB:have-&gt;cough] [SUB:running-&gt;has] [SUB:temperature-&gt;been] for [INS:the] [INS:cough] [INS:has] [SUB:five-&gt;been] [SUB:days-&gt;for] [SUB:yes-&gt;how] [SUB:yes-&gt;long] for about a week now a week yes okay [DEL:all] [SUB:right-&gt;alright] so the cough did it start suddenly or gradually the cough started suddenly just started like that i just [DEL:just] [DEL:woke] [DEL:up] [DEL:more] [DEL:morning] [DEL:and] [DEL:started] [DEL:coughing] [DEL:about] [DEL:a] [DEL:week] [DEL:ago] [DEL:yes] was there was there any symptoms like [SUB:catarrh-&gt;qatar] or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes [DEL:okay] so now the cough how does it sound does it sound like [INS:the] barking does it sound like [INS:a] [SUB:it-&gt;and] [SUB:is-&gt;it] comes in [DEL:bouts] and then you have to take a deep breath [DEL:when] when you say barking [DEL:do] [DEL:you] are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] no no no no no no [SUB:mine-&gt;no] [SUB:is-&gt;no] [SUB:not-&gt;no] [SUB:that-&gt;no] [SUB:i-&gt;no] [SUB:did-&gt;no] [SUB:not-&gt;no] [SUB:i-&gt;no] [SUB:did-&gt;no] [SUB:not-&gt;no] [SUB:experience-&gt;no] [SUB:anything-&gt;no] [SUB:like-&gt;no] [SUB:that-&gt;no] [SUB:okay-&gt;no] [SUB:so-&gt;no] [SUB:is-&gt;no] [SUB:the-&gt;no] [SUB:cough-&gt;no] [SUB:productive-&gt;no] [SUB:of-&gt;no] [SUB:phlegm-&gt;no] [SUB:yes-&gt;no] [SUB:yes-&gt;no] [SUB:it-&gt;no] [SUB:is-&gt;no] [SUB:productive-&gt;no] [SUB:when-&gt;no] [SUB:i-&gt;no] [SUB:yes-&gt;no] [SUB:when-&gt;no] [SUB:i-&gt;no] [SUB:cough-&gt;no] [SUB:i-&gt;no] [SUB:bring-&gt;no] [SUB:out-&gt;no] [SUB:some-&gt;no] [SUB:some-&gt;no] substance from my mouth yes so what is the colour of the substance [SUB:err-&gt;yeah] it is about [INS:yeah] it is clear it is whitish it is [SUB:not-&gt;normal] it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no [DEL:there] [DEL:was] [DEL:no] [DEL:blood] [DEL:in] [DEL:it] there was no blood in it there was no blood in it at any point [DEL:yes] and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [INS:i] [SUB:vomiting-&gt;am] i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough no no [SUB:there-&gt;that] was [INS:not] [INS:in] [SUB:nothing-&gt;my] i was not i had nothing my my even when i was coughing my chest was not [SUB:paining-&gt;burning] me nothing it was just the cough [SUB:then-&gt;and] i i discovered after a few days after that i [DEL:just] [SUB:started-&gt;was] running temperature too my body was very very hot it was very hot [DEL:that] i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not [INS:pain] [SUB:paining-&gt;in] me at all [SUB:your-&gt;the] chest was not [INS:pain] [SUB:paining-&gt;in] me is there anybody coughing around you no there [INS:is] nobody i stay alone right now so i have nobody around me i do not stay with people so i do not [SUB:have-&gt;remember] anybody around me that is coughing too and [SUB:at-&gt;i] [SUB:work-&gt;walk] [SUB:too-&gt;to] there is nobody coughing around me so okay so you stay alone you are not [DEL:here] in [SUB:an-&gt;a] [SUB:overcrowded-&gt;crowded] place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i started to have some difficulty in breathing so like that got me really scared [DEL:like] i was i was [DEL:i] [DEL:was] [DEL:just] feeling breathless for a moment comes and goes [SUB:then-&gt;and] and since that since then the breathlessness [SUB:has-&gt;have] become more worsened so that is what exactly prompted me to [INS:come] [SUB:completely-&gt;quickly] to see you [INS:so] you are finding it difficult to breathe yes [INS:the] [INS:cough] yes when you sleep at night [INS:do] you sweat excessively no at all i do not i do not [SUB:slept-&gt;sleep] i do not sweat [SUB:when-&gt;in] [SUB:i-&gt;a] sleep [SUB:at-&gt;department] [SUB:night-&gt;yes] okay so what is what [SUB:relieves-&gt;removes] the breathlessness any [DEL:change] [SUB:in-&gt;changing] position that relieves the breathlessness or [DEL:it] is constant no it is not associated with any any position nothing [DEL:i] [SUB:just-&gt;and] it just comes and goes like i just feel breathless [SUB:for-&gt;with] a while then it [SUB:relieves-&gt;releases] me then it comes again especially when [DEL:i] [DEL:am] especially when i am coughing okay has this worsened progressively yes yes [SUB:it-&gt;that] [SUB:has-&gt;is] gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to [SUB:work-&gt;walk] for the past two days because of the cough and the fact that [DEL:i] [DEL:have] i have not been feeling well generally [DEL:in] [DEL:my] [DEL:body] so [DEL:that] [DEL:is] [SUB:so-&gt;no] [SUB:now-&gt;no] this fever that you were having was it did it start suddenly or gradually [DEL:it] started it started gradually then became i became very hot and [DEL:it] has been like that it has been like that so the fever is high grade [DEL:you] [DEL:are] very hot yes yes it is [SUB:high-&gt;i] [SUB:did-&gt;do] you [SUB:at-&gt;have] any [INS:points] [INS:that] [SUB:point-&gt;you] [SUB:yes-&gt;can] check by yourself at home your temperature yes i did i did i have a [SUB:thermometer-&gt;stomach] [SUB:it-&gt;i] was about [INS:there] was about [INS:thirty] [INS:eight] [INS:point] [INS:nine] [INS:thirty] [SUB:thirtyeightnine-&gt;point] [SUB:thirtyeightnine-&gt;nine] okay and what [SUB:does-&gt;do] what do you do that [SUB:relieves-&gt;releases] the fever [INS:well] i took some i took some [INS:past] [SUB:paracetamol-&gt;more] it relieved [SUB:a-&gt;the] bit then but it [DEL:did] did not last long i just [DEL:i] i became hot again and it has been like that ever since so i just want to ask you some questions has [SUB:anything-&gt;this] happened before in the past okay has it happened in the past no no no no this is the first time i am [DEL:experiencing] [DEL:that] [DEL:is] [DEL:why] [SUB:i-&gt;expressing] [SUB:am-&gt;this] this is the first time i am [SUB:experiencing-&gt;expressing] this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic [INS:do] [INS:you] [SUB:during-&gt;do] [SUB:your-&gt;you] [SUB:blood-&gt;need] [SUB:group-&gt;a] [SUB:and-&gt;blood] [SUB:genotype-&gt;pressure] no i am not [INS:to] doctor i am fine no i have [DEL:nothing] [DEL:and] [DEL:that] [DEL:is] [DEL:why] [DEL:this] [SUB:is-&gt;not] [SUB:surprising-&gt;no] are you [DEL:hypertensive] [DEL:what] [DEL:did] [SUB:you-&gt;a] [SUB:say-&gt;hypertensive] [SUB:i-&gt;or] [SUB:cannot-&gt;diabetic] [SUB:hear-&gt;are] you [DEL:properly] [DEL:sir] [DEL:are] [SUB:you-&gt;a] hypertensive or diabetic none none none none [DEL:no] no i have none of them i have none of them so what have you what have you done to care for yourself so far [DEL:i] [DEL:just] [DEL:i] [DEL:just] i just [SUB:tried-&gt;try] to get some cough syrup [INS:up] but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew i know i needed to like [SUB:come-&gt;because] to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that [SUB:i-&gt;current] [SUB:can-&gt;but] [SUB:remember-&gt;none] have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your [SUB:to-&gt;so] the symptoms you are having so do you have headache headache [INS:it] just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no [DEL:okay] okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] [INS:no] no no [SUB:i-&gt;no] [SUB:do-&gt;no] [SUB:not-&gt;no] [SUB:have-&gt;no] [SUB:any-&gt;no] [SUB:diarrhea-&gt;no] [SUB:or-&gt;no] [SUB:vomiting-&gt;no] no [SUB:i-&gt;no] [SUB:have-&gt;no] [SUB:not-&gt;no] [SUB:vomited-&gt;no] [SUB:at-&gt;no] [SUB:all-&gt;no] [SUB:you-&gt;no] [SUB:have-&gt;no] [SUB:any-&gt;no] [SUB:bone-&gt;no] [SUB:pain-&gt;no] [SUB:yes-&gt;no] no [SUB:the-&gt;no] no [SUB:the-&gt;no] [SUB:most-&gt;no] [SUB:it-&gt;no] [SUB:is-&gt;the] [SUB:just-&gt;most] [SUB:it-&gt;of] [SUB:is-&gt;the] just the [SUB:shortest-&gt;shouters] of breath [DEL:i] have been [SUB:having-&gt;happening] the difficulty in breathing [DEL:i] have been [DEL:having] [DEL:that] [SUB:is-&gt;happening] [SUB:just-&gt;so] that is [DEL:just] [DEL:so] [SUB:in-&gt;the] summary you are telling me in summary you are telling me you had [DEL:you] you have had cough fever and difficulty in breathing yes right and your cough is productive yes [DEL:all] [SUB:right-&gt;alright] so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know [DEL:if] to know whatever is going on in your chest [DEL:whether] there is a chest infection that is causing you to have a fever and the and the cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count [INS:or] a full blood count [DEL:which] [SUB:will-&gt;to] tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do [DEL:you] [SUB:know-&gt;a] [SUB:electrocyte-&gt;neutrophil] segmentation [SUB:rates-&gt;rate] to know whether there is an inflammatory process [SUB:going-&gt;brain] on do you understand and then we are also going to take your sputum your the phlegm and we are going to send it for culture sensitivity to know what bacteria is is being cultured please i just want to ask you do you smoke no no i do not [INS:so] doctor i am a good christian i do not smoke i do not drink you do not you do not drink alcohol either i do not i do not do any of those i do not do [SUB:drugs-&gt;jobs] i do not do any of that i am going to ask you some other questions do you have [INS:there] [SUB:their-&gt;are] kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i [DEL:will] [DEL:need] [DEL:to] [DEL:take] [DEL:basically] [SUB:i-&gt;do] [SUB:just-&gt;not] want to ask [INS:if] [INS:i] [SUB:ifi-&gt;do] [SUB:just-&gt;not] want to ask if you have multiple sexual partners and [DEL:then] your sexual practices no no [DEL:you] [DEL:have] oral sex [DEL:i] [DEL:am] [DEL:married] no [SUB:not-&gt;none] at all not at all [DEL:i] [DEL:am] [DEL:married] so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like [DEL:diagnosis] [DEL:the] [SUB:because-&gt;diagnoses] the because of what is causing the cough and the fever we have some [DEL:this] [SUB:thing-&gt;just] [SUB:at-&gt;in] the back of our mind which could be the because do you understand we think you have a pneumonia pneumonia [DEL:a] chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start you on [DEL:the] cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you [DEL:will] start [SUB:treatment-&gt;treatments] with the antibiotics [DEL:and] and the cough syrup there will be the breathlessness [INS:business] is going to reduce but we your we would have checked [DEL:your] your oxygen saturation and we [DEL:will] see that it is fine so there will be no need to place you on on oxygen so you are [DEL:going] [SUB:to-&gt;against] [SUB:have-&gt;having] you do [DEL:a] full [SUB:blood-&gt;block] [SUB:count-&gt;out] in sputum and [INS:end] [SUB:microscopy-&gt;microscopic] culture sensitivity [DEL:you] are going to have you [SUB:do-&gt;doing] [SUB:any-&gt;the] [SUB:erythrocyte-&gt;enteric] [SUB:segmentation-&gt;site] [SUB:rate-&gt;sedimentation] [SUB:and-&gt;rates] [SUB:you-&gt;and] are going to do a chest xray so let us see if it is [DEL:a] structural problem or a functional problem do you understand okay [DEL:doctor] [DEL:so] [DEL:doctor] [DEL:do] [DEL:i] do you want to ask [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital or do i [INS:have] [SUB:that-&gt;to] [SUB:can-&gt;go] [SUB:i-&gt;home] can i be treated from home because i do not know [DEL:we] [DEL:we] we are going to admit you for some time to evaluate you and because of the breathlessness you are having right [DEL:and] [DEL:then] [DEL:we] [DEL:will] [DEL:start] [DEL:you] [DEL:on] [DEL:on] [DEL:intravenous] [DEL:intravenous] [DEL:that] [DEL:is] okay that is [DEL:cool] [DEL:culture] [DEL:and] [DEL:sensitivity] [DEL:could] [DEL:take] [DEL:about] [DEL:seventytwo] [DEL:hours] [DEL:to] [DEL:to] [DEL:five] [DEL:days] [DEL:before] [DEL:it] [DEL:will] [DEL:be] [DEL:ready] [DEL:do] [DEL:you] [DEL:understand] [DEL:yeah] [DEL:no] [DEL:problem] [DEL:doctor] [DEL:thank] [DEL:you] [DEL:no] [SUB:problem-&gt;fine] [SUB:doctor-&gt;so] thank you very much i think that is fine i will just yeah i will just do the [SUB:labs-&gt;laps] and wait for [SUB:just-&gt;is] for you to start the treatment thank you</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor [SUB:sadeko-&gt;shadakoff] good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine [INS:on] not too fine that is why i came to the hospital today what [SUB:was-&gt;is] the complaints so doctor i have been coughing for about a week now and i have been also [SUB:also-&gt;at] [SUB:have-&gt;yes] you also have what so and i also [DEL:have] [DEL:i] have also been running temperature for about five days [DEL:so] [DEL:you] [SUB:have-&gt;it] [SUB:running-&gt;is] [SUB:temperature-&gt;been] [SUB:for-&gt;really] five days yes yes [INS:and] [INS:the] [INS:cough] [INS:has] [INS:been] [INS:for] [INS:the] [INS:cough] [INS:has] [INS:been] [INS:for] [INS:how] [INS:long] for about a week now a week yes okay all right so the cough did [SUB:it-&gt;this] start [INS:soddening] [SUB:suddenly-&gt;the] or gradually the cough started suddenly just started like that i [DEL:just] just woke up more morning and started coughing [SUB:about-&gt;by] a week ago yes [DEL:was] [DEL:there] was there any symptoms like [SUB:catarrh-&gt;qatar] or [DEL:any] any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like [SUB:barking-&gt;backing] does [SUB:it-&gt;this] sound like it [DEL:is] comes in [SUB:bouts-&gt;body] and then you have to take a [DEL:deep] [DEL:breath] [SUB:when-&gt;different] when you say [DEL:barking] [DEL:do] [SUB:you-&gt;backing] are you do you mean like a dog or what do you mean by [SUB:barking-&gt;backing] yes yes sounds like a dog [DEL:barking] [SUB:no-&gt;back] no no no no no mine is not [DEL:that] [DEL:i] [DEL:did] [DEL:not] [DEL:i] [DEL:did] [DEL:not] [DEL:experience] [DEL:anything] [DEL:like] that okay so is the cough productive of [SUB:phlegm-&gt;flame] yes yes it is productive [DEL:when] [DEL:i] yes when i cough i bring out [DEL:some] some substance from my mouth yes so what is the colour of the substance [SUB:err-&gt;yeah] it is about [INS:yeah] it is clear it is whitish [DEL:it] [DEL:is] [DEL:not] it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point [SUB:yes-&gt;okay] and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [DEL:vomiting] i do not vomit at all okay and you did not have [SUB:catarrh-&gt;catar] or difficulty in swallowing prior to [INS:the] onset of the cough [INS:no] no no [SUB:there-&gt;i] was nothing i was not i had nothing [DEL:my] [DEL:my] even when i was coughing my chest was not [SUB:paining-&gt;painting] me nothing it was just the cough [DEL:then] [SUB:i-&gt;and] i discovered after a few days after that i [SUB:just-&gt;was] [SUB:started-&gt;hired] running temperature too my body was very very hot it was very hot [DEL:that] i was shivering so you are telling me [DEL:there] [DEL:is] [DEL:no] there is no cough there is no chest pain no [DEL:there] [DEL:is] there is no chest pain my chest was not paining me at all [SUB:your-&gt;it] [SUB:chest-&gt;just] was not [DEL:paining] [SUB:me-&gt;pain] is there anybody coughing around you no there [INS:is] nobody i stay alone right now so i have nobody around me i do not [SUB:stay-&gt;tell] [SUB:with-&gt;you] people so i do not [DEL:have] [DEL:anybody] [DEL:around] [DEL:me] [DEL:that] [SUB:is-&gt;remember] coughing too and [SUB:at-&gt;i] [SUB:work-&gt;walk] too there is nobody coughing around me [DEL:so] okay so you stay alone you are not [DEL:here] in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and [DEL:i] [DEL:was] i [SUB:started-&gt;said] to have some difficulty in breathing so like that got me really scared [DEL:like] i was [DEL:i] [DEL:was] [DEL:i] [DEL:was] [DEL:just] feeling breathless for a moment comes and goes [DEL:then] and since that since then the breathlessness has become more worsened so that is what exactly prompted me to [INS:come] [SUB:completely-&gt;quickly] to see you you are finding it difficult to breathe yes yes when you sleep at night [INS:do] you sweat excessively no at all [DEL:i] [DEL:do] [DEL:not] i do not [SUB:slept-&gt;sleep] i do not sweat [DEL:when] [DEL:i] [DEL:sleep] [SUB:at-&gt;yes] [SUB:night-&gt;okay] okay so what is what relieves the breathlessness any change in position that relieves the breathlessness or [DEL:it] [SUB:is-&gt;this] constant no it is not associated with [DEL:any] any position nothing i just it just comes and goes like i just feel breathless for a while then it relieves me then it comes again especially when i am [SUB:especially-&gt;sitting] when i am coughing [DEL:okay] has this worsened progressively yes yes [SUB:it-&gt;that] [SUB:has-&gt;is] gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that [DEL:i] [DEL:have] i have not been feeling well generally in my body so that is [DEL:so] now this fever that you were having was it did [SUB:it-&gt;you] start [DEL:suddenly] [DEL:or] [SUB:gradually-&gt;sodding] it [SUB:started-&gt;gradually] it started gradually then [DEL:became] i became very hot and [DEL:it] has been like that it has been like that so the fever is [DEL:high] [SUB:grade-&gt;highgrade] you are very hot yes yes it is high did you [INS:attend] [INS:a] [SUB:at-&gt;question] [SUB:any-&gt;to] [SUB:point-&gt;try] [SUB:yes-&gt;and] check by yourself at [DEL:home] your temperature yes i did i did i [DEL:have] [SUB:a-&gt;average] thermometer [DEL:it] [DEL:was] [SUB:about-&gt;i] was about thirtyeightnine [SUB:thirtyeightnine-&gt;thirtynine] okay and [DEL:what] [DEL:does] what do you do that relieves the fever i took some [DEL:i] [DEL:took] [SUB:some-&gt;past] [SUB:paracetamol-&gt;more] it relieved [SUB:a-&gt;the] bit then but it did [INS:it] did not last long [SUB:i-&gt;it] [SUB:just-&gt;is] [SUB:i-&gt;just] [SUB:i-&gt;it] became [SUB:hot-&gt;what] again and it has been like that ever since so i just want to ask you some questions has [INS:this] [SUB:anything-&gt;thing] happened before in the past okay has it happened in the past no no no no this is the first time i am [DEL:experiencing] [DEL:that] [SUB:is-&gt;expressing] [SUB:why-&gt;as] i am this is the first time i am experiencing this kind of thing okay [SUB:this-&gt;it] is the first time are you do you have any medical condition like are you asthmatic [INS:do] [INS:you] [SUB:during-&gt;need] [SUB:your-&gt;a] blood group and genotype [INS:oh] no i am not doctor i am fine no i have nothing [DEL:and] [DEL:that] [DEL:is] [DEL:why] [DEL:this] [DEL:is] [DEL:surprising] are [DEL:you] [DEL:hypertensive] [DEL:what] [DEL:did] you [SUB:say-&gt;hypocensing] i cannot hear you properly sir are you hypertensive or diabetic [DEL:none] none none [SUB:none-&gt;no] no no i have none of them i have none of them so what have you what have you done to care for yourself so far [DEL:i] [DEL:just] [DEL:i] [DEL:just] i just tried to get some [DEL:cough] [DEL:syrup] [SUB:but-&gt;coughs] [SUB:they-&gt;here] [SUB:did-&gt;up] [SUB:not-&gt;but] they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started [DEL:i] [DEL:knew] [DEL:i] [DEL:knew] i know i needed [DEL:to] [DEL:like] [DEL:come] to speak to someone to a doctor so that is why i came today for you to like for me to [DEL:like] know what is wrong with me and treat myself basically [DEL:have] [DEL:you] [DEL:been] have you been admitted before no [DEL:not] [DEL:not] not that [SUB:i-&gt;current] [SUB:can-&gt;but] [SUB:remember-&gt;none] have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the symptoms you are having so do you have headache headache [INS:yes] [SUB:just-&gt;it] comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain no no i do not have [DEL:any] [DEL:diarrhea] [SUB:or-&gt;a] [SUB:vomiting-&gt;problem] no i [SUB:have-&gt;am] not vomited at all you have any bone pain yes no [DEL:the] no the most [DEL:it] [DEL:is] [DEL:just] it is just the [SUB:shortest-&gt;shortness] of breath i have been having the difficulty in breathing [DEL:i] [SUB:have-&gt;has] been having [DEL:that] [DEL:is] [DEL:just] [DEL:that] [DEL:is] [DEL:just] so in summary you are telling me [DEL:in] [DEL:summary] [SUB:you-&gt;some] are telling me you had [DEL:you] you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know if to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever [DEL:and] [DEL:the] and the cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count [INS:of] a full blood count [DEL:which] [SUB:will-&gt;to] tell us whether there is an infection going on depending on the parameters that are [SUB:elevated-&gt;indicated] or reduced do you understand we are going to do [DEL:you] [SUB:know-&gt;a] [SUB:electrocyte-&gt;neutrocyte] segmentation [SUB:rates-&gt;rate] to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum [DEL:your] the [SUB:phlegm-&gt;flame] and we are going to send it for [SUB:culture-&gt;cultural] sensitivity to know what bacteria [DEL:is] is being [SUB:cultured-&gt;caught] please i just want to ask you do you smoke no no i do not [INS:so] doctor i am a good christian i [DEL:do] [SUB:not-&gt;just] [SUB:smoke-&gt;spoke] i do not [DEL:drink] [DEL:you] [DEL:do] [SUB:not-&gt;think] you do not drink alcohol either [DEL:i] [DEL:do] [DEL:not] i do not [SUB:do-&gt;drink] any of those i do not do drugs i do not [DEL:do] [SUB:any-&gt;drink] of that i am going to ask you some other questions do you have [INS:there] [SUB:their-&gt;are] kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start [SUB:treating-&gt;with] me [DEL:and] [DEL:what] [DEL:i] [DEL:will] [DEL:need] [DEL:to] [DEL:take] [DEL:basically] i just want to ask [INS:if] [SUB:ifi-&gt;i] just want to ask if you have multiple sexual partners and [DEL:then] your sexual practices no no [INS:do] you have oral sex i am married no not at all not at all [DEL:i] [DEL:am] [DEL:married] so we are going to start you from the history and the examination [SUB:we-&gt;you] have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis [DEL:the] [DEL:because] the because of what is causing the cough and the fever we have some [DEL:this] [DEL:thing] at the back of our mind which could be the because [DEL:do] you understand we think you have a [DEL:pneumonia] pneumonia a chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start [DEL:you] on the cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you [DEL:will] start treatment with the antibiotics [DEL:and] and the cough syrup there will be the breathlessness is going to reduce but [DEL:we] [DEL:your] we [SUB:would-&gt;will] have checked [DEL:your] your oxygen saturation and we [DEL:will] see that it is fine so there will be no need to place you [DEL:on] on oxygen so [SUB:you-&gt;we] are going to have you do a full [SUB:blood-&gt;block] count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscopic] [SUB:culture-&gt;control] sensitivity [SUB:you-&gt;i] [SUB:are-&gt;am] going to have you do [SUB:any-&gt;an] [SUB:erythrocyte-&gt;intrusive] [SUB:segmentation-&gt;sedimentation] rate and [SUB:you-&gt;we] are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor [DEL:so] [DEL:doctor] [DEL:do] [DEL:i] [SUB:do-&gt;okay] you want to ask [INS:me] [SUB:the-&gt;a] question [SUB:if-&gt;do] you have any questions yes i was going to ask that are you going to keep me in [SUB:the-&gt;your] hospital [DEL:or] [DEL:do] [DEL:i] [DEL:that] [DEL:can] [DEL:i] can i be treated from home because i do not know [DEL:we] [DEL:we] we are going to admit you for some time to evaluate you and because of the breathlessness you are having right [DEL:and] [DEL:then] [DEL:we] [DEL:will] [DEL:start] [DEL:you] [DEL:on] [DEL:on] [DEL:intravenous] [DEL:intravenous] [DEL:that] [SUB:is-&gt;okay] okay that is [DEL:cool] [DEL:culture] [DEL:and] [DEL:sensitivity] [DEL:could] [DEL:take] [SUB:about-&gt;fine] seventytwo hours [DEL:to] to five days [SUB:before-&gt;for] [SUB:it-&gt;you] [SUB:will-&gt;to] be ready do you understand [DEL:yeah] no problem doctor [DEL:thank] [DEL:you] no problem doctor thank you very much i think that is fine i will just yeah i will just do the labs and wait [DEL:for] [DEL:just] for you to start the treatment thank you</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor sadeko good [SUB:afternoon-&gt;shadekoff] good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to the hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also [INS:complaints] also have [INS:coughing] you also have what so and i also have i have also been running temperature for about five days so you have running temperature for five days yes yes [INS:cough] [INS:cough] [INS:cough] for about a week now a week yes okay all right so the cough did it start suddenly or gradually the cough started suddenly just started like that i just just woke up more morning and started coughing about a week ago yes was there was there any symptoms like catarrh or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like barking does it sound like it is comes in [SUB:bouts-&gt;barking] and then you have to take a deep breath when when you say barking do you are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no mine is not that i did not i did not experience anything like that okay so is the cough productive of phlegm yes yes it is productive when i yes when i cough i bring out some some substance from my mouth yes so what is the colour of the substance err it is about it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like vomiting i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough [SUB:no-&gt;cough] no there was nothing i was not i had nothing my my even when i was coughing my chest was not paining me nothing it was just the cough then i i discovered after a few days after that i just started running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not paining me at all your [DEL:chest] was not [DEL:paining] me is there anybody coughing around you no there nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and at work too there is nobody coughing around me so okay so you stay alone you are not here in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i started to have some difficulty in breathing so like that got me really scared like i was i was i was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to completely to see you you are finding it difficult to breathe yes yes when you sleep at night you sweat excessively no at all i do not i do not slept i do not sweat when i sleep at night okay so what is what relieves the breathlessness any change in position that relieves the breathlessness or it is constant no it is not associated with any any position nothing i just it just comes and goes like i just feel [SUB:breathless-&gt;breathlessness] for a while then it relieves me then it comes again especially when i am especially when i am coughing okay has this worsened progressively yes yes it has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to [SUB:work-&gt;walk] for the past two days because of the cough and the fact that i have i have not been feeling well generally in my body so that is so now this fever that you were having was it did it start suddenly or gradually it started it started gradually then became i became very hot and it has been like that it has been like that so the fever is high grade you are very hot yes yes it is high did you at any point yes check by yourself at home your [SUB:temperature-&gt;job] yes i did i did i have a [SUB:thermometer-&gt;thirtyeightnine] it was about was about [SUB:thirtyeightnine-&gt;thirtysevennine] [SUB:thirtyeightnine-&gt;thirtysevennine] okay and what does what do you do that relieves the fever i took some i took some [SUB:paracetamol-&gt;more] it relieved a bit then but it did did not last long i just i i became hot again and it has been like that ever since so i just want to ask you some questions has anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why i am this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic during your blood group and genotype no i am not doctor i am fine no i have nothing and that is why this is surprising are you [DEL:hypertensive] what did you say i cannot hear you properly sir are you hypertensive or diabetic none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just i just tried to get some cough syrup but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew i know i needed to like come to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that i can remember have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the symptoms you are having so do you have headache headache just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;kata] no at all okay do you have any abdominal pain no no i do not have any [DEL:diarrhea] [SUB:or-&gt;abdominal] [SUB:vomiting-&gt;pain] no i have [SUB:not-&gt;abdominal] [SUB:vomited-&gt;pain] at all you have any bone pain yes no [INS:vomited] the no [SUB:the-&gt;bone] [SUB:most-&gt;pain] it is just it is just the [SUB:shortest-&gt;shoulders] of breath i have been having the difficulty in breathing i have been having that is just that is just so in summary you are telling me in summary you are telling me you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know if to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and the and the cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your the [SUB:phlegm-&gt;deflame] and we are going to send it for culture sensitivity to know what bacteria is is being cultured please i just want to ask you do you smoke no no i do not doctor i am a good christian i do not smoke i do not drink you do not you do not drink alcohol either i do not i do not [SUB:do-&gt;drink] any of those i do not do drugs i do not [SUB:do-&gt;drink] any of that i am going to ask you some other questions do you have their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i will need to take basically i just want to ask ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex i am married no not at all not at all i am married so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because the because of what is causing the cough and the fever we have some this thing at the back of our mind which could be the because do you understand we think you have a pneumonia pneumonia a chest infection so we are going to start you on a [SUB:broad-&gt;blood] spectrum antibiotics right and then we are going to start you on the cough [SUB:syrup-&gt;serum] right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start treatment with the antibiotics and and the cough syrup there will be the breathlessness is going to reduce but we your we would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on on oxygen so you are going to have you do a full blood count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscop] [SUB:culture-&gt;contrast] sensitivity you are going to have you do any [SUB:erythrocyte-&gt;ultrasound] segmentation rate and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor so doctor do i do you want to ask the question if you have any questions yes i was going to ask that are you going to keep me in the hospital or do i that can i can i be treated from home because i do not know we we we are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then we will start you on on [SUB:intravenous-&gt;okay] [SUB:intravenous-&gt;okay] that is okay that is cool [SUB:culture-&gt;investigation] and sensitivity could take about seventytwo hours to to five days before it will be ready do you understand yeah no problem doctor thank you no problem doctor [INS:labs] [INS:treatment] thank you very much i think that is fine i will just yeah i will just do the labs and wait for just for you to start the treatment thank you</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor sadeko good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to the hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also also have you also have what so and i also have i have also been running temperature for about five days so you [SUB:have-&gt;cough] running [SUB:temperature-&gt;been] for [INS:cough] five days yes yes for about a week now a week yes okay all right so the cough did it start suddenly or gradually the cough started suddenly just started like that i just just woke up more morning and started [DEL:coughing] about a week ago yes was there was there any symptoms like [SUB:catarrh-&gt;qatar] or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like barking does it sound like it is comes in bouts and then you have to take a deep breath when when you say barking do you are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no mine is not that i did not i did not experience anything like that okay so is the [SUB:cough-&gt;no] productive of [SUB:phlegm-&gt;no] yes yes it is productive when i yes when i [SUB:cough-&gt;no] i bring out some some substance from my mouth yes so what is the colour of the substance err it is about it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no [DEL:blood] in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [SUB:vomiting-&gt;am] i do not vomit at all okay and you did not have catarrh or difficulty [DEL:in] swallowing prior to onset of the cough no no there was nothing i was not i had nothing my my even when i was coughing my chest was not [SUB:paining-&gt;burning] me nothing it was just the cough then i i discovered after a few days after that i just started running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not [INS:pain] [SUB:paining-&gt;in] me at all your chest was not [INS:pain] [SUB:paining-&gt;in] me is there anybody coughing around you no there nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and at work too there is nobody coughing around me so okay so you stay alone you are not here in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i started to have some difficulty in breathing so like that got me really scared like i was i was i was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to completely to see you you are finding it difficult to breathe yes [INS:cough] yes when you sleep at night you sweat excessively no at all i do not i do not slept i do not sweat when i sleep at night okay so what is what relieves the breathlessness any change in position that relieves the breathlessness or it is constant no it is not associated with any any position nothing i just it just comes and goes like i just feel breathless for a while then it relieves me then it comes again especially when i am especially when i am coughing okay has this worsened progressively yes yes it has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to [SUB:work-&gt;walk] for the past two days because of the cough and the fact that i have i have not been feeling well generally in my body so that is so now this fever that you were having was it did it start suddenly or gradually it started it started gradually then became i became very hot and it has been like that it has been like that so the fever is high grade you are very hot yes yes it is high did you at any point yes check by yourself at home your temperature yes i did i did i have a [SUB:thermometer-&gt;stomach] it was about was about [SUB:thirtyeightnine-&gt;point] [SUB:thirtyeightnine-&gt;nine] okay and what does what do you do that relieves the fever i took some i took some [SUB:paracetamol-&gt;more] it relieved a bit then but it did did not last long i just i i became hot again and it has been like that ever since so i just want to ask you some questions has anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why i am this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic during your [SUB:blood-&gt;need] [SUB:group-&gt;a] [SUB:and-&gt;blood] [SUB:genotype-&gt;pressure] no i am not doctor i am fine no i have nothing and that is why this is surprising are you [DEL:hypertensive] what did you [SUB:say-&gt;hypertensive] i [SUB:cannot-&gt;diabetic] hear you properly sir are you hypertensive or diabetic none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just i just tried to get some cough syrup but they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew i know i needed to like come to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that i can remember have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the symptoms you are having so do you have headache headache just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain no no i do not have any [SUB:diarrhea-&gt;no] or [SUB:vomiting-&gt;no] no i have not [SUB:vomited-&gt;no] at all you have any [SUB:bone-&gt;no] [SUB:pain-&gt;no] yes no the no the most it is just it is just the [SUB:shortest-&gt;shouters] of breath i have been having the difficulty in breathing i have been having that is just that is just so in summary you are telling me in summary you are telling me you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know if to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and the and the cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know [SUB:electrocyte-&gt;neutrophil] segmentation [SUB:rates-&gt;rate] to know whether there is an inflammatory process [SUB:going-&gt;brain] on do you understand and then we are also going to take your sputum your the phlegm and we are going to send it for culture sensitivity to know what bacteria is is being cultured please i just want to ask you do you smoke no no i do not doctor i am a good christian i do not smoke i do not drink you do not you do not drink alcohol either i do not i do not do any of those i do not do [SUB:drugs-&gt;jobs] i do not do any of that i am going to ask you some other questions do you have their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i will need to take basically i just want to ask ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex i am married no not at all not at all i am married so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because the because of what is causing the cough and the fever we have some this thing at the back of our mind which could be the because do you understand we think you have a pneumonia pneumonia a chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start you on the cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start [SUB:treatment-&gt;treatments] with the antibiotics and and the cough syrup there will be the breathlessness is going to reduce but we your we would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on on oxygen so you are going to have you do a full [SUB:blood-&gt;block] [SUB:count-&gt;out] in sputum and [INS:end] [SUB:microscopy-&gt;microscopic] culture sensitivity you are going to have you do any [SUB:erythrocyte-&gt;enteric] [SUB:segmentation-&gt;site] [SUB:rate-&gt;sedimentation] and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor so doctor do i do you want to ask the question if you have any questions yes i was going to ask that are you going to keep me in the hospital or do i that can i can i be treated from home because i do not know we we we are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then we will start you on on [DEL:intravenous] [DEL:intravenous] that is okay that is cool [DEL:culture] and [DEL:sensitivity] could take about seventytwo hours to to five days before it will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just yeah i will just do the [SUB:labs-&gt;laps] and wait for just for you to start the treatment thank you</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>good afternoon sir i am doctor [SUB:sadeko-&gt;shadakoff] good afternoon good afternoon doctor how are you doing today sir doctor i am not i am not too fine not too fine that is why i came to the hospital today what was the complaints so doctor i have been coughing for about a week now and i have been also also have you also have what so and i also have i have also been running temperature for about five days so you have running [SUB:temperature-&gt;been] for five days yes yes [INS:cough] [INS:cough] for about a week now a week yes okay all right so the cough did it start suddenly or gradually the cough started suddenly just started like that i just just woke up more morning and started coughing about a week ago yes was there was there any symptoms like [SUB:catarrh-&gt;qatar] or any any difficulty in swallowing before the cough started no none like that i had nothing like that nothing like that you had nothing like that yes okay so now the cough how does it sound does it sound like [SUB:barking-&gt;backing] does it sound like it is comes in bouts and then you have to take a deep breath when when you say barking do you are you do you mean like a dog or what do you mean by barking yes yes sounds like a dog barking no no no no no no mine is not that i did not i did not experience anything like that okay so is the cough productive of [SUB:phlegm-&gt;flame] yes yes it is productive when i yes when i cough i bring out some some substance from my mouth yes so what is the colour of the substance err it is about it is clear it is whitish it is not it is just normal it is looking like saliva but it is very thick it is very thick was there blood in it at any point no there was no blood in it there was no blood in it there was no blood in it at any point yes and after you cough do you feel like vomiting or do you vomit no i do not i do not i do not feel like [DEL:vomiting] i do not vomit at all okay and you did not have [SUB:catarrh-&gt;catar] or difficulty in swallowing prior to onset of the cough no no there was nothing i was not i had nothing my my even when i was coughing my chest was not [SUB:paining-&gt;painting] me nothing it was just the cough then i i discovered after a few days after that i just started running temperature too my body was very very hot it was very hot that i was shivering so you are telling me there is no there is no cough there is no chest pain no there is there is no chest pain my chest was not paining me at all your [SUB:chest-&gt;just] was not [DEL:paining] [SUB:me-&gt;pain] is there anybody coughing around you no there nobody i stay alone right now so i have nobody around me i do not stay with people so i do not have anybody around me that is coughing too and at work too there is nobody coughing around me so okay so you stay alone you are not here in an overcrowded place yes but yes but doctor i noticed what actually prompted me to come is the fact that about two days ago i noticed that the cough became worsened and i was i started to have some difficulty in breathing so like that got me really scared like i was i was i was just feeling breathless for a moment comes and goes then and since that since then the breathlessness has become more worsened so that is what exactly prompted me to completely to see you you are finding it difficult to breathe yes yes when you sleep at night you sweat excessively no at all i do not i do not slept i do not sweat when i sleep at night okay so what is what relieves the breathlessness any change in position that relieves the breathlessness or it is constant no it is not associated with any any position nothing i just it just comes and goes like i just feel breathless for a while then it relieves me then it comes again especially when i am especially when i am coughing okay has this worsened progressively yes yes it has gotten very bad doctor that is why i came to the hospital does it affect does it affect your daily activities yes it does doctor i have not been able to work for the past two days because of the cough and the fact that i have i have not been feeling well generally in my body so that is so now this fever that you were having was it did it start suddenly or gradually it started it started gradually then became i became very hot and it has been like that it has been like that so the fever is [DEL:high] [SUB:grade-&gt;highgrade] you are very hot yes yes it is high did you at any point yes check by yourself at home your temperature yes i did i did i have a thermometer it was about was about thirtyeightnine [SUB:thirtyeightnine-&gt;thirtynine] okay and what does what do you do that relieves the fever i took some i took some [SUB:paracetamol-&gt;more] it relieved a bit then but it did did not last long i just i i became hot again and it has been like that ever since so i just want to ask you some questions has anything happened before in the past okay has it happened in the past no no no no this is the first time i am experiencing that is why i am this is the first time i am experiencing this kind of thing okay this is the first time are you do you have any medical condition like are you asthmatic during your blood group and genotype no i am not doctor i am fine no i have nothing and that is why this is surprising are you [DEL:hypertensive] what did you [SUB:say-&gt;hypocensing] i cannot hear you properly sir are you hypertensive or diabetic none none none none no no i have none of them i have none of them so what have you what have you done to care for yourself so far i just i just i just tried to get some [DEL:cough] [DEL:syrup] [SUB:but-&gt;coughs] they did not they did not seem to work properly they did not seem to work and since the difficulty [INS:in] breathing started i knew i knew i know i needed to like come to speak to someone to a doctor so that is why i came today for you to like for me to like know what is wrong with me and treat myself basically have you been have you been admitted before no not not not that i can remember have you done any surgical procedure before no no okay so i am just going to ask you some other questions just to know what exactly could be related to your to the symptoms you are having so do you have headache headache just comes once in a while maybe because the cough i have not been able to sleep really so kind of yeah kind of yes okay so any loss of consciousness no no no no okay okay do you have [SUB:catarrh-&gt;catar] no at all okay do you have any abdominal pain no no i do not have any [DEL:diarrhea] or [SUB:vomiting-&gt;problem] no i have not vomited at all you have any bone pain yes no the no the most it is just it is just the [SUB:shortest-&gt;shortness] of breath i have been having the difficulty in breathing i have been having that is just that is just so in summary you are telling me in summary you are telling me you had you you have had cough fever and difficulty in breathing yes right and your cough is productive yes all right so i am going to have to have to examine you right i am going to have to examine you and i am going to have to listen to your chest to know if to know whatever is going on in your chest whether there is a chest infection that is causing you to have a fever and the and the cough do you understand and then we are going to have you do some investigations like a chest xray a complete blood count a full blood count which will tell us whether there is an infection going on depending on the parameters that are elevated or reduced do you understand we are going to do you know electrocyte segmentation rates to know whether there is an inflammatory process going on do you understand and then we are also going to take your sputum your the [SUB:phlegm-&gt;flame] and we are going to send it for [SUB:culture-&gt;cultural] sensitivity to know what bacteria is is being [SUB:cultured-&gt;caught] please i just want to ask you do you smoke no no i do not doctor i am a good christian i do not [SUB:smoke-&gt;spoke] i do not [DEL:drink] you do not you do not drink alcohol either i do not i do not [SUB:do-&gt;drink] any of those i do not do drugs i do not do [SUB:any-&gt;drink] of that i am going to ask you some other questions do you have their kind of personal questions can i go ahead yeah i just want to know doctor i just want to i just want to be fine i just want to know how soon you can start treating me and what i will need to take basically i just want to ask ifi just want to ask if you have multiple sexual partners and then your sexual practices no no you have oral sex i am married no not at all not at all i am married so we are going to start you from the history and the examination we have done and then we are going to ask you to do some investigations however we have some differentials like diagnosis the because the because of what is causing the cough and the fever we have some this thing at the back of our mind which could be the because do you understand we think you have a [DEL:pneumonia] pneumonia a chest infection so we are going to start you on a broad spectrum antibiotics right and then we are going to start you on the cough syrup right to treat the cough while we wait for the results of our investigations do you understand okay and then since there is no history of asthma by the time you will start treatment with the antibiotics and and the cough syrup there will be the breathlessness is going to reduce but we your we would have checked your your oxygen saturation and we will see that it is fine so there will be no need to place you on on oxygen so you are going to have you do a full [SUB:blood-&gt;block] count [SUB:in-&gt;a] sputum and [SUB:microscopy-&gt;microscopic] [SUB:culture-&gt;control] sensitivity you are going to have you do any [SUB:erythrocyte-&gt;intrusive] [SUB:segmentation-&gt;sedimentation] rate and you are going to do a chest xray so let us see if it is a structural problem or a functional problem do you understand okay doctor so doctor do i do you want to ask the question if you have any questions yes i was going to ask that are you going to keep me in the hospital or do i that can i can i be treated from home because i do not know we we we are going to admit you for some time to evaluate you and because of the breathlessness you are having right and then we will start you on on [DEL:intravenous] [DEL:intravenous] that is okay that is cool [DEL:culture] and [DEL:sensitivity] could take about seventytwo hours to to five days before it will be ready do you understand yeah no problem doctor thank you no problem doctor thank you very much i think that is fine i will just yeah i will just do the labs and wait for just for you to start the treatment thank you</t>
         </is>
       </c>
     </row>
@@ -1322,12 +1412,12 @@
 3          3       3         my         my         =            &lt;NA&gt;
 4          4       4       name       name         =            &lt;NA&gt;
 ...      ...     ...        ...        ...       ...             ...
-1999    1873    1784      thank      thank         =            &lt;NA&gt;
-2000    1874    1785        you        you         =            &lt;NA&gt;
-2001    1875    1786       very       very         =            &lt;NA&gt;
-2002    1876    1787       much       much         =            &lt;NA&gt;
-2003    1877    &lt;NA&gt;     doctor          _       del             500
-[2004 rows x 6 columns]</t>
+1998    1873    1784      thank      thank         =            &lt;NA&gt;
+1999    1874    1785        you        you         =            &lt;NA&gt;
+2000    1875    1786       very       very         =            &lt;NA&gt;
+2001    1876    1787       much       much         =            &lt;NA&gt;
+2002    1877    &lt;NA&gt;     doctor          _       del             500
+[2003 rows x 6 columns]</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
@@ -1339,12 +1429,12 @@
 3          3       3         my         my         =            &lt;NA&gt;
 4          4       4       name       name         =            &lt;NA&gt;
 ...      ...     ...        ...        ...       ...             ...
-1910    1873    1707      thank      thank         =            &lt;NA&gt;
-1911    1874    1708        you        you         =            &lt;NA&gt;
-1912    1875    1709       very       very         =            &lt;NA&gt;
-1913    1876    1710       much       much         =            &lt;NA&gt;
-1914    1877    1711     doctor     doctor         =            &lt;NA&gt;
-[1915 rows x 6 columns]</t>
+1906    1873    1707      thank      thank         =            &lt;NA&gt;
+1907    1874    1708        you        you         =            &lt;NA&gt;
+1908    1875    1709       very       very         =            &lt;NA&gt;
+1909    1876    1710       much       much         =            &lt;NA&gt;
+1910    1877    1711     doctor     doctor         =            &lt;NA&gt;
+[1911 rows x 6 columns]</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
@@ -1356,12 +1446,12 @@
 3          3       3         my         my         =            &lt;NA&gt;
 4          4       4       name       name         =            &lt;NA&gt;
 ...      ...     ...        ...        ...       ...             ...
-1898    1873    1703      thank      thank         =            &lt;NA&gt;
-1899    1874    1704        you        you         =            &lt;NA&gt;
-1900    1875    1705       very       very         =            &lt;NA&gt;
-1901    1876    1706       much       much         =            &lt;NA&gt;
-1902    1877    1707     doctor     doctor         =            &lt;NA&gt;
-[1903 rows x 6 columns]</t>
+1897    1873    1703      thank      thank         =            &lt;NA&gt;
+1898    1874    1704        you        you         =            &lt;NA&gt;
+1899    1875    1705       very       very         =            &lt;NA&gt;
+1900    1876    1706       much       much         =            &lt;NA&gt;
+1901    1877    1707     doctor     doctor         =            &lt;NA&gt;
+[1902 rows x 6 columns]</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
@@ -1386,17 +1476,47 @@
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may [DEL:i] help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about about four days now and i have been abdominal pain two alongside so that [DEL:is] those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the [SUB:stool-&gt;tool] is [SUB:it-&gt;he] watery is he semi solid or it is [DEL:in] normal form well from formed stools it is very watery very watery very watery yes okay all right so like how many episodes of you said you have been still stolen for over four days right yes and how many episodes do you [DEL:do] you have [SUB:per-&gt;for] day of stooling my about six about six to seven episodes actually about around that of passage of what watery [SUB:stool-&gt;to] yes yes yes yes doctor okay okay so is the stool containing [SUB:mucus-&gt;mucous] is it mucoid no no no there is no [SUB:mucus-&gt;mucous] no [SUB:mucus-&gt;mucous] in it was there any blood in it no blood at all there [SUB:is-&gt;was] no blood in it okay did you change did you eat [DEL:a] from a new restaurant or did you did you eat something different ermactually a few days ago [DEL:i] like just before it started i actually had a take [DEL:out] in a restaurant with my family which was all [SUB:of-&gt;heads] [DEL:us] ate and one of my child actually [SUB:vomited-&gt;vomitedited] but the vomiting stopped and [SUB:he-&gt;it] feels good now so it is just me right now with the complaints i have of the of the loose [SUB:stool-&gt;yes] are you also [DEL:vomiting] yes ii vomited about two two episodes about two times yes what what what what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomit] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know [SUB:it-&gt;i] just i just [SUB:vomited-&gt;wanted] that [SUB:is-&gt;tell] [SUB:all-&gt;so] [SUB:i-&gt;like] i cannot really remember how you came out to be honest okay was there any is there any abdominal distension distension like [DEL:a] swelling swelling yeah was there swelling in your stomach no just the muscle [INS:is] there any abdominal [INS:distension] [INS:distension] like [INS:swelling] [INS:swelling] yeah was there [INS:swelling] [INS:in] your [INS:stomach] no just [INS:abdominal] pain the pain is just at my the lower part of my stomach okuhm [SUB:all-&gt;alright] right [DEL:all] right thank you so you said your son also ate ate the same the same food that you bought and he is now vomiting how is he feeling now he feels he is okay [DEL:he] after the episode of vomiting he [DEL:he] got [DEL:he] got well and he is okay how is your appetite like my appetite is [DEL:is] here and there know it is not really good like [SUB:so-&gt;before] now let [DEL:us] okay okay so let us talk about let [DEL:us] talk about your the pain you were having so can you describe the pain for me what is the what [DEL:is] the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it [INS:i] will describe [INS:it] [INS:as] [INS:a] [INS:cramp] [INS:pain] like the yeah i feel [INS:do] you want [INS:me] [INS:to] show [INS:so] that [INS:is] [INS:a] kind [INS:of] [INS:pain] [INS:is] [INS:it] [INS:i] will describe it like like has a cramp pain like [INS:it] the [SUB:pain-&gt;been] [SUB:i-&gt;a] feel during menstruation so that is the kind of pain like that is the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just just the lower part [DEL:of] my like moving [DEL:to] the back just the lower part [DEL:it] does not move [DEL:to] your back no no not [DEL:at] [DEL:all] it stays in the same space yes yes okay okay so what what do you think makes this pain worse well maybe if i if i do not eat i do not know if i do not eat here maybe [INS:do] not know if [INS:i] [INS:do] not eat yeah maybe something around that yeah but i do not feel like if it just comes and goes i do not feel like there [INS:is] anything that makes you [SUB:it-&gt;to] [SUB:worse-&gt;want] [SUB:per-&gt;to] [SUB:se-&gt;say] but i will say maybe if i do not eat yes okay what what what relieves the pain [INS:i] [INS:am] not nothing i do not know i [SUB:do-&gt;did] not know when you anything that [INS:it] would reduce the [SUB:pain-&gt;that] it just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will give the pain like five [INS:out] [SUB:or-&gt;of] ten five five over ten yes no problem so let us yeah take some history [DEL:do] you have are you hypertensive no i am not are you diabetic no i am not [DEL:do] you are you a known [SUB:peptic-&gt;because] also patient no no are you lactose intolerant no the only the only ailment [SUB:i-&gt;be] [DEL:am] being treated for [SUB:i-&gt;you] [SUB:am-&gt;a] being treated for [SUB:is-&gt;no] [SUB:asthma-&gt;are] [SUB:i-&gt;you] [SUB:am-&gt;lactose] [SUB:a-&gt;intolerant] known [SUB:asthmatic-&gt;the] and and i have [SUB:am-&gt;been] [SUB:on-&gt;treated] [SUB:i-&gt;for] use [SUB:inhalers-&gt;asthmatic] and [INS:i] how many how many exacerbations do you have in a year about [DEL:in] the last one just one okay [INS:one] okay that is good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not [DEL:i] do not [DEL:do] any of those i do not [DEL:at] [DEL:all] and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i [DEL:i] feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my i feel sometimes my mouth is kind of dry [SUB:to-&gt;too] kind of okay okay okay no problem so do you asides the asthma do you have any other ailments that you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no [DEL:at] [DEL:all] [DEL:i] [DEL:do] not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [DEL:vomiting] was there any any of your family members that also had the same symptoms no no no no no other just me just [DEL:me] and my son yes okay no [DEL:problem] okay [DEL:do] you i am just going to ask some questions just to rule [DEL:out] every other thing do you [DEL:do] you have headaches no doctor do you have chest pain no doctor [INS:i] [SUB:at-&gt;do] [SUB:all-&gt;not] no do you have an abdominal pain [DEL:oh] do you you have an abdominal pain do you have any change in your bowel habits i do not know how to answer that other [DEL:than] the just the the okay i think [DEL:i] think [DEL:i] think that is fine your urine your your [DEL:urine] has it has [DEL:it] changed in quantity no not at all how about the frequency of urination has it changed no no my urination is fine do you have any [DEL:do] you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and they can also come to have [INS:a] differential diagnosis of what could be the because of your symptoms and [SUB:we-&gt;i] would like to examine you right check your level of hydration check your general physical appearance [DEL:to] see whether you and access your your general health right we also like to do an abdominal examination right to [DEL:to] also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some infection which could have which could have caused the diarrhea you want to say something so what exactly is wrong what exactly is wrong what exactly [DEL:is] the because okay it is just the food i ate right [DEL:so] yeah it looks like you have had a food poisoning however [INS:we] are going [INS:to] have [INS:to] evaluate you and find [INS:out] had [SUB:a-&gt;exactly] [SUB:food-&gt;is] [SUB:poisoning-&gt;the] but however we are going to [INS:do] some very serious tests [INS:i] [INS:am] have to check your [INS:blood] [INS:count] [INS:to] make sure there [INS:is] some [INS:infection] [INS:i] [INS:do] not know [INS:to] evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to know if there is [DEL:a] there [DEL:is] some infection which could be gastroenteritis [SUB:we-&gt;you] want to do your erythrocyte [SUB:sedimentation-&gt;segmentation] rates to know if there is any sign any any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and then [DEL:we] would also want to do a stool culture microscopy and sensitivity and to look out for parasites and some bacteria that could cause you to be having diarrhea we also check your retroviral status to know if you have [INS:a] retroviral disease which could also be a because of [DEL:of] diarrhea although that comes in the chronic chronic setting however [INS:we] would also need to just rule that out do you understand okay doctor okay however we are going to start you on [DEL:on] some some fluids to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your electrolytes electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan [INS:to] rule throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would [DEL:be] could be causing the diarrhea and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get [SUB:on-&gt;out] with [SUB:it-&gt;here] you are fine yeah so that will be fine thank you so you will be attended to [SUB:all-&gt;alright] right thank you very much doctor</t>
+          <t>okay good afternoon my name is doctor shadepo good afternoon my name is ms sharon yes okay so do you have any [PROBLEM: complaints] yes doctor i have been schooling for about about four days now and i have been [PROBLEM: abdominal pain] too alongside so those are my two [PROBLEM: complaints] okay so which one started first the stooling or the [PROBLEM: abdominal pain] the stooling started first about four days ago okay so now like what is the consistency of the of this tool is he watery is he [MEDICINE: semisolid] or it is normal from well from the stores it is very watery very watery very much yes okay all right so like how many episodes of  you said you have been still in for over four days right yes and how many episodes do you you have for the of student anyways about six or six to seven episodes actually about around that of passage of what is to yes yes yes yes doctor okay okay so is the stool containing mucous is it mucoid no no no it is not mucous no [PROBLEM: mucous] in it was there any [PROBLEM: blood] in it no [PROBLEM: blood] at all there was no [PROBLEM: blood] in it okay did from a new restaurant or did you eat something different actually a few days ago just before it started i had a takeout in a restaurant with my family which was all heads and one of my children actually [PROBLEM: vomitedited] but the [PROBLEM: vomiting] stopped and it feels good now so it is just me right now with the [PROBLEM: complaints] i have of the of the loose yes i i [PROBLEM: vomited] about two episodes but two times yes yes what was inside the [PROBLEM: vomit] what was the components of the [PROBLEM: vomit] was it what you ate or was it [PROBLEM: greenish] or was there [PROBLEM: blood] in it no there was no [PROBLEM: blood] it was just the contents of what i ate was the [PROBLEM: vomiting] was it projectile so what do you mean by projector  when it comes with force when it comes with force well i really do not know i just i just wanted to tell so like i cannot really remember how it came out to be honest okay was there any is there any [PROBLEM: abdominal distension] distension like [PROBLEM: swelling] [PROBLEM: swelling] yeah was there [PROBLEM: swelling] in your [ANATOMICAL_STRUCTURE: stomach] no just the [ANATOMICAL_STRUCTURE: muscle] is there any [PROBLEM: abdominal distension] distension like [PROBLEM: swelling] [PROBLEM: swelling] yeah was there [PROBLEM: swelling] in your [ANATOMICAL_STRUCTURE: stomach] no just [PROBLEM: abdominal pain] the [PROBLEM: pain] is just at the lower part of my [ANATOMICAL_STRUCTURE: stomach] okay alright alright thank you so you said your son also ate the same food that you bought and he is now [PROBLEM: vomiting] how is he feeling now he feels he is okay after the episode of [PROBLEM: vomiting] he got well and he is okay how is your [BODY_FUNCTION: appetite] like my [BODY_FUNCTION: appetite] is here and there no it is not really good like before okay so let us talk about the [PROBLEM: pain] you were having so can you describe the [PROBLEM: pain] for me what is the nature of the [PROBLEM: pain] is it a [SEVERITY: sharp] [PROBLEM: pain] or a [PROBLEM: pain] that holds you and needs you what kind of [PROBLEM: pain] is it i will describe it as a [PROBLEM: cramp] [PROBLEM: pain] like the [PROBLEM: pain] i feel do you want me to show so that is a kind of [PROBLEM: pain] is it i will describe it like like as a [PROBLEM: cramp] [PROBLEM: pain] like it is been a few during menstruation so that is the kind of [PROBLEM: pain] like that is the way i can describe it and where is this [PROBLEM: pain] located in your [ANATOMICAL_STRUCTURE: abdomen] the lower part the lower part does this [PROBLEM: pain] does it move to another part of your [ANATOMICAL_STRUCTURE: body] where you start feeling it no just [ANATOMICAL_STRUCTURE: back] just go back no it stays in the same space yes yes okay okay so what what do you think makes this [PROBLEM: pain] [SEVERITY: worse] well maybe if i if i do not eat i do not know if i do not eat here maybe do not know if i do not eat yeah maybe something around that yeah but i do not feel like if it just comes and goes i do not feel like there is anything that makes you to want to say but i would say maybe if i do not eat yes okay what relieves the [PROBLEM: pain] i am not saying i do not know i did not know when you said that it would he said that it just comes and goes on this one okay so on a scale of zero to ten let us say zero means that you do not have any [PROBLEM: pain] at all and ten is the worst [PROBLEM: pain] you have felt in your life so what would you give this [PROBLEM: pain] i will give the [PROBLEM: pain] like five out of ten five five over ten yes no [PROBLEM: problem] so let us take some history are you [PROBLEM: hypertensive] no i am not are you [PROBLEM: diabetic] no i am not are you a [PROBLEM: nonpeptic] because a patient no are you [MEDICINE: lactose] intolerant no i do not like to be treated are you a [PROBLEM: nonpeptic ulcer] patient no are you [MEDICINE: lactose] intolerant no the only ailment i have been treated for is [PROBLEM: asthmatic] and i use [MEDICINE: inhalers] how many exhibitions do you have in a year last one just one okay one okay that is good have you had any previous history of [PROCEDURE: blood transfusion] any history of [PROCEDURE: surgeries] no none at all do you drink [SUBSTANCE_ABUSE: alcohol] or do you [SUBSTANCE_ABUSE: smoke] no i do not do any of those i do not and since you have been feeling these [PROBLEM: symptoms] that you are having has it progressively worsened yeah i feel so so that is why i actually came to the hospital yesterday to see the doctor and probably know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your [ANATOMICAL_STRUCTURE: body] is dry has your urine reduced no not at all no no do you feel [PROBLEM: weak] yeah i feel kind of [PROBLEM: weak] yeah when i feel something my [ANATOMICAL_STRUCTURE: mouth] is kind of [PROBLEM: dry] too kind of okay okay no [PROBLEM: problem] so do you aside the [PROBLEM: asthma] do you have any other ailments that you think the doctor should know about no not at all at all i have no other medical condition do you have any [PROBLEM: drug allergies] no i do not react to any [SUBSTANCE_ABUSE: drugs] at all are you married yes i am married with two kids do you live with your husband yes i do are your kids living with you yes what did you say doctor and your kids live with you as well yes they are so aside your son or your child who are the [PROBLEM: vomitting] was there any of your family members that also had the same [PROBLEM: symptoms] no no no no dad just me and my son yes okay okay i am just going to ask some questions just to realize every other thing do you have [PROBLEM: headaches] no do you have [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] no doctor i do not know do you have an [PROBLEM: abdominal pain] do you have an [PROBLEM: abdominal pain] do you have any change in your bowel habits i do not know how to answer that i think that is fine your [LABORATORY_DATA: urine] has it [LAB_RESULT: changed] in quantity no not at all how about the [PROBLEM: frequency of urination] has it changed no no [BODY_FUNCTION: urination] is fine do you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] no all right no [PROBLEM: problem] so thank you for answering my questions those questions are basically there so that we can pinpoint where there is a [PROBLEM: problem] and you can also come to have a differential diagnosis of what could be the because of your [PROBLEM: symptoms] and i would like to examine you check your level of [PROCEDURE: hydration] check your general physical appearance see whether you can access your general health we also like to do an [PROCEDURE: abdominal examination] right to also give us more information on the [PROBLEM: abdominal pain] you are having if it could lead us to what is causing the [PROBLEM: symptoms] you are having the [PROBLEM: abdominal pain] and the stooling do you understand yes although it seems like what you ate the restaurants you got food from they must have been where you got some [PROBLEM: infection] it could have caused the [PROBLEM: diarrhea] you want to say something so what exactly is drunk what exactly is drunk it is just the food i ate right yeah it looks like you have had a [PROBLEM: food poisoning] however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very serious tests i am going to check your [LABORATORY_DATA: blood count] to make sure there is some [PROBLEM: infection] i do not know to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your [LABORATORY_DATA: blood count] to make this there is some [PROBLEM: infection] which could be [PROBLEM: gastroenteritis] you want to do your  [LABORATORY_DATA: erythrocyte segmentation rate] to know if there is any any type of kind of [PROBLEM: inflammatory disorder] that could cause [PROBLEM: diarrhea] like [PROBLEM: inflammatory disease] right and they would also want to do a [LABORATORY_DATA: stool culture microscopy] and sensitivity to look out for [LABORATORY_DATA: parasites] and some bacteria that could cause you to be having [PROBLEM: diarrhea] we also check your retroviral status to know if you have a [PROBLEM: retroviral disease] which could also be a because of [PROBLEM: diarrhea] although that comes in a chronic setting however we would also need to just rule that out do you understand okay doctor okay however we are going to [MED_STATUS: start] you on some [MEDICINE: fluids] to give you some strength and restore your [LABORATORY_DATA: hydration level] because you have been using some fluid from this tooling and the [PROBLEM: vomiting] we also check your [LABORATORY_DATA: electrolytes] [LABORATORY_DATA: electrolytes] to know what your [LABORATORY_DATA: electrolyte] picture looks like and the ones that will be needed to be that will need to be corrected do you understand and also lastly we also want to do an [PROCEDURE: abdominal scan] to rule out any [PROBLEM: structural or functional problems] that could be in the [ANATOMICAL_STRUCTURE: abdomen] which could be causing the [PROBLEM: diarrhea] and the [PROBLEM: abdominal pain] do you understand yes thank you doctor thank you very much do you have any more questions for me no i am fine i am fine i am good let us just get out of here so i can be fine thank you so you will be attended to alright thank you very much</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may [DEL:i] help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and [SUB:i-&gt;having] have been abdominal pain two alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is [SUB:it-&gt;he] watery is he semi solid or [DEL:it] is [SUB:in-&gt;it] normal form well formed stools it is very watery very watery very watery yes okay [DEL:all] right so like how many episodes of you said you have been stolen for over four days right yes and how many episodes do you do you have per day of stooling my about six about six to seven episodes actually about around that number yes of passage of the water watery [SUB:stool-&gt;tube] yes yes yes doctor okay okay so is this [INS:is] the [SUB:stool-&gt;still] containing mucus is it mucoid no no there is no mucus no [DEL:mucus] in it was there any blood in it no blood at all there is no blood in it okay did you change did you eat [DEL:a] from a new restaurant or did you did you eat something different ermactually a few days ago [DEL:i] like just before [SUB:it-&gt;you] started i actually had [SUB:a-&gt;the] take out in a restaurant with my family which all [SUB:of-&gt;was] [SUB:us-&gt;it] ate and [SUB:one-&gt;all] of my child actually vomited but the vomiting stopped and [SUB:he-&gt;it] feels good now so it is just [DEL:me] right now with the [SUB:complaints-&gt;complaint] i have of the of the loose [SUB:stool-&gt;so] are you also vomiting yes [INS:i] [INS:i] ii vomited about two two episodes about two times yes what what what what was inside the vomit what was the con components [DEL:of] the [DEL:vomitus] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know [SUB:it-&gt;i] just i just want [INS:to] tell [SUB:vomited-&gt;you] that is [SUB:all-&gt;the] [SUB:i-&gt;line] i cannot really remember how you came out to be honest okay was there any is there any abdominal [SUB:distension-&gt;distention] [SUB:distension-&gt;distention] like a swelling swelling yeah was there swelling in your stomach no just the abdominal pain the pain is just at my the lower part of my stomach okuhm [SUB:all-&gt;alright] right [DEL:all] right thank you so you said your son also ate ate the same the same food that you bought and [DEL:he] is now vomiting how is he feeling now [SUB:he-&gt;it] feels [SUB:he-&gt;it] is okay [DEL:he] after the episode [DEL:of] [DEL:vomiting] he [DEL:he] got he got well and [SUB:he-&gt;it] is okay how is your appetite like my appetite is [SUB:is-&gt;yeah] here and there know it is not really good like so now this let [SUB:us-&gt;before] okay okay so let us talk about let us talk about your the pain you were having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it yeah i will describe it like like has a [SUB:cramp-&gt;camp] pain like the pain i feel during menstruation so that is the kind of pain like that [DEL:is] the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to any another part of your body when you start feeling it no just just the lower part of my like moving [DEL:to] the [DEL:back] just the lower part [DEL:it] does not move [DEL:to] your [DEL:back] no no not [DEL:at] [DEL:all] [DEL:it] stays [DEL:in] the same space yes yes okay okay so what what do you think makes this [SUB:pain-&gt;play] worse well maybe if i if [DEL:i] do not eat i do not know if [DEL:i] [DEL:do] not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse [SUB:per-&gt;i] [SUB:se-&gt;say] but i will say maybe if i do not eat yes okay what what what relieves the pain not nothing i do not know i do not know anything that reduce the [DEL:pain] [DEL:it] just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i would will the pain like five [INS:out] [SUB:or-&gt;of] ten five [INS:out] [INS:of] ten yes no problem [DEL:so] let us yeah take some history do you have are you hypertensive no i am not are you diabetic no i am not do you are you a known [SUB:peptic-&gt;ulcer] also patient no no are you lactose intolerant no the only the only ailment i [SUB:am-&gt;will] being treated for [INS:is] [INS:asthma] i [SUB:am-&gt;have] being treated for is asthma i [SUB:am-&gt;have] [SUB:a-&gt;nonasthmatic] known [DEL:asthmatic] and and i am on i use inhalers and how many recently how many exacerbations do you have in a year how about [DEL:in] the last one just one okay okay that [SUB:is-&gt;was] good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those [DEL:i] [DEL:do] not [DEL:at] [DEL:all] and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i [DEL:i] feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your [SUB:body-&gt;bodys] [DEL:is] dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my [DEL:i] feel sometimes my mouth is kind of dry to kind of okay okay okay no problem so do you asides the asthma do you have any other ailments that you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no [DEL:at] [DEL:all] [DEL:i] [DEL:do] not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [INS:vomit] [SUB:vomiting-&gt;symptoms] was there any any of your family members that also had the same symptoms no no no no no other just me just [DEL:me] and my son yes okay no problem okay do you i am just going to ask some questions just to rule out every other thing do you [DEL:do] you have headaches no doctor do you have chest pain [INS:i] no doctor [SUB:at-&gt;i] [SUB:all-&gt;thought] no do you have an abdominal pain [DEL:oh] do you you have an abdominal pain [DEL:do] you have any change in your bowel habits i do not know how to answer that other [DEL:than] the just the the okay i think [DEL:i] think [DEL:i] think that is fine your urine your your urine has it has [DEL:it] changed in quantity no not at all how about the frequency of urination has it changed no no my [DEL:urination] [DEL:is] fine do you have any [DEL:do] you have any bone pain no [DEL:all] right no [DEL:problem] so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and they can also come to have differential diagnosis of what could be the because of your symptoms and [SUB:we-&gt;they] would like to examine you right check your level of hydration check your general physical appearance to see whether you you and access your your general health right we also like to do an abdominal examination right to [DEL:to] also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes yes although although it seems like what you ate the restaurants you got food from there must have been where you got some [INS:so] infection which could have which could have caused the [SUB:diarrhea-&gt;diarrhoea] you want to say something yeah so what exactly is wrong what exactly is wrong what exactly is the because [INS:it] okay it is just the food [DEL:i] ate right [DEL:so] yeah [DEL:it] looks like you have had [DEL:a] [DEL:food] poisoning had [SUB:a-&gt;the] food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to know if there is [DEL:a] there [DEL:is] some infection which could be [SUB:gastroenteritis-&gt;gastritis] we want to do your erythrocyte sedimentation rates to know if there is any sign any any type [DEL:of] kind of inflammatory disorder that could cause [SUB:diarrhea-&gt;diarrhoea] like inflammatory bowel disease right and then [DEL:we] would also want to do [SUB:a-&gt;is] [SUB:stool-&gt;to] culture microscopy and sensitivity and to look out for parasites and some bacteria that could cause you to be having [SUB:diarrhea-&gt;diarrhoea] [SUB:we-&gt;and] also check your retroviral status to know if you have [SUB:retroviral-&gt;viral] disease which could also be a because of of diarrhoea [SUB:diarrhea-&gt;or] although that comes in the chronic [INS:a] chronic setting however [INS:we] would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some fluids to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your electrolytes electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan [INS:to] rule throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would [DEL:be] could be causing the [SUB:diarrhea-&gt;diarrhoea] and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine yeah so that will be fine thank you so you will [SUB:be-&gt;been] attended to [SUB:all-&gt;alright] right thank you very much doctor</t>
+          <t>okay good afternoon my name is doctor [MEDICINE: shadekum] good afternoon my name is miss sharon yes okay so do you have any [PROBLEM: complaints] yes doctor i have been straining for about four days now and having [PROBLEM: abdominal pain] alongside so that is just my two [PROBLEM: complaints] okay okay so which one started first the stooling or the [PROBLEM: abdominal pain] yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is he watery is he semi solid or is it normal form well formed it is very watery very watery so like how many episodes of  you said you have been stalling for over four days right yes and how many episodes do you do you have per day of stalling about six or six to seven episodes actually about around that number yes of passage of the [MEDICAL_DEVICE: water riser tube] yes yes yes doctor okay okay so   is this is it still containing mucus is it [MEDICINE: mucoid] no no there is no [PROBLEM: mucus] in it was there any [PROBLEM: blood] in it no [PROBLEM: blood] at all there is no [PROBLEM: blood] in it okay did you change did you eat from a new restaurant or did you did you eat something different actually a few days ago just before you started i actually had the take out in a restaurant with my family which all was it and  all of my child actually [PROBLEM: vomited] but the [PROBLEM: vomiting] stopped and it feels good now so it is just right now with the [PROBLEM: complaint] i have of the of the loose so are you also [PROBLEM: vomiting] yes i i have [PROBLEM: vomited] about two  two episodes about two times yes well what what was inside the [PROBLEM: vomit] what was the con  components was it what you ate or was it [PROBLEM: greenish] or was there [PROBLEM: blood] in it no there was no [PROBLEM: blood] it was just the contents of what i ate was the [PROBLEM: vomiting] was it projectile so what do you mean by projectile when it comes with force when it comes with force well i really do not know i just i just want to tell you that is the line i cannot really remember how it came out to be honest is there any is there any [PROBLEM: abdominal distention] [PROBLEM: distention] like a [PROBLEM: swelling] [PROBLEM: swelling] yeah is there [PROBLEM: swelling] in your [ANATOMICAL_STRUCTURE: stomach] no just the [PROBLEM: abdominal pain] the [PROBLEM: pain] is just at my lower part of my [ANATOMICAL_STRUCTURE: stomach] okay alright alright thank you so you said your son also ate ate the same the same food that you bought and is now [PROBLEM: vomiting] how is he feeling now it feels it is okay after the he got he got well and it is okay how is your [BODY_FUNCTION: appetite] like my [BODY_FUNCTION: appetite] is yeah there no it is not really good like so now this like before okay okay so let us talk about let us talk about your the [PROBLEM: pain] we are having so can you describe the [PROBLEM: pain] for me what is the what is the nature of the [PROBLEM: pain] is it a [SEVERITY: sharp] [PROBLEM: pain] or a [PROBLEM: pain] that holds you and needs what kind of [PROBLEM: pain] is it i would describe it as a camp [PROBLEM: pain] like a [PROBLEM: pain] i feel during menstruation so that is the kind of [PROBLEM: pain] i can describe it and where is this [PROBLEM: pain] located in your [ANATOMICAL_STRUCTURE: abdomen] the lower parts the lower parts does this [PROBLEM: pain] does it move to any other part of your [ANATOMICAL_STRUCTURE: body] when you start feeling it no just the lower part of my [ANATOMICAL_STRUCTURE: abdomen] the same space yes yes okay okay so what do you think makes this play worse well if i do not eat i do not know maybe something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse i say but i was saying if i do not eat yes okay what really how is the [PROBLEM: pain]  not saying i do not know i do not know i just comes and goes on this one okay so on a scale of zero to ten let us say zero means that you do not have any [PROBLEM: pain] at all and ten is the worst [PROBLEM: pain] you felt in your life so what would you give this [PROBLEM: pain] i would give this [PROBLEM: pain] like five out of ten five out of ten no [PROBLEM: problem] let us take some history do you are you [PROBLEM: hypertensive] no i am not are you [PROBLEM: diabetic] no i am not do you are you a [PROBLEM: nonpeptic ulcer] patient no no are you [MEDICINE: lactose] intolerant no the only the only payment i will be treating for is [PROBLEM: asthma] i have been treated for is [PROBLEM: asthma] i have [PROBLEM: nonasthmatic] and i am on i use [MEDICINE: inhalers] and how many recently how many exhibitions do you have in a year how about last one just one okay okay that was good have you had any previous history of [PROCEDURE: blood transfusion] any history of [PROCEDURE: surgeries] no no none at all okay do you drink [SUBSTANCE_ABUSE: alcohol] or do you [SUBSTANCE_ABUSE: smoke] no i do not i do not do any of those and since you have been feeling these [PROBLEM: symptoms] that you are having as it progressively worsened yeah i feel so so that is why i actually came to the hospital just to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your bodys dry has your urine reduced no not at all no no do you feel [PROBLEM: weak] yeah i feel kind of [PROBLEM: weak] yeah yeah my [ANATOMICAL_STRUCTURE: mouth] is kind of [PROBLEM: dry] to kind of okay okay no [PROBLEM: problem] so do you aside the [PROBLEM: asthma] do you have any other ailments that you think the doctor should know about no not at all at all i have no other medical condition do you have any [PROBLEM: drug allergies] no i do not react to any [SUBSTANCE_ABUSE: drugs] at all are you married yes i am married with two kids  yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who are the the [PROBLEM: vomit symptoms] was there any any of your family members that also had the same [PROBLEM: symptoms] no no no that just me and my son yes no [PROBLEM: problem]  okay do you i am just going to ask some questions just to rule out every other thing do you have [PROBLEM: headaches] no do you have [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] i know doctor i thought no do you have an [PROBLEM: abdominal pain] do you have an [PROBLEM: abdominal pain] you have any change in your bowel habits i do not know how to answer that i think that is fine your [LABORATORY_DATA: urine your urine] has it [LAB_RESULT: changed] in quantity no not at all how about the [PROBLEM: frequency of urination] has it changed no no do you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] no so  thank you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a [PROBLEM: problem] and then can also come to have differential diagnosis of what could be the because of your [PROBLEM: symptoms] and they would like to examine you right check your level of [PROCEDURE: hydration] check your  general  physical appearance to see whether you you and access your general health we also like to do an [PROCEDURE: abdominal examination] right to also give us more information on the [PROBLEM: abdominal pain] you are having if it could lead us to what is causing the [PROBLEM: symptoms] you are having the [PROBLEM: abdominal pain] and the the stooling do you understand yes yes although although it seems like what you ate the restaurants you got food from there must have been where you got  some  so [PROBLEM: infection] which could have which could have caused the [PROBLEM: diarrhoea] you want to say something yeah so what exactly is drawn what exactly is wrong what exactly is the because it is it is just the [PROBLEM: food poisoning] by the [PROBLEM: food poisoning] but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some really series of tests i am going to check your [LABORATORY_DATA: blood count] to see if there is some [PROBLEM: infection] be [PROBLEM: gastritis] we want to do your  [LABORATORY_DATA: erythrocyte sedimentation] rate to know if there is any any any type kind of [PROBLEM: inflammatory disorder] that could cause [PROBLEM: diarrhoea] like [PROBLEM: inflammatory bowel disease] right and they would also want to do is to [LABORATORY_DATA: culture microscopy] and sensitivity and to look out for  parasites and some bacteria that could cause you to be having [PROBLEM: diarrhoea] and also check your  retroviral status to know if   your [PROBLEM: abdominal viral disease] which could also be a because of  of [PROBLEM: diarrhoea] or do that comes in a chronic  a chronic  setting however we would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some [MEDICINE: fluids] to  you know give you some strength and restore your [LABORATORY_DATA: hydration level] because you have been losing some fluid from  this tooling and the [PROBLEM: vomiting] we also check your [LABORATORY_DATA: electrolytes] [LABORATORY_DATA: electrolytes] to know what your electrolyte picture looks like and the ones that will be needed to be that will need to be corrected do you understand and also lastly we would also want to check do an [PROCEDURE: abdominal scan] to rule out any [PROBLEM: structural or functional problems] that could be in the [ANATOMICAL_STRUCTURE: abdomen] which could be causing the [PROBLEM: diarrhoea] and then the the [PROBLEM: abdominal pain] do you understand yes thank you doctor thank you very much yes do you have any more questions for me i am fine i am fine i am good let us just get on with it so yeah so that can be fine thank you so you have been attended to alright thank you very much doctor</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may [DEL:i] help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and [SUB:i-&gt;having] have been abdominal pain two alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the [SUB:of-&gt;tool] the [DEL:stool] is [SUB:it-&gt;he] watery is he semi solid or it is [SUB:in-&gt;a] normal form [SUB:well-&gt;wellformed] formed stools it is very watery very watery very watery yes okay all right so like how many episodes of you said you have been stolen for over four days right yes and how many episodes do you [DEL:do] you have per day of stooling my about six about six to seven episodes actually about around that number yes of passage of watery stool yes yes yes doctor okay okay so is the [SUB:stool-&gt;tool] containing mucus is it mucoid no no no there is no mucus no mucus [DEL:in] [DEL:it] was there any blood in it no blood at all there is no blood in it okay did you change did you eat [DEL:a] from a new restaurant or did you did you eat something different ermactually a few days ago i like just before [SUB:it-&gt;i] started i actually had a take [DEL:out] in a restaurant with my family which all of us ate and one of my child actually vomited but the vomiting stopped and [SUB:he-&gt;it] feels good now so it is just [DEL:me] right now with the complaints i have of the [DEL:of] the loose [SUB:stool-&gt;yes] are you also [SUB:vomiting-&gt;said] yes ii [DEL:vomited] about two two episodes about two times yes what what what what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomiters] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know [DEL:it] just i just [SUB:vomited-&gt;wanted] that [SUB:is-&gt;ask] [DEL:all] i [DEL:i] cannot really remember how you came out to be honest okay was there any is there any abdominal distension distension like a swelling swelling yeah was there swelling in your stomach no just the abdominal pain the pain is just at my the lower part of my stomach okuhm all right all right thank you so you said your son also ate ate the same the same [DEL:food] that you bought and he is now vomiting how is he feeling now he feels he is okay [DEL:he] after the episode of vomiting he [DEL:he] got [DEL:he] got well and [SUB:he-&gt;it] is okay okay how is your appetite like my appetite is [DEL:is] here and there know it is not really good like so now let us okay okay so let us talk about let us talk about your the pain you were having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it yeah i will describe it like like has a cramp pain like the pain i feel during my [SUB:menstruation-&gt;session] so that is the kind of pain like that is the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just just the lower part [DEL:of] my like moving [DEL:to] the back just the lower part [DEL:it] does not move [DEL:to] your [DEL:back] no no not [DEL:at] [DEL:all] [DEL:it] stays [DEL:in] the same space yes yes okay okay so what what do you think makes this pain worse [DEL:well] maybe if i if [DEL:i] do not eat i do not know if [SUB:i-&gt;is] [SUB:do-&gt;easier] not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it [SUB:worse-&gt;well] per se but i will say maybe if i do not eat yes okay what what what relieves the pain nothing i do not know i do not know anything that reduce the [DEL:pain] [DEL:it] just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will give the pain like five or ten five over ten yes no problem so let us yeah take some history [DEL:do] you have are you hypertensive no i am not are you diabetic no i am not do you are you a known [SUB:peptic-&gt;ulcer] also patient no no are you lactose [INS:in] intolerant no the only the only ailment i am being treated for i [SUB:am-&gt;have] being treated for is asthma [SUB:i-&gt;my] [SUB:am-&gt;nonasmatic] [DEL:a] known [DEL:asthmatic] and and i am [SUB:on-&gt;only] i use [SUB:inhalers-&gt;als] and how many how many exacerbations do you have in a year about [DEL:in] the last one just one okay okay that is good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those i do not have [INS:it] at all and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i [DEL:i] feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my i feel sometimes my mouth is kind of dry to kind [SUB:of-&gt;up] okay okay okay no problem so do you have asides the asthma do you have any other ailments that you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no at all i do not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the vomiting was there any any of your family members that also had the same symptoms no no no no no that other just me and just me and my son yes okay no [DEL:problem] okay do you i am just going to ask some questions just to rule [DEL:out] every other thing do you [DEL:do] you have headaches no not [INS:at] doctor do you have chest pain no doctor at all no do you have an abdominal pain [DEL:oh] do you you have an abdominal pain do you have any change in your [SUB:bowel-&gt;dowel] habits yeah i do not know how to answer that other than the just the the okay i think [DEL:i] think [DEL:i] think that is fine your urine your your [DEL:urine] has it has [DEL:it] changed in quantity no not at all how about the frequency of urination has it changed no no my [SUB:urination-&gt;initial] [DEL:is] fine [DEL:do] you have any [DEL:do] you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and then they can also come to have differential diagnosis of what could be the because of your symptoms and then we would like to examine you right check your level of [SUB:hydration-&gt;vibration] check your general physical appearance to see whether you and access your your general health right we also like to do an abdominal examination right [SUB:to-&gt;so] [DEL:to] also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some infection which could have which could have caused the [DEL:diarrhea] you want to say something so what exactly is wrong what exactly is wrong what exactly is the because okay it is just the food i ate right [DEL:so] yeah it looks like you have had a food poisoning had [SUB:a-&gt;the] food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series [DEL:of] tests i am going to check your blood count to know if there is [DEL:a] there [DEL:is] some infection which could be [INS:a] gastroenteritis we want to do your erythrocyte sedimentation rates to know if there is any sign any any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and then we would also want to do a stool culture microscopy and sensitivity and to look out for parasites and some [SUB:bacteria-&gt;bacterias] that could cause you to be having diarrhea we also check your retroviral status to know if you have [INS:a] retroviral disease which could also be a because of [DEL:of] diarrhea although that comes in the chronic chronic setting however [INS:i] would also need to just rule that out do you understand okay doctor okay however we are going to start you on [DEL:on] some some [DEL:fluids] to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your [SUB:electrolytes-&gt;electrolyte] electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan [INS:to] rule throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would [DEL:be] could be causing the diarrhea and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine yeah [DEL:so] that will [DEL:be] fine thank you so you will be attended to all right thank you very much doctor</t>
+          <t>okay good afternoon my name is doctor shadiko yeah good afternoon yeah good afternoon my name is miss sharon yes okay so do you have any [PROBLEM: complaints] yes doctor i have been stooling for about four days now and having [PROBLEM: abdominal pain] too alongside so that is those are my two [PROBLEM: complaints] okay okay so which one started first the stooling or the [PROBLEM: abdominal pain] yeah the stooling started first about four days ago okay so now like what is the consistency of this tool is he watery is he [MEDICINE: semisolid] or it is a normal form wellformed stool it is very watery very watery very watchful yes okay all right so like how many episodes of you said you have been stooling for about four days right yes and how many episodes do you have per day of stooling about six about six to seven episodes actually about around that number yes of passage of watery stool yes yes yes doctor okay okay so is this tool containing mucus is it [MEDICINE: mucoid] no no no it is not mucus no mucus was there any [PROBLEM: blood] in it no [PROBLEM: blood] at all there is no [PROBLEM: blood] in it okay did you change did you eat from a new restaurant or did you eat something different actually a few days ago i like just before i started i actually had a takeout in a restaurant with my family which all of us ate and one of my child actually [PROBLEM: vomited] but the [PROBLEM: vomiting] stopped and it feels good now so it is just right now with the [PROBLEM: complaints] i have of the loose yes i have only said about two episodes but two times yes well what was inside the [PROBLEM: vomit] what was the components of the [PROBLEM: vomiters] was it what you ate or was it [PROBLEM: greenish] or was there [PROBLEM: blood] in it no there was no [PROBLEM: blood] it was just the content of what i ate was the [PROBLEM: vomiting] was it projectile so what do you mean by projectile when it comes with force when it comes to force well i really do not know i just wanted to ask i cannot really remember how it came out to be honest okay was there any is there any [PROBLEM: abdominal distension] distension like a [PROBLEM: swelling] [PROBLEM: swelling] yeah was there [PROBLEM: swelling] in your [ANATOMICAL_STRUCTURE: stomach] no just the [PROBLEM: abdominal pain] the [PROBLEM: pain] is just at my lower part of my [ANATOMICAL_STRUCTURE: stomach] okay all right all right thank you so you said your son also bought and he is now [PROBLEM: vomiting] how is he feeling now he feels he is okay after the appearance of [PROBLEM: vomiting] he got well and it is okay okay how is your [BODY_FUNCTION: appetite] like my [BODY_FUNCTION: appetite] is here yeah no it is not really good so now let us okay okay so let us talk about let us talk about your the [PROBLEM: pain] you are having so can you describe the [PROBLEM: pain] for me what is the what is the nature of the [PROBLEM: pain] is it a [SEVERITY: sharp] [PROBLEM: pain] or a [PROBLEM: pain] that holds you and leaves you what kind of [PROBLEM: pain] is it i will describe it like like as a cramp [PROBLEM: pain] like the [PROBLEM: pain] i feel during my session so that is the kind of [PROBLEM: pain] like that is the way i can describe it and where is this [PROBLEM: pain] located in your [ANATOMICAL_STRUCTURE: abdomen] the lower part the lower part does this [PROBLEM: pain] does it move to another part of your [ANATOMICAL_STRUCTURE: body] when you start feeling it no just back just the lower part no is this the same space yes yes okay so what do you think makes this [PROBLEM: pain] [SEVERITY: worse] maybe if i do not eat i do not know it is easier maybe something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it well per se but i would say maybe if i do not eat yes okay what relieves the [PROBLEM: pain] nothing i do not know i do not know if that just comes and goes on this one okay so on a scale of zero to ten let us say zero means that you do not have any [PROBLEM: pain] at all and ten is the worst [PROBLEM: pain] you felt in your life so what would you give this [PROBLEM: pain] i will give the [PROBLEM: pain] like five or ten five over ten okay no [PROBLEM: problem] so let us take some history are you [PROBLEM: hypertensive] no i am not are you [PROBLEM: diabetic] no i am not do you are you a [PROBLEM: nonpeptic ulcer] patient no no are you [MEDICINE: lactose] in tolerant no the only aim i am treating for i have been treated for is [PROBLEM: asthma] my [PROBLEM: nonasmatic] and i am only i use als how many how many examples do you have in a year about last one just one okay okay that is good have you had any previous history of [PROCEDURE: blood transfusion] any history of [PROCEDURE: surgeries] no no not at all okay do you drink [SUBSTANCE_ABUSE: alcohol] or do you [SUBSTANCE_ABUSE: smoke] no i do not i do not do any of those i do not have it at all and since you have been feeling these [PROBLEM: symptoms] that you are having has it progressively worsened yeah i feel so so that is why i actually came to the hospital just today to see the doctor and probably know what is wrong with me and take care of it basically have you been feeling very testy have you been feeling like your [ANATOMICAL_STRUCTURE: body] is dry has your urine reduced no not at all no no do you feel [PROBLEM: weak] yeah i feel kind of [PROBLEM: weak] yeah yeah i feel sometimes my [ANATOMICAL_STRUCTURE: mouth] is kind of dry to cut up okay okay okay no [PROBLEM: problem] so do you have asides the [PROBLEM: asthma] do you have any other ailments that you think the doctor should know about no not at all at all i have no other medical condition do you have any [PROBLEM: drug allergies] no i do not react at all i do not react to any [MEDICINE: drugs] at all are you married yes i am married you took it yes okay and you live with your husband yes yes i do and your kids live with you yeah what did you say doctor are your kids live with you as well yes they are so asides your son or your child who are the [PROBLEM: vomiting] was there any of your family members that also had the same [PROBLEM: symptoms] no no no no no that is just me and just me and my son yes okay do you i am just going to ask some questions just to raise every other thing do you have [PROBLEM: headaches] no not at all do you have [ANATOMICAL_STRUCTURE: chest] [PROBLEM: pain] no doctor at all no do you have an [PROBLEM: abdominal pain] do you have an [PROBLEM: abdominal pain] do you have any change in your dowel habits yeah i do not know how to answer that other than the okay i think that is fine your [LABORATORY_DATA: urine] has it [LAB_RESULT: changed] in quantity no not at all how about the [PROBLEM: frequency of urination] has it changed no no my initial you have any [ANATOMICAL_STRUCTURE: bone] [PROBLEM: pain] no all right no [PROBLEM: problem] so thank you for answering my questions those questions are basically there so that we can pinpoint where there is a [PROBLEM: problem] and then we can also come to have differential diagnosis of what could be the because of your [PROBLEM: symptoms] and then we would like to examine you right check your level of vibration check your general physical appearance to see whether you can access your general health we also like to do an [PROCEDURE: abdominal examination] right so also give us more information on the [PROBLEM: abdominal pain] you are having if you could lead us to what is causing the [PROBLEM: symptoms] you have in the [PROBLEM: abdominal pain] and the stooling do you understand yes although although it seems like what you ate the restaurant you got food from there must have been where you got some [PROBLEM: infection] you want to say something so what exactly is drug what exactly is wrong what exactly is the because okay it is just the food i had right yeah it looks like you have had a [PROBLEM: food poisoning] or the [PROBLEM: food poisoning] but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very serious tests i am going to check your [LABORATORY_DATA: blood count] to make there is some [PROBLEM: infection] which could be a [PROBLEM: gastroenteritis] we want to do your [LABORATORY_DATA: erythrocyte sedimentation rate] to know if there is any type of kind of [PROBLEM: inflammatory disorder] that could cause [PROBLEM: diarrhea] like [PROBLEM: inflammatory disease] right and then we would also want to do a [LABORATORY_DATA: stool culture microscopy] and sensitivity to look out for [LABORATORY_DATA: parasites] and some [LABORATORY_DATA: bacterias] that could cause you to be having [PROBLEM: diarrhea] we also check your retroviral status to know if you have a [PROBLEM: retroviral disease] which could also be a because of [PROBLEM: diarrhea] although that comes in a chronic chronic setting however i would also need to just rule that out do you understand okay doctor okay however we are going to start you on some foods to give you some strength and restore your [LABORATORY_DATA: hydration level] because you have been [PROBLEM: losing some fluid] from the stooling and the [PROBLEM: vomiting] we also check your [LABORATORY_DATA: electrolyte] [LABORATORY_DATA: electrolytes] to know what your [LABORATORY_DATA: electrolyte] picture looks like and the ones that will be needed to be that would need to be corrected do you understand and also lastly we also want to check do an [PROCEDURE: abdominal scan] to rule out any structural or functional [PROBLEM: problems] that could be in the [ANATOMICAL_STRUCTURE: abdomen] which could be causing the [PROBLEM: diarrhea] and the [PROBLEM: abdominal pain] do you understand yes thank you doctor thank you very much yes do you have any more questions for me i am fine i am fine i am good let us just get on with it thank you so you will be attended to all right thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor [DEL:sadeko] [DEL:yeah] [DEL:good] [DEL:afternoon] [DEL:how] [DEL:may] [DEL:i] [DEL:help] [DEL:you] [SUB:yeah-&gt;shadepo] good afternoon my name is [SUB:miss-&gt;ms] sharon yes okay so do you have any complaints yes doctor i have been [SUB:stooling-&gt;schooling] for [INS:about] about four days now and i have been abdominal pain [SUB:two-&gt;too] alongside so [DEL:that] [DEL:is] those are my two complaints [DEL:okay] okay so which one started first the stooling or the abdominal pain [DEL:yeah] the stooling started first about four days ago okay so now like what is the consistency of the of [SUB:the-&gt;this] [SUB:stool-&gt;tool] is [SUB:it-&gt;he] watery is he [DEL:semi] [SUB:solid-&gt;semisolid] or it is [DEL:in] normal [SUB:form-&gt;from] well [INS:from] [SUB:formed-&gt;the] [SUB:stools-&gt;stores] it is very watery very watery very [SUB:watery-&gt;much] yes okay all right so like how many episodes of you said you have been [INS:still] [SUB:stolen-&gt;in] for over four days right yes and how many episodes do you [DEL:do] you have [SUB:per-&gt;for] [SUB:day-&gt;the] of [SUB:stooling-&gt;student] [SUB:my-&gt;anyways] about six [SUB:about-&gt;or] six to seven episodes actually about around that of passage of [INS:what] [INS:is] [SUB:watery-&gt;to] [SUB:stool-&gt;yes] yes yes yes doctor okay okay so is the stool containing [SUB:mucus-&gt;mucous] is it mucoid [INS:no] no no [SUB:there-&gt;it] is [SUB:no-&gt;not] [SUB:mucus-&gt;mucous] no [SUB:mucus-&gt;mucous] in it was there any blood in it no blood at all there [SUB:is-&gt;was] no blood in it okay did [DEL:you] [DEL:change] [DEL:did] [DEL:you] [DEL:eat] [DEL:a] from a new restaurant or [DEL:did] [DEL:you] did you eat something different [SUB:ermactually-&gt;actually] a few days ago [DEL:i] [DEL:like] just before it started i [DEL:actually] had a [DEL:take] [SUB:out-&gt;takeout] in a restaurant with my family which [DEL:all] [SUB:of-&gt;was] [SUB:us-&gt;all] [SUB:ate-&gt;heads] and one of my [SUB:child-&gt;children] actually [SUB:vomited-&gt;vomitedited] but [INS:the] vomiting stopped and [SUB:he-&gt;it] feels good now so it is just me right now with the complaints i have of the of the loose [DEL:stool] [DEL:are] [DEL:you] [DEL:also] [SUB:vomiting-&gt;yes] [SUB:yes-&gt;i] [SUB:ii-&gt;i] vomited about [DEL:two] two episodes [SUB:about-&gt;but] two times yes [DEL:what] [DEL:what] [SUB:what-&gt;yes] what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomit] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the [SUB:content-&gt;contents] of what i ate was the vomiting was it projectile so what do you mean by [SUB:projectile-&gt;projector] [SUB:ermwhen-&gt;when] it comes with force when it comes with force well i really do not know [SUB:it-&gt;i] just i just [SUB:vomited-&gt;wanted] [SUB:that-&gt;to] [SUB:is-&gt;tell] [SUB:all-&gt;so] [SUB:i-&gt;like] i cannot really remember how [SUB:you-&gt;it] came out to be honest okay was there any is there any abdominal distension distension like [DEL:a] swelling swelling yeah was there swelling in your stomach no just the [INS:muscle] [INS:is] [INS:there] [INS:any] [INS:abdominal] [INS:distension] [INS:distension] [INS:like] [INS:swelling] [INS:swelling] [INS:yeah] [INS:was] [INS:there] [INS:swelling] [INS:in] [INS:your] [INS:stomach] [INS:no] [INS:just] abdominal pain the pain is just at [DEL:my] the lower part of my stomach [DEL:okuhm] [DEL:all] [SUB:right-&gt;okay] [SUB:all-&gt;alright] [SUB:right-&gt;alright] thank you so you said your son also ate [DEL:ate] [DEL:the] [DEL:same] the same food that you bought and he is now vomiting how is he feeling now he feels he is okay [DEL:he] after the episode of vomiting [DEL:he] [DEL:he] [DEL:got] he got well and he is okay how is your appetite like my appetite [DEL:is] is here and there [SUB:know-&gt;no] it is not really good like [DEL:so] [DEL:now] [DEL:let] [DEL:us] [SUB:okay-&gt;before] okay so let us talk about [DEL:let] [DEL:us] [DEL:talk] [DEL:about] [DEL:your] the pain you were having so can you describe the pain for me [DEL:what] [DEL:is] [DEL:the] what is the nature of the pain is it a sharp pain or a pain that holds you and [SUB:leaves-&gt;needs] you [SUB:whatwhat-&gt;what] kind of pain is it [INS:i] [INS:will] [INS:describe] [INS:it] [INS:as] [INS:a] [INS:cramp] [INS:pain] [INS:like] [INS:the] [INS:pain] [INS:i] [INS:feel] [INS:do] [INS:you] [INS:want] [INS:me] [INS:to] [INS:show] [INS:so] [INS:that] [INS:is] [INS:a] [INS:kind] [INS:of] [INS:pain] [INS:is] [SUB:yeah-&gt;it] i will describe it like like [SUB:has-&gt;as] a cramp pain like [INS:it] [SUB:the-&gt;is] [SUB:pain-&gt;been] [SUB:i-&gt;a] [SUB:feel-&gt;few] during menstruation so that is the kind of pain like that is the way i can describe it and [DEL:where] where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body [SUB:when-&gt;where] you start feeling it no just [DEL:just] [DEL:the] [DEL:lower] [DEL:part] [DEL:of] [DEL:my] [DEL:like] [DEL:moving] [DEL:to] [DEL:the] back just [DEL:the] [DEL:lower] [DEL:part] [DEL:it] [DEL:does] [DEL:not] [DEL:move] [DEL:to] [SUB:your-&gt;go] back no [DEL:no] [DEL:not] [DEL:at] [DEL:all] it stays in the same space yes yes okay okay so what what do you think makes this pain worse well maybe if i if i do not eat i do not know if i do not eat [INS:here] [INS:maybe] [INS:do] [INS:not] [INS:know] [INS:if] [INS:i] [INS:do] [INS:not] [INS:eat] [INS:yeah] [INS:maybe] something around that yeah but i do not feel like if it just comes and goes i do not feel like [INS:there] [INS:is] anything that makes [INS:you] [SUB:it-&gt;to] [SUB:worse-&gt;want] [SUB:per-&gt;to] [SUB:se-&gt;say] but i [SUB:will-&gt;would] say maybe if i do not eat yes okay [DEL:what] [DEL:what] what relieves the pain [INS:i] [INS:am] [INS:not] [SUB:nothing-&gt;saying] i do not know i [SUB:do-&gt;did] not know [INS:when] [INS:you] [SUB:anything-&gt;said] that [INS:it] [INS:would] [SUB:reduce-&gt;he] [SUB:the-&gt;said] [SUB:pain-&gt;that] it just comes and goes on [SUB:its-&gt;this] one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will [INS:give] the pain like five [INS:out] [SUB:or-&gt;of] ten five [INS:five] [INS:over] ten yes no problem so let us [DEL:yeah] take some history [DEL:do] [DEL:you] [DEL:have] are you hypertensive no i am not are you diabetic no i am not [DEL:do] [DEL:you] are you a [SUB:known-&gt;nonpeptic] [SUB:peptic-&gt;because] [SUB:also-&gt;a] patient [DEL:no] no are you lactose intolerant no [DEL:the] [DEL:only] [SUB:the-&gt;i] [SUB:only-&gt;do] [SUB:ailment-&gt;not] [SUB:i-&gt;like] [SUB:am-&gt;to] [SUB:being-&gt;be] treated [SUB:for-&gt;are] [SUB:i-&gt;you] [SUB:am-&gt;a] [SUB:being-&gt;nonpeptic] [SUB:treated-&gt;ulcer] [SUB:for-&gt;patient] [SUB:is-&gt;no] [SUB:asthma-&gt;are] [SUB:i-&gt;you] [SUB:am-&gt;lactose] [SUB:a-&gt;intolerant] [SUB:known-&gt;no] [SUB:asthmatic-&gt;the] [SUB:and-&gt;only] [SUB:and-&gt;ailment] i [INS:have] [SUB:am-&gt;been] [SUB:on-&gt;treated] [SUB:i-&gt;for] [SUB:use-&gt;is] [SUB:inhalers-&gt;asthmatic] and [INS:i] [SUB:how-&gt;use] [SUB:many-&gt;inhalers] how many [SUB:exacerbations-&gt;exhibitions] do you have in a year [DEL:about] [DEL:in] [DEL:the] last one just one okay [INS:one] okay that is good have you had any previous history of blood transfusion any history of surgeries [DEL:no] no none at all [DEL:okay] do you drink alcohol or do you smoke no [DEL:i] [DEL:do] [DEL:not] i do not do any of those i do not [DEL:at] [DEL:all] and since you have been feeling these symptoms that you are having [DEL:has] has it progressively worsened yeah [DEL:i] i feel so so that is why i actually came to the hospital [DEL:just] [SUB:today-&gt;yesterday] to see the doctor and [SUB:properly-&gt;probably] know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah [DEL:yeah] [DEL:my] [SUB:my-&gt;when] i feel [SUB:sometimes-&gt;something] my mouth is kind of dry [SUB:to-&gt;too] kind of [DEL:okay] okay okay no problem so do you [SUB:asides-&gt;aside] the asthma do you have any other ailments [INS:that] you think the doctor should know about no not at all at all i have [DEL:no] [DEL:other] no other medical condition do you have any drug allergies no [DEL:i] [DEL:do] [DEL:not] [DEL:react] [DEL:no] [DEL:at] [DEL:all] i do not react to any drugs at all [DEL:okay] [DEL:please] are you married yes i am married with two kids [DEL:yes] [DEL:okay] [DEL:and] [SUB:you-&gt;do] you live with your husband [DEL:yes] yes i do [SUB:and-&gt;are] your kids [SUB:live-&gt;living] with you [SUB:yeah-&gt;yes] what did you say doctor and your kids live with you as well yes they are so aside [DEL:your] your son or your child who [DEL:had] [SUB:the-&gt;are] the [SUB:vomiting-&gt;vomitting] was there [DEL:any] any of your family members that also had the same symptoms no no no no [DEL:no] [DEL:other] [DEL:just] [SUB:me-&gt;dad] just me and my son yes okay [DEL:no] [DEL:problem] okay [DEL:do] [DEL:you] i am just going to ask some questions just to [DEL:rule] [SUB:out-&gt;realize] every other thing [DEL:do] [DEL:you] do you have headaches no [DEL:doctor] do you have chest pain no doctor [INS:i] [SUB:at-&gt;do] [SUB:all-&gt;not] [SUB:no-&gt;know] do you have an abdominal pain [DEL:oh] do [DEL:you] you have an abdominal pain do you have any change in your bowel habits i do not know how to answer that [DEL:other] [DEL:than] [DEL:the] [DEL:just] [DEL:the] [DEL:the] [DEL:okay] [DEL:i] [DEL:think] [DEL:i] [DEL:think] i think that is fine your urine [DEL:your] [DEL:your] [DEL:urine] [DEL:has] [DEL:it] has it changed in quantity no not at all how about the frequency of urination has it changed no no [DEL:my] urination is fine [DEL:do] [DEL:you] [DEL:have] [DEL:any] do you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you [DEL:for] for answering my questions those questions are basically there so that we can pinpoint [DEL:where] [DEL:and] where there is a problem and [SUB:they-&gt;you] can also come to have [INS:a] differential diagnosis of what could be the because of your symptoms and [SUB:we-&gt;i] would like to examine you [DEL:right] check your level of hydration check your general physical appearance [DEL:to] see whether you [SUB:and-&gt;can] access [DEL:your] your general health [DEL:right] we also like to do an abdominal examination right [DEL:to] to also give us more information on the abdominal pain you are having if [SUB:you-&gt;it] could lead us to what is causing the symptoms you are having the abdominal pain and [DEL:the] the stooling do you understand yes [DEL:although] although it seems like what you ate the restaurants you got food from [SUB:there-&gt;they] must have been where you got some infection [DEL:which] [DEL:could] [DEL:have] [SUB:which-&gt;it] could have caused the diarrhea you want to say something so what exactly is [SUB:wrong-&gt;drunk] what exactly is [DEL:wrong] [DEL:what] [DEL:exactly] [DEL:is] [DEL:the] [DEL:because] [SUB:okay-&gt;drunk] it is just the food i ate right [DEL:so] yeah it looks like you have had a food poisoning [INS:however] [INS:we] [INS:are] [INS:going] [INS:to] [INS:have] [INS:to] [INS:evaluate] [INS:you] [INS:and] [INS:find] [INS:out] [SUB:had-&gt;what] [SUB:a-&gt;exactly] [SUB:food-&gt;is] [SUB:poisoning-&gt;the] [SUB:but-&gt;because] [SUB:however-&gt;so] we are going to [INS:do] [INS:some] [INS:very] [INS:serious] [INS:tests] [INS:i] [INS:am] [INS:going] [INS:to] [INS:check] [INS:your] [INS:blood] [INS:count] [INS:to] [INS:make] [INS:sure] [INS:there] [INS:is] [INS:some] [INS:infection] [INS:i] [INS:do] [INS:not] [SUB:have-&gt;know] to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to [DEL:know] [DEL:if] [DEL:there] [SUB:is-&gt;make] [SUB:a-&gt;this] there is some infection which could be gastroenteritis [SUB:we-&gt;you] want to do your erythrocyte [SUB:sedimentation-&gt;segmentation] [SUB:rates-&gt;rate] to know if there is [DEL:any] [DEL:sign] any any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and [DEL:then] [SUB:we-&gt;they] would also want to do a stool culture microscopy and sensitivity [DEL:and] to look out for parasites and some bacteria that could cause you to be having diarrhea we also check your retroviral status to know if you have [INS:a] retroviral disease which could also be a because [DEL:of] of diarrhea although that comes in [DEL:the] [SUB:chronic-&gt;a] chronic setting however [INS:we] would also need to just rule that out do you understand okay doctor okay however we are going to start you on [DEL:on] [DEL:some] some fluids to [DEL:you] [DEL:know] give you some strength and restore your hydration level because you have been [SUB:losing-&gt;using] some fluid [DEL:from] from [SUB:the-&gt;this] [SUB:stooling-&gt;tooling] and the vomiting we [DEL:will] also check your electrolytes electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be [DEL:that] [DEL:will] that will need to be corrected do you understand [DEL:okay] and also lastly we [DEL:would] also want to [DEL:check] do an abdominal scan [INS:to] [INS:rule] [SUB:throughout-&gt;out] any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which [DEL:would] [DEL:be] could be causing the diarrhea and [DEL:the] [DEL:the] the abdominal pain do you understand yes thank you doctor thank you very much [DEL:yes] do you have any more questions for me no i am fine i am fine i am good let us just get [DEL:on] [DEL:with] [DEL:it] [DEL:you] [SUB:are-&gt;out] [SUB:fine-&gt;of] [SUB:yeah-&gt;here] so [SUB:that-&gt;i] [SUB:will-&gt;can] be fine thank you so you will be attended to [DEL:all] [SUB:right-&gt;alright] thank you very much [DEL:doctor]</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor [DEL:sadeko] [DEL:yeah] [DEL:good] [DEL:afternoon] [DEL:how] [DEL:may] [DEL:i] [DEL:help] [DEL:you] [SUB:yeah-&gt;shadekum] good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been [SUB:stooling-&gt;straining] for about four days now and [DEL:i] [DEL:have] [SUB:been-&gt;having] abdominal pain [DEL:two] alongside so that is [DEL:those] [SUB:are-&gt;just] my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is [SUB:it-&gt;he] watery is he semi solid or [DEL:it] is [SUB:in-&gt;it] normal form well formed [DEL:stools] it is very watery very watery [DEL:very] [DEL:watery] [DEL:yes] [DEL:okay] [DEL:all] [DEL:right] so like how many episodes of you said you have been [SUB:stolen-&gt;stalling] for over four days right yes and how many episodes do you do you have per day of [DEL:stooling] [SUB:my-&gt;stalling] about six [SUB:about-&gt;or] six to seven episodes actually about around that [INS:number] [INS:yes] of passage of [INS:the] [INS:water] [SUB:watery-&gt;riser] [SUB:stool-&gt;tube] yes yes yes doctor okay okay so [INS:is] [INS:this] is [SUB:the-&gt;it] [SUB:stool-&gt;still] containing mucus is it mucoid no no there is [DEL:no] [DEL:mucus] no mucus in it was there any blood in it no blood at all there is no blood in it okay did you change did you eat [DEL:a] from a new restaurant or did you did you eat something different [SUB:ermactually-&gt;actually] a few days ago [DEL:i] [DEL:like] just before [SUB:it-&gt;you] started i actually had [SUB:a-&gt;the] take out in a restaurant with my family which all [DEL:of] [SUB:us-&gt;was] [SUB:ate-&gt;it] and [SUB:one-&gt;all] of my child actually vomited but [INS:the] vomiting stopped and [SUB:he-&gt;it] feels good now so it is just [DEL:me] right now with the [SUB:complaints-&gt;complaint] i have of the of the loose [SUB:stool-&gt;so] are you also vomiting yes [INS:i] [INS:i] [SUB:ii-&gt;have] vomited about two two episodes about two times yes [DEL:what] [SUB:what-&gt;well] what what was inside the vomit what was the [DEL:components] [DEL:of] [SUB:the-&gt;con] [SUB:vomitus-&gt;components] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the [SUB:content-&gt;contents] of what i ate was the vomiting was it projectile so what do you mean by projectile [SUB:ermwhen-&gt;when] it comes with force when it comes with force well i really do not know [SUB:it-&gt;i] just i just [INS:want] [INS:to] [INS:tell] [SUB:vomited-&gt;you] that is [SUB:all-&gt;the] [SUB:i-&gt;line] i cannot really remember how [SUB:you-&gt;it] came out to be honest [DEL:okay] [SUB:was-&gt;is] there any is there any abdominal [SUB:distension-&gt;distention] [SUB:distension-&gt;distention] like a swelling swelling yeah [SUB:was-&gt;is] there swelling in your stomach no just the abdominal pain the pain is just at my [DEL:the] lower part of my stomach [DEL:okuhm] [DEL:all] [SUB:right-&gt;okay] [SUB:all-&gt;alright] [SUB:right-&gt;alright] thank you so you said your son also ate ate the same the same food that you bought and [DEL:he] is now vomiting how is he feeling now [SUB:he-&gt;it] feels [SUB:he-&gt;it] is okay [DEL:he] after the [DEL:episode] [DEL:of] [DEL:vomiting] [DEL:he] he got he got well and [SUB:he-&gt;it] is okay how is your appetite like my appetite is [DEL:is] [DEL:here] [SUB:and-&gt;yeah] there [SUB:know-&gt;no] it is not really good like so now [INS:this] [SUB:let-&gt;like] [SUB:us-&gt;before] okay okay so let us talk about let us talk about your the pain [SUB:you-&gt;we] [SUB:were-&gt;are] having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and [DEL:leaves] [SUB:you-&gt;needs] [SUB:whatwhat-&gt;what] kind of pain is it [DEL:yeah] i [SUB:will-&gt;would] describe it [DEL:like] [DEL:like] [SUB:has-&gt;as] a [SUB:cramp-&gt;camp] pain like [SUB:the-&gt;a] pain i feel during menstruation so that is the kind of pain [DEL:like] [DEL:that] [DEL:is] [DEL:the] [DEL:way] i can describe it and [DEL:where] where is this pain located in your abdomen the lower [SUB:part-&gt;parts] the lower [SUB:part-&gt;parts] does this pain does it move to [INS:any] [SUB:another-&gt;other] part of your body when you start feeling it no [DEL:just] just the lower part of my [DEL:like] [DEL:moving] [DEL:to] [DEL:the] [DEL:back] [DEL:just] [DEL:the] [DEL:lower] [DEL:part] [DEL:it] [DEL:does] [DEL:not] [DEL:move] [DEL:to] [DEL:your] [DEL:back] [DEL:no] [DEL:no] [DEL:not] [DEL:at] [DEL:all] [DEL:it] [DEL:stays] [SUB:in-&gt;abdomen] the same space yes yes okay okay so [DEL:what] what do you think makes this [SUB:pain-&gt;play] worse well [DEL:maybe] [DEL:if] [DEL:i] if i do not eat i do not know [DEL:if] [DEL:i] [DEL:do] [DEL:not] [SUB:eat-&gt;maybe] something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse [SUB:per-&gt;i] [SUB:se-&gt;say] but i [DEL:will] [SUB:say-&gt;was] [SUB:maybe-&gt;saying] if i do not eat yes okay what [SUB:what-&gt;really] [SUB:what-&gt;how] [SUB:relieves-&gt;is] the pain [INS:not] [SUB:nothing-&gt;saying] i do not know i do not know [DEL:anything] [DEL:that] [DEL:reduce] [DEL:the] [DEL:pain] [SUB:it-&gt;i] just comes and goes on [SUB:its-&gt;this] one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you [DEL:have] felt in your life so what would you give this pain i [INS:would] [SUB:will-&gt;give] [SUB:the-&gt;this] pain like five [INS:out] [SUB:or-&gt;of] ten five [INS:out] [SUB:ten-&gt;of] [SUB:yes-&gt;ten] no problem [DEL:so] let us [DEL:yeah] take some history do you [DEL:have] are you hypertensive no i am not are you diabetic no i am not do you are you a [DEL:known] [SUB:peptic-&gt;nonpeptic] [SUB:also-&gt;ulcer] patient no no are you lactose intolerant no the only the only [SUB:ailment-&gt;payment] i [SUB:am-&gt;will] [SUB:being-&gt;be] [SUB:treated-&gt;treating] for [INS:is] [INS:asthma] i [SUB:am-&gt;have] [SUB:being-&gt;been] treated for is asthma i [DEL:am] [DEL:a] [DEL:known] [SUB:asthmatic-&gt;have] [SUB:and-&gt;nonasthmatic] and i am on i use inhalers and how many [INS:recently] how many [SUB:exacerbations-&gt;exhibitions] do you have in a year [DEL:about] [SUB:in-&gt;how] [SUB:the-&gt;about] last one just one okay okay that [SUB:is-&gt;was] good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those [DEL:i] [DEL:do] [DEL:not] [DEL:at] [DEL:all] and since you have been feeling these symptoms that you are having [DEL:has] [SUB:has-&gt;as] it progressively worsened yeah [DEL:i] i feel so so that is why i actually came to the hospital just [DEL:today] to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your [DEL:body] [SUB:is-&gt;bodys] dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah [DEL:my] [DEL:my] [DEL:i] [DEL:feel] [DEL:sometimes] my mouth is kind of dry to kind of [DEL:okay] okay okay no problem so do you [SUB:asides-&gt;aside] the asthma do you have any other ailments [INS:that] you think the doctor should know about no not at all at all i have [DEL:no] [DEL:other] no other medical condition do you have any drug allergies no [DEL:i] [DEL:do] [DEL:not] [DEL:react] [DEL:no] [DEL:at] [DEL:all] i do not react to any drugs at all [DEL:okay] [DEL:please] are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who [SUB:had-&gt;are] the the [INS:vomit] [SUB:vomiting-&gt;symptoms] was there any any of your family members that also had the same symptoms no no no [DEL:no] [DEL:no] [DEL:other] [DEL:just] [SUB:me-&gt;that] just me and my son yes [DEL:okay] no problem okay do you i am just going to ask some questions just to rule out every other thing [DEL:do] [DEL:you] do you have headaches no [DEL:doctor] do you have chest pain [INS:i] [SUB:no-&gt;know] doctor [SUB:at-&gt;i] [SUB:all-&gt;thought] no do you have an abdominal pain [DEL:oh] do [DEL:you] you have an abdominal pain [DEL:do] you have any change in your bowel habits i do not know how to answer that [DEL:other] [DEL:than] [DEL:the] [DEL:just] [DEL:the] [DEL:the] [DEL:okay] [DEL:i] [DEL:think] [DEL:i] [DEL:think] i think that is fine your urine [DEL:your] your urine [DEL:has] [DEL:it] has it changed in quantity no not at all how about the frequency of urination has it changed no no [DEL:my] [DEL:urination] [DEL:is] [DEL:fine] [DEL:do] [DEL:you] [DEL:have] [DEL:any] do you have any bone pain no [DEL:all] [DEL:right] [DEL:no] [DEL:problem] so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and [SUB:they-&gt;then] can also come to have differential diagnosis of what could be the because of your symptoms and [SUB:we-&gt;they] would like to examine you right check your level of hydration check your general physical appearance to see whether [INS:you] you and access [DEL:your] your general health [DEL:right] we also like to do an abdominal examination right [DEL:to] to also give us more information on the abdominal pain you are having if [SUB:you-&gt;it] could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand [INS:yes] yes although although it seems like what you ate the restaurants you got food from there must have been where you got some [INS:so] infection which could have which could have caused the [SUB:diarrhea-&gt;diarrhoea] you want to say something [INS:yeah] so what exactly is [SUB:wrong-&gt;drawn] what exactly is wrong what exactly is the because [DEL:okay] it is [DEL:just] [DEL:the] [DEL:food] [DEL:i] [DEL:ate] [DEL:right] [DEL:so] [DEL:yeah] it [DEL:looks] [DEL:like] [DEL:you] [SUB:have-&gt;is] [SUB:had-&gt;just] [SUB:a-&gt;the] food poisoning [SUB:had-&gt;by] [SUB:a-&gt;the] food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some [SUB:very-&gt;really] series of tests i am going to check your blood count to [SUB:know-&gt;see] if [DEL:there] [DEL:is] [DEL:a] there is some infection [DEL:which] [DEL:could] be [SUB:gastroenteritis-&gt;gastritis] we want to do your erythrocyte sedimentation [SUB:rates-&gt;rate] to know if there is any [DEL:sign] any any type [DEL:of] kind of inflammatory disorder that could cause [SUB:diarrhea-&gt;diarrhoea] like inflammatory bowel disease right and [DEL:then] [SUB:we-&gt;they] would also want to do [SUB:a-&gt;is] [SUB:stool-&gt;to] culture microscopy and sensitivity and to look out for parasites and some bacteria that could cause you to be having [SUB:diarrhea-&gt;diarrhoea] [SUB:we-&gt;and] also check your retroviral status to know if [SUB:you-&gt;your] [SUB:have-&gt;abdominal] [SUB:retroviral-&gt;viral] disease which could also be a because of of [INS:diarrhoea] [SUB:diarrhea-&gt;or] [SUB:although-&gt;do] that comes in [SUB:the-&gt;a] chronic [INS:a] chronic setting however [INS:we] would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some fluids to you know give you some strength and restore your hydration level because you have been losing some fluid [DEL:from] from [SUB:the-&gt;this] [SUB:stooling-&gt;tooling] and the vomiting we [DEL:will] also check your electrolytes electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be [DEL:that] [DEL:will] that will need to be corrected do you understand [DEL:okay] and also lastly we would also want to check do an abdominal scan [INS:to] [INS:rule] [SUB:throughout-&gt;out] any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which [DEL:would] [DEL:be] could be causing the [SUB:diarrhea-&gt;diarrhoea] and [SUB:the-&gt;then] the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me [DEL:no] i am fine i am fine i am good let us just get on with it [DEL:you] [DEL:are] [SUB:fine-&gt;so] yeah so that [SUB:will-&gt;can] be fine thank you so you [SUB:will-&gt;have] [SUB:be-&gt;been] attended to [DEL:all] [SUB:right-&gt;alright] thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor [SUB:sadeko-&gt;shadiko] yeah good afternoon [DEL:how] [DEL:may] [DEL:i] [DEL:help] [DEL:you] yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and [DEL:i] [DEL:have] [SUB:been-&gt;having] abdominal pain [SUB:two-&gt;too] alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency [DEL:of] [DEL:the] of [SUB:the-&gt;this] [SUB:stool-&gt;tool] is [SUB:it-&gt;he] watery is he [DEL:semi] [SUB:solid-&gt;semisolid] or it is [SUB:in-&gt;a] normal form [DEL:well] [SUB:formed-&gt;wellformed] [SUB:stools-&gt;stool] it is very watery very watery very [SUB:watery-&gt;watchful] yes okay all right so like how many episodes of you said you have been [SUB:stolen-&gt;stooling] for [SUB:over-&gt;about] four days right yes and how many episodes [DEL:do] [DEL:you] do you have per day of stooling [DEL:my] about six about six to seven episodes actually about around that [INS:number] [INS:yes] of passage of watery stool yes yes yes doctor okay okay so is [SUB:the-&gt;this] [SUB:stool-&gt;tool] containing mucus is it mucoid [INS:no] no no [SUB:there-&gt;it] is [SUB:no-&gt;not] mucus no mucus [DEL:in] [DEL:it] was there any blood in it no blood at all there is no blood in it okay did you change did you eat [DEL:a] from a new restaurant or [DEL:did] [DEL:you] did you eat something different [SUB:ermactually-&gt;actually] a few days ago i like just before [SUB:it-&gt;i] started i actually had a [DEL:take] [SUB:out-&gt;takeout] in a restaurant with my family which all of us ate and one of my child actually vomited but [INS:the] vomiting stopped and [SUB:he-&gt;it] feels good now so it is just [DEL:me] right now with the complaints i have [DEL:of] [DEL:the] of the loose [DEL:stool] [DEL:are] [DEL:you] [SUB:also-&gt;yes] [SUB:vomiting-&gt;i] [SUB:yes-&gt;have] [SUB:ii-&gt;only] [SUB:vomited-&gt;said] about [DEL:two] two episodes [SUB:about-&gt;but] two times yes [DEL:what] [DEL:what] [SUB:what-&gt;well] what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomiters] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile [SUB:ermwhen-&gt;when] it comes with force when it comes [SUB:with-&gt;to] force well i really do not know [DEL:it] [DEL:just] i just [DEL:vomited] [DEL:that] [SUB:is-&gt;wanted] [SUB:all-&gt;to] [SUB:i-&gt;ask] i cannot really remember how [SUB:you-&gt;it] came out to be honest okay was there any is there any abdominal distension distension like a swelling swelling yeah was there swelling in your stomach no just the abdominal pain the pain is just at my [DEL:the] lower part of my stomach [SUB:okuhm-&gt;okay] all right all right thank you so you said your son also [DEL:ate] [DEL:ate] [DEL:the] [DEL:same] [DEL:the] [DEL:same] [DEL:food] [DEL:that] [DEL:you] bought and he is now vomiting how is he feeling now he feels he is okay [DEL:he] after the [SUB:episode-&gt;appearance] of vomiting [DEL:he] [DEL:he] [DEL:got] he got well and [SUB:he-&gt;it] is [INS:okay] okay how is your appetite like my appetite [DEL:is] is here [DEL:and] [SUB:there-&gt;yeah] [SUB:know-&gt;no] it is not really good [DEL:like] so now let us okay okay so let us talk about let us talk about your the pain you [SUB:were-&gt;are] having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you [SUB:whatwhat-&gt;what] kind of pain is it [DEL:yeah] i will describe it like like [SUB:has-&gt;as] a cramp pain like the pain i feel during [INS:my] [SUB:menstruation-&gt;session] so that is the kind of pain like that is the way i can describe it and [DEL:where] where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just [DEL:just] [DEL:the] [DEL:lower] [DEL:part] [DEL:of] [DEL:my] [DEL:like] [DEL:moving] [DEL:to] [DEL:the] back just the lower part [DEL:it] [DEL:does] [DEL:not] [DEL:move] [DEL:to] [DEL:your] [DEL:back] no [DEL:no] [DEL:not] [DEL:at] [DEL:all] [DEL:it] [SUB:stays-&gt;is] [SUB:in-&gt;this] the same space yes yes [DEL:okay] okay so [DEL:what] what do you think makes this pain worse [DEL:well] maybe [DEL:if] [DEL:i] if i do not eat i do not know [DEL:if] [SUB:i-&gt;it] [SUB:do-&gt;is] [SUB:not-&gt;easier] [SUB:eat-&gt;maybe] something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it [SUB:worse-&gt;well] per se but i [SUB:will-&gt;would] say maybe if i do not eat yes okay [DEL:what] [DEL:what] what relieves the pain nothing i do not know i do not know [SUB:anything-&gt;if] that [DEL:reduce] [DEL:the] [DEL:pain] [DEL:it] just comes and goes on [SUB:its-&gt;this] one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you [DEL:have] felt in your life so what would you give this pain i will [INS:give] the pain like five or ten five [INS:over] ten [SUB:yes-&gt;okay] no problem so let us [DEL:yeah] take some history [DEL:do] [DEL:you] [DEL:have] are you hypertensive no i am not are you diabetic no i am not do you are you a [DEL:known] [SUB:peptic-&gt;nonpeptic] [SUB:also-&gt;ulcer] patient no no are you lactose [DEL:intolerant] [SUB:no-&gt;in] [SUB:the-&gt;tolerant] [SUB:only-&gt;no] the only [SUB:ailment-&gt;aim] i am [DEL:being] [SUB:treated-&gt;treating] for i [SUB:am-&gt;have] [SUB:being-&gt;been] treated for is asthma [DEL:i] [DEL:am] [DEL:a] [DEL:known] [SUB:asthmatic-&gt;my] [SUB:and-&gt;nonasmatic] and i am [SUB:on-&gt;only] i use [DEL:inhalers] [SUB:and-&gt;als] how many how many [SUB:exacerbations-&gt;examples] do you have in a year about [DEL:in] [DEL:the] last one just one okay okay that is good have you had any previous history of blood transfusion any history of surgeries no no [SUB:none-&gt;not] at all okay do you drink alcohol or do you smoke no i do not i do not do any of those i do not [INS:have] [INS:it] at all and since you have been feeling these symptoms that you are having [DEL:has] has it progressively worsened yeah [DEL:i] i feel so so that is why i actually came to the hospital just today to see the doctor and [SUB:properly-&gt;probably] know what is wrong with me and take care of it basically have you been feeling very [SUB:thirsty-&gt;testy] have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah [DEL:my] [DEL:my] i feel sometimes my mouth is kind of dry to [SUB:kind-&gt;cut] [SUB:of-&gt;up] okay okay okay no problem so do you [INS:have] asides the asthma do you have any other ailments [INS:that] you think the doctor should know about no not at all at all i have [DEL:no] [DEL:other] no other medical condition do you have any drug allergies no i do not react [DEL:no] at all i do not react to any drugs at all [DEL:okay] [DEL:please] are you married yes i am married [SUB:with-&gt;you] [SUB:two-&gt;took] [SUB:kids-&gt;it] yes okay and [DEL:you] you live with your husband yes yes i do and your kids live with you yeah what did you say doctor [SUB:and-&gt;are] your kids live with you as well yes they are so [DEL:aside] [SUB:your-&gt;asides] your son or your child who [DEL:had] [SUB:the-&gt;are] the vomiting was there [DEL:any] any of your family members that also had the same symptoms no no no no no [INS:that] [SUB:other-&gt;is] just me [INS:and] just me and my son yes [DEL:okay] [DEL:no] [DEL:problem] okay do you i am just going to ask some questions just to [DEL:rule] [SUB:out-&gt;raise] every other thing [DEL:do] [DEL:you] do you have headaches no [INS:not] [INS:at] [SUB:doctor-&gt;all] do you have chest pain no doctor at all no do you have an abdominal pain [DEL:oh] do [DEL:you] you have an abdominal pain do you have any change in your [SUB:bowel-&gt;dowel] habits [INS:yeah] i do not know how to answer that other than [DEL:the] [DEL:just] [DEL:the] the okay [DEL:i] [DEL:think] [DEL:i] [DEL:think] i think that is fine your urine [DEL:your] [DEL:your] [DEL:urine] [DEL:has] [DEL:it] has it changed in quantity no not at all how about the frequency of urination has it changed no no my [DEL:urination] [DEL:is] [DEL:fine] [DEL:do] [DEL:you] [DEL:have] [DEL:any] [SUB:do-&gt;initial] you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you [DEL:for] for answering my questions those questions are basically there so that we can pinpoint [DEL:where] [DEL:and] where there is a problem and [INS:then] [SUB:they-&gt;we] can also come to have differential diagnosis of what could be the because of your symptoms and [INS:then] we would like to examine you right check your level of [SUB:hydration-&gt;vibration] check your general physical appearance to see whether you [SUB:and-&gt;can] access [DEL:your] your general health [DEL:right] we also like to do an abdominal examination right [DEL:to] [SUB:to-&gt;so] also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you [SUB:are-&gt;have] [SUB:having-&gt;in] the abdominal pain and [DEL:the] the stooling do you understand yes although although it seems like what you ate the [SUB:restaurants-&gt;restaurant] you got food from there must have been where you got some infection [DEL:which] [DEL:could] [DEL:have] [DEL:which] [DEL:could] [DEL:have] [DEL:caused] [DEL:the] [DEL:diarrhea] you want to say something so what exactly is [SUB:wrong-&gt;drug] what exactly is wrong what exactly is the because okay it is just the food i [SUB:ate-&gt;had] right [DEL:so] yeah it looks like you have had a food poisoning [SUB:had-&gt;or] [SUB:a-&gt;the] food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very [DEL:series] [SUB:of-&gt;serious] tests i am going to check your blood count to [DEL:know] [DEL:if] [DEL:there] [DEL:is] [SUB:a-&gt;make] there is some infection which could be [INS:a] gastroenteritis we want to do your erythrocyte sedimentation [SUB:rates-&gt;rate] to know if there is [DEL:any] [DEL:sign] [DEL:any] any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and then we would also want to do a stool culture microscopy and sensitivity [DEL:and] to look out for parasites and some [SUB:bacteria-&gt;bacterias] that could cause you to be having diarrhea we also check your retroviral status to know if you have [INS:a] retroviral disease which could also be a because [DEL:of] of diarrhea although that comes in [SUB:the-&gt;a] chronic chronic setting however [INS:i] would also need to just rule that out do you understand okay doctor okay however we are going to start you on [DEL:on] [DEL:some] some [SUB:fluids-&gt;foods] to [DEL:you] [DEL:know] give you some strength and restore your hydration level because you have been losing some fluid [DEL:from] from the stooling and the vomiting we [DEL:will] also check your [SUB:electrolytes-&gt;electrolyte] electrolytes to know what [DEL:is] your electrolyte picture looks like and the ones that will be needed to be [DEL:that] [DEL:will] that [SUB:will-&gt;would] need to be corrected do you understand [DEL:okay] and also lastly we [DEL:would] also want to check do an abdominal scan [INS:to] [INS:rule] [SUB:throughout-&gt;out] any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which [DEL:would] [DEL:be] could be causing the diarrhea and [DEL:the] [DEL:the] the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me [DEL:no] i am fine i am fine i am good let us just get on with it [DEL:you] [DEL:are] [DEL:fine] [DEL:yeah] [DEL:so] [DEL:that] [DEL:will] [DEL:be] [DEL:fine] thank you so you will be attended to all right thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may i help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and i have been abdominal pain two alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is it watery is he semi [SUB:solid-&gt;semisolid] or it is in normal form well formed stools it is very watery very watery very watery yes okay all right so like how many episodes of you said you have been stolen for over four days right yes and how many episodes do you do you have per day of stooling my about six about six to seven episodes actually about around that of passage of watery stool yes yes yes doctor okay okay so is the stool containing mucus is it mucoid no no there is no [SUB:mucus-&gt;mucous] no [SUB:mucus-&gt;mucous] in it was there any blood in it no blood at all there is no blood in it okay did you change did you eat a from a new restaurant or did you did you eat something different ermactually a few days ago i like just before it started i actually had a take out in a restaurant with my family which all of us ate and one of my child actually [SUB:vomited-&gt;vomitedited] but vomiting stopped and he feels good now so it is just me right now with the complaints i have of the of the loose [DEL:stool] are you also [SUB:vomiting-&gt;yes] yes ii vomited about two two episodes about two times yes what what what what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomit] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know it just i just [SUB:vomited-&gt;wanted] that is all i i cannot really remember how you came out to be honest okay was there any is there any abdominal distension distension like a swelling swelling yeah was there swelling in your stomach no just the [INS:muscle] [INS:abdominal] [INS:distension] [INS:swelling] [INS:swelling] [INS:swelling] [INS:stomach] abdominal pain the pain is just at my the lower part of my stomach okuhm all right all right thank you so you said your son also ate ate the same the same food that you bought and he is now vomiting how is he feeling now he feels he is okay he after the episode of vomiting he he got he got well and he is okay how is your appetite like my appetite is is here and there know it is not really good like so now let us okay okay so let us talk about let us talk about your the pain you were having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it [INS:cramp] [INS:pain] [INS:pain] [INS:pain] yeah i will describe it like like has a cramp pain like the [SUB:pain-&gt;been] i feel during menstruation so that is the kind of pain like that is the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just just the lower part of my like moving to the back just the lower part it does not move to your back no no not at all it stays in the same space yes yes okay okay so what what do you think makes this pain worse well maybe if i if i do not eat i do not know if i do not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse per se but i will say maybe if i do not eat yes okay what what what relieves the pain nothing i do not know i do not know anything that reduce the [SUB:pain-&gt;that] it just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will the pain like five or ten five ten yes no problem so let us yeah take some history do you have are you hypertensive no i am not are you diabetic no i am not do you are you a [SUB:known-&gt;nonpeptic] [SUB:peptic-&gt;because] also patient no no are you lactose intolerant no the only the only ailment i am being treated for i am [SUB:being-&gt;nonpeptic] [SUB:treated-&gt;ulcer] for is [SUB:asthma-&gt;are] i [SUB:am-&gt;lactose] a known [SUB:asthmatic-&gt;the] and and i am on i use [SUB:inhalers-&gt;asthmatic] and how [SUB:many-&gt;inhalers] how many exacerbations do you have in a year about in the last one just one okay okay that is good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those i do not at all and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i i feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my i feel sometimes my mouth is kind of dry to kind of okay okay okay no problem so do you asides the asthma do you have any other ailments you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no at all i do not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [SUB:vomiting-&gt;vomitting] was there any any of your family members that also had the same symptoms no no no no no other just me just me and my son yes okay no [DEL:problem] okay do you i am just going to ask some questions just to rule out every other thing do you do you have headaches no doctor do you have chest pain no doctor at all no do you have an abdominal pain oh do you you have an abdominal pain do you have any change in your bowel habits i do not know how to answer that other than the just the the okay i think i think i think that is fine your urine your your [DEL:urine] has it has it changed in quantity no not at all how about the frequency of urination has it changed no no my urination is fine do you have any do you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and they can also come to have differential diagnosis of what could be the because of your symptoms and we would like to examine you right check your level of hydration check your general physical appearance to see whether you and access your your general health right we also like to do an abdominal examination right to to also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some infection which could have which could have caused the diarrhea you want to say something so what exactly is wrong what exactly is wrong what exactly is the because okay it is just the food i ate right so yeah it looks like you have had a food poisoning had a [SUB:food-&gt;is] [SUB:poisoning-&gt;the] but however we are going to [INS:blood] [INS:count] [INS:infection] have to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to know if there is a there is some infection which could be gastroenteritis we want to do your erythrocyte [SUB:sedimentation-&gt;segmentation] [SUB:rates-&gt;rate] to know if there is any sign any any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and then we would also want to do a stool culture microscopy and sensitivity and to look out for parasites and some bacteria that could cause you to be having diarrhea we also check your retroviral status to know if you have retroviral disease which could also be a because of of diarrhea although that comes in the chronic chronic setting however would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some fluids to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your electrolytes electrolytes to know what is your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would be could be causing the diarrhea and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine yeah so that will be fine thank you so you will be attended to all right thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may i help you [SUB:yeah-&gt;shadekum] good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and i have been abdominal pain two alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is it watery is he semi solid or it is in normal form well formed stools it is very watery very watery very watery yes okay all right so like how many episodes of you said you have been stolen for over four days right yes and how many episodes do you do you have per day of stooling my about six about six to seven episodes actually about around that of passage of [INS:water] [SUB:watery-&gt;riser] [SUB:stool-&gt;tube] yes yes yes doctor okay okay so is the stool containing mucus is it mucoid no no there is no [DEL:mucus] no mucus in it was there any blood in it no blood at all there is no blood in it okay did you change did you eat a from a new restaurant or did you did you eat something different ermactually a few days ago i like just before it started i actually had a take out in a restaurant with my family which all of us ate and one of my child actually vomited but vomiting stopped and he feels good now so it is just me right now with the [SUB:complaints-&gt;complaint] i have of the of the loose [SUB:stool-&gt;so] are you also vomiting yes ii vomited about two two episodes about two times yes what what what what was inside the vomit what was the components of the [SUB:vomitus-&gt;components] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know it just i just [SUB:vomited-&gt;you] that is all i i cannot really remember how you came out to be honest okay was there any is there any abdominal [SUB:distension-&gt;distention] [SUB:distension-&gt;distention] like a swelling swelling yeah was there swelling in your stomach no just the abdominal pain the pain is just at my the lower part of my stomach okuhm all right all right thank you so you said your son also ate ate the same the same food that you bought and he is now vomiting how is he feeling now he feels he is okay he after the episode of [DEL:vomiting] he he got he got well and he is okay how is your appetite like my appetite is is here and there know it is not really good like so now let us okay okay so let us talk about let us talk about your the pain you were having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it yeah i will describe it like like has a [SUB:cramp-&gt;camp] pain like the pain i feel during menstruation so that is the kind of pain like that is the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just just the lower part of my like moving to the [DEL:back] just the lower part it does not move to your [DEL:back] no no not at all it stays [SUB:in-&gt;abdomen] the same space yes yes okay okay so what what do you think makes this [SUB:pain-&gt;play] worse well maybe if i if i do not eat i do not know if i do not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse per se but i will say maybe if i do not eat yes okay what what what relieves the pain nothing i do not know i do not know anything that reduce the [DEL:pain] it just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will the pain like five or ten five ten yes no problem so let us yeah take some history do you have are you hypertensive no i am not are you diabetic no i am not do you are you a known [SUB:peptic-&gt;nonpeptic] [SUB:also-&gt;ulcer] patient no no are you lactose intolerant no the only the only ailment i am being treated for [INS:asthma] i am being treated for is asthma i am a known [SUB:asthmatic-&gt;have] [SUB:and-&gt;nonasthmatic] and i am on i use inhalers and how many how many exacerbations do you have in a year about in the last one just one okay okay that is good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those i do not at all and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i i feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my i feel sometimes my mouth is kind of dry to kind of okay okay okay no problem so do you asides the asthma do you have any other ailments you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no at all i do not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the [INS:vomit] [SUB:vomiting-&gt;symptoms] was there any any of your family members that also had the same symptoms no no no no no other just me just me and my son yes okay no problem okay do you i am just going to ask some questions just to rule out every other thing do you do you have headaches no doctor do you have chest pain no doctor at all no do you have an abdominal pain oh do you you have an abdominal pain do you have any change in your bowel habits i do not know how to answer that other than the just the the okay i think i think i think that is fine your urine your your urine has it has it changed in quantity no not at all how about the frequency of urination has it changed no no my [DEL:urination] is fine do you have any do you have any bone pain no all right no [DEL:problem] so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and they can also come to have differential diagnosis of what could be the because of your symptoms and we would like to examine you right check your level of hydration check your general physical appearance to see whether you and access your your general health right we also like to do an abdominal examination right to to also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some infection which could have which could have caused the [SUB:diarrhea-&gt;diarrhoea] you want to say something so what exactly is wrong what exactly is wrong what exactly is the because okay it is just the food i ate right so yeah it looks like you have had a food poisoning had a food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to know if there is a there is some infection which could be [SUB:gastroenteritis-&gt;gastritis] we want to do your erythrocyte sedimentation rates to know if there is any sign any any type of kind of inflammatory disorder that could cause [SUB:diarrhea-&gt;diarrhoea] like inflammatory bowel disease right and then we would also want to do a [SUB:stool-&gt;to] culture microscopy and sensitivity and to look out for parasites and some bacteria that could cause you to be having [SUB:diarrhea-&gt;diarrhoea] we also check your retroviral status to know if you [SUB:have-&gt;abdominal] [SUB:retroviral-&gt;viral] disease which could also be a because of of [INS:diarrhoea] [SUB:diarrhea-&gt;or] although that comes in the chronic chronic setting however would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some fluids to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your electrolytes electrolytes to know what is your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would be could be causing the [SUB:diarrhea-&gt;diarrhoea] and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine yeah so that will be fine thank you so you will be attended to all right thank you very much doctor</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>okay good afternoon my name is doctor sadeko yeah good afternoon how may i help you yeah good afternoon my name is miss sharon yes okay so do you have any complaints yes doctor i have been stooling for about four days now and i have been abdominal pain two alongside so that is those are my two complaints okay okay so which one started first the stooling or the abdominal pain yeah the stooling started first about four days ago okay so now like what is the consistency of the of the stool is it watery is he semi [SUB:solid-&gt;semisolid] or it is in normal form well formed stools it is very watery very watery very watery yes okay all right so like how many episodes of you said you have been stolen for over four days right yes and how many episodes do you do you have per day of stooling my about six about six to seven episodes actually about around that of passage of watery stool yes yes yes doctor okay okay so is the stool containing mucus is it mucoid no no there is no mucus no mucus in it was there any blood in it no blood at all there is no blood in it okay did you change did you eat a from a new restaurant or did you did you eat something different ermactually a few days ago i like just before it started i actually had a take out in a restaurant with my family which all of us ate and one of my child actually vomited but vomiting stopped and he feels good now so it is just me right now with the complaints i have of the of the loose [DEL:stool] are you also [SUB:vomiting-&gt;i] yes ii [SUB:vomited-&gt;said] about two two episodes about two times yes what what what what was inside the vomit what was the components of the [SUB:vomitus-&gt;vomiters] was it what you ate or was it greenish or was there blood in it no there was no blood it was just the content of what i ate was the vomiting was it projectile so what do you mean by projectile ermwhen it comes with force when it comes with force well i really do not know it just i just [DEL:vomited] that is all i i cannot really remember how you came out to be honest okay was there any is there any abdominal distension distension like a swelling swelling yeah was there swelling in your stomach no just the abdominal pain the pain is just at my the lower part of my stomach okuhm all right all right thank you so you said your son also ate ate the same the same food that you bought and he is now vomiting how is he feeling now he feels he is okay he after the episode of vomiting he he got he got well and he is okay how is your appetite like my appetite is is here and there know it is not really good like so now let us okay okay so let us talk about let us talk about your the pain you were having so can you describe the pain for me what is the what is the nature of the pain is it a sharp pain or a pain that holds you and leaves you whatwhat kind of pain is it yeah i will describe it like like has a cramp pain like the pain i feel during [SUB:menstruation-&gt;session] so that is the kind of pain like that is the way i can describe it and where where is this pain located in your abdomen the lower part the lower part does this pain does it move to another part of your body when you start feeling it no just just the lower part of my like moving to the back just the lower part it does not move to your [DEL:back] no no not at all it stays in the same space yes yes okay okay so what what do you think makes this pain worse well maybe if i if i do not eat i do not know if i do not eat something around that yeah but i do not feel like if it just comes and goes i do not feel like anything that makes it worse per se but i will say maybe if i do not eat yes okay what what what relieves the pain nothing i do not know i do not know anything that reduce the [DEL:pain] it just comes and goes on its one okay so on a scale of zero to ten let us say zero means that you do not have any pain at all and ten is the worst pain you have felt in your life so what would you give this pain i will the pain like five or ten five ten yes no problem so let us yeah take some history do you have are you hypertensive no i am not are you diabetic no i am not do you are you a known [SUB:peptic-&gt;nonpeptic] [SUB:also-&gt;ulcer] patient no no are you lactose intolerant no the only the only ailment i am being treated for i am being treated for is asthma i am a known [SUB:asthmatic-&gt;my] [SUB:and-&gt;nonasmatic] and i am on i use [DEL:inhalers] and how many how many exacerbations do you have in a year about in the last one just one okay okay that is good have you had any previous history of blood transfusion any history of surgeries no no none at all okay do you drink alcohol or do you smoke no i do not i do not do any of those i do not at all and since you have been feeling these symptoms that you are having has has it progressively worsened yeah i i feel so so that is why i actually came to the hospital just today to see the doctor and properly know what is wrong with me and take care of it basically have you been feeling very thirsty have you been feeling like your body is dry has your urine reduced no not at all no no do you feel weak yeah i feel kind of weak yeah yeah my my i feel sometimes my mouth is kind of dry to kind of okay okay okay no problem so do you asides the asthma do you have any other ailments you think the doctor should know about no not at all at all i have no other no other medical condition do you have any drug allergies no i do not react no at all i do not react to any drugs at all okay please are you married yes i am married with two kids yes okay and you you live with your husband yes yes i do and your kids live with you yeah what did you say doctor and your kids live with you as well yes they are so aside your your son or your child who had the the vomiting was there any any of your family members that also had the same symptoms no no no no no other just me just me and my son yes okay no [DEL:problem] okay do you i am just going to ask some questions just to rule out every other thing do you do you have headaches no doctor do you have chest pain no doctor at all no do you have an abdominal pain oh do you you have an abdominal pain do you have any change in your bowel habits i do not know how to answer that other than the just the the okay i think i think i think that is fine your urine your your [DEL:urine] has it has it changed in quantity no not at all how about the frequency of urination has it changed no no my [DEL:urination] is fine do you have any do you have any bone pain no all right no problem so [SUB:ermthank-&gt;thank] you for for answering my questions those questions are basically there so that we can pinpoint where and where there is a problem and they can also come to have differential diagnosis of what could be the because of your symptoms and we would like to examine you right check your level of [SUB:hydration-&gt;vibration] check your general physical appearance to see whether you and access your your general health right we also like to do an abdominal examination right to to also give us more information on the abdominal pain you are having if you could lead us to what is causing the symptoms you are having the abdominal pain and the the stooling do you understand yes although although it seems like what you ate the restaurants you got food from there must have been where you got some infection which could have which could have caused the [DEL:diarrhea] you want to say something so what exactly is wrong what exactly is wrong what exactly is the because okay it is just the food i ate right so yeah it looks like you have had a food poisoning had a food poisoning but however we are going to have to evaluate you and find out what exactly is the because so we are going to do some very series of tests i am going to check your blood count to know if there is a there is some infection which could be gastroenteritis we want to do your erythrocyte sedimentation [SUB:rates-&gt;rate] to know if there is any sign any any type of kind of inflammatory disorder that could cause diarrhea like inflammatory [DEL:bowel] disease right and then we would also want to do a stool culture microscopy and sensitivity and to look out for parasites and some [SUB:bacteria-&gt;bacterias] that could cause you to be having diarrhea we also check your retroviral status to know if you have retroviral disease which could also be a because of of diarrhea although that comes in the chronic chronic setting however would also need to just rule that out do you understand okay doctor okay however we are going to start you on on some some [SUB:fluids-&gt;foods] to you know give you some strength and restore your hydration level because you have been losing some fluid from from the stooling and the vomiting we will also check your [SUB:electrolytes-&gt;electrolyte] electrolytes to know what is your electrolyte picture looks like and the ones that will be needed to be that will that will need to be corrected do you understand okay and also lastly we would also want to check do an abdominal scan throughout any structural or functional problems that could be in the [SUB:abdominal-&gt;abdomen] which would be could be causing the diarrhea and the the the abdominal pain do you understand yes thank you doctor thank you very much yes do you have any more questions for me no i am fine i am fine i am good let us just get on with it you are fine yeah so that will be fine thank you so you will be attended to all right thank you very much doctor</t>
         </is>
       </c>
     </row>

</xml_diff>